<commit_message>
Audit final: taiere stalpi fata 1872, tracker aliniat (glulam 90x200, M12, Heco 8x200, joiste 100/280/720/1120/1550/1980), interax 440, coltare C1+C2=16, buget realist
</commit_message>
<xml_diff>
--- a/Tracker_materiale_casuta.xlsx
+++ b/Tracker_materiale_casuta.xlsx
@@ -876,7 +876,7 @@
     <row r="2" ht="15.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Proiect cu Tudor (11 ani)  ·  casuta pe 4 stalpi + terasa cu copac integrat  ·  actualizat manual pe masura ce cumparam</t>
+          <t>Proiect cu Tudor (11 ani) · casuta pe 4 stalpi + balcon · buget = TOT proiectul (Faza 1 platforma ~5000 + Faza 2 pereti/acoperis/balustrada/scara). Doar platforma Faza 1: vezi foaia "Platforma premium" / "Comanda Hornbach". Ajusteaza C3 la plafonul tau real.</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="C3" s="52" t="n">
-        <v>4000</v>
+        <v>6600</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="48">
@@ -1008,27 +1008,27 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="48">
-      <c r="A11" s="58" t="inlineStr">
+      <c r="A11" s="94" t="inlineStr">
         <is>
           <t>Structura</t>
         </is>
       </c>
-      <c r="B11" s="59" t="inlineStr">
+      <c r="B11" s="95" t="inlineStr">
         <is>
           <t>Stalpi KVH (portanti)</t>
         </is>
       </c>
-      <c r="C11" s="58" t="inlineStr">
+      <c r="C11" s="94" t="inlineStr">
         <is>
           <t>4000x100x100 mm</t>
         </is>
       </c>
-      <c r="D11" s="58" t="inlineStr">
+      <c r="D11" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="E11" s="58" t="inlineStr">
+      <c r="E11" s="94" t="inlineStr">
         <is>
           <t>7337253</t>
         </is>
@@ -1036,7 +1036,7 @@
       <c r="F11" s="60" t="n">
         <v>4</v>
       </c>
-      <c r="G11" s="58" t="inlineStr">
+      <c r="G11" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -1048,7 +1048,7 @@
         <f>IF(AND(F11&lt;&gt;"",H11&lt;&gt;""),F11*H11,"")</f>
         <v/>
       </c>
-      <c r="J11" s="63" t="inlineStr">
+      <c r="J11" s="96" t="inlineStr">
         <is>
           <t>Cumparat</t>
         </is>
@@ -1058,7 +1058,7 @@
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="L11" s="59" t="inlineStr">
+      <c r="L11" s="95" t="inlineStr">
         <is>
           <t>Cei 4 stalpi principali ai casutei</t>
         </is>
@@ -1067,7 +1067,7 @@
     <row r="12" ht="32.25" customHeight="1" s="48">
       <c r="A12" s="65" t="inlineStr">
         <is>
-          <t>Stoc nealocat</t>
+          <t>Cadru</t>
         </is>
       </c>
       <c r="B12" s="66" t="inlineStr">
@@ -1117,42 +1117,42 @@
       </c>
       <c r="L12" s="66" t="inlineStr">
         <is>
-          <t>Nerindeluiti — cumparati, fara utilizare alocata inca; posibil fundatie terasa/scara</t>
+          <t>4 din cele 6 joiste podea (fata-spate, consola 700)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="21.75" customHeight="1" s="48">
-      <c r="A13" s="58" t="inlineStr">
+      <c r="A13" s="94" t="inlineStr">
         <is>
           <t>Structura</t>
         </is>
       </c>
-      <c r="B13" s="59" t="inlineStr">
-        <is>
-          <t>Suport metalic stalp pe beton</t>
-        </is>
-      </c>
-      <c r="C13" s="58" t="inlineStr">
-        <is>
-          <t>pt 100x100 mm</t>
-        </is>
-      </c>
-      <c r="D13" s="58" t="inlineStr">
-        <is>
-          <t>Hornbach</t>
-        </is>
-      </c>
-      <c r="E13" s="58" t="n"/>
+      <c r="B13" s="95" t="inlineStr">
+        <is>
+          <t>Papuc reazem U stalpi (in beton)</t>
+        </is>
+      </c>
+      <c r="C13" s="94" t="inlineStr">
+        <is>
+          <t>101x100, otel 4 mm</t>
+        </is>
+      </c>
+      <c r="D13" s="94" t="inlineStr">
+        <is>
+          <t>Leroy Merlin</t>
+        </is>
+      </c>
+      <c r="E13" s="94" t="n"/>
       <c r="F13" s="60" t="n">
         <v>4</v>
       </c>
-      <c r="G13" s="58" t="inlineStr">
+      <c r="G13" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
       </c>
       <c r="H13" s="61" t="n">
-        <v>78.19</v>
+        <v>19.69</v>
       </c>
       <c r="I13" s="62">
         <f>IF(AND(F13&lt;&gt;"",H13&lt;&gt;""),F13*H13,"")</f>
@@ -1160,13 +1160,13 @@
       </c>
       <c r="J13" s="72" t="inlineStr">
         <is>
-          <t>De decis</t>
-        </is>
-      </c>
-      <c r="K13" s="59" t="n"/>
-      <c r="L13" s="59" t="inlineStr">
-        <is>
-          <t>Doar daca fundatiile NU au mustati/buloane turnate</t>
+          <t>Cumparat</t>
+        </is>
+      </c>
+      <c r="K13" s="95" t="n"/>
+      <c r="L13" s="95" t="inlineStr">
+        <is>
+          <t>Deja in beton — il avem; stalpul intra in U</t>
         </is>
       </c>
     </row>
@@ -1178,12 +1178,12 @@
       </c>
       <c r="B14" s="66" t="inlineStr">
         <is>
-          <t>Grinzi perimetrale (rama)</t>
+          <t>Grinzi principale (glulam)</t>
         </is>
       </c>
       <c r="C14" s="65" t="inlineStr">
         <is>
-          <t>KVH 80x140x4000</t>
+          <t>Glulam 90x200x4000</t>
         </is>
       </c>
       <c r="D14" s="65" t="inlineStr">
@@ -1191,9 +1191,13 @@
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="E14" s="65" t="n"/>
+      <c r="E14" s="65" t="inlineStr">
+        <is>
+          <t>5483835</t>
+        </is>
+      </c>
       <c r="F14" s="67" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G14" s="65" t="inlineStr">
         <is>
@@ -1201,7 +1205,7 @@
         </is>
       </c>
       <c r="H14" s="68" t="n">
-        <v>175</v>
+        <v>479</v>
       </c>
       <c r="I14" s="69">
         <f>IF(AND(F14&lt;&gt;"",H14&lt;&gt;""),F14*H14,"")</f>
@@ -1215,42 +1219,46 @@
       <c r="K14" s="66" t="n"/>
       <c r="L14" s="66" t="inlineStr">
         <is>
-          <t>Rama portanta a platformei, peste stalpi</t>
+          <t>2 grinzi; fata pe varful stalpului, spate pe polita + 2x M12</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="48">
-      <c r="A15" s="58" t="inlineStr">
+      <c r="A15" s="94" t="inlineStr">
         <is>
           <t>Cadru</t>
         </is>
       </c>
-      <c r="B15" s="59" t="inlineStr">
-        <is>
-          <t>Traverse podea (solute)</t>
-        </is>
-      </c>
-      <c r="C15" s="58" t="inlineStr">
-        <is>
-          <t>60x100, interax ~40cm</t>
-        </is>
-      </c>
-      <c r="D15" s="58" t="inlineStr">
+      <c r="B15" s="95" t="inlineStr">
+        <is>
+          <t>Joiste podea (completare)</t>
+        </is>
+      </c>
+      <c r="C15" s="94" t="inlineStr">
+        <is>
+          <t>KVH 100x100x4000</t>
+        </is>
+      </c>
+      <c r="D15" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="E15" s="58" t="n"/>
+      <c r="E15" s="94" t="inlineStr">
+        <is>
+          <t>7337253</t>
+        </is>
+      </c>
       <c r="F15" s="60" t="n">
-        <v>6</v>
-      </c>
-      <c r="G15" s="58" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="G15" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
       </c>
       <c r="H15" s="61" t="n">
-        <v>94</v>
+        <v>149</v>
       </c>
       <c r="I15" s="62">
         <f>IF(AND(F15&lt;&gt;"",H15&lt;&gt;""),F15*H15,"")</f>
@@ -1261,10 +1269,10 @@
           <t>De cumparat</t>
         </is>
       </c>
-      <c r="K15" s="59" t="n"/>
-      <c r="L15" s="59" t="inlineStr">
-        <is>
-          <t>Sustin podeaua intre grinzi</t>
+      <c r="K15" s="95" t="n"/>
+      <c r="L15" s="95" t="inlineStr">
+        <is>
+          <t>Inca 2 (la cele 4 Leroy) = 6 joiste, fata-spate</t>
         </is>
       </c>
     </row>
@@ -1276,18 +1284,26 @@
       </c>
       <c r="B16" s="66" t="inlineStr">
         <is>
-          <t>Dusumea / scandura podea</t>
+          <t>Dusumea larice</t>
         </is>
       </c>
       <c r="C16" s="65" t="inlineStr">
         <is>
-          <t>28x120 mm</t>
-        </is>
-      </c>
-      <c r="D16" s="65" t="n"/>
-      <c r="E16" s="65" t="n"/>
+          <t>Konsta 28x145x3000</t>
+        </is>
+      </c>
+      <c r="D16" s="65" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="E16" s="65" t="inlineStr">
+        <is>
+          <t>6224073</t>
+        </is>
+      </c>
       <c r="F16" s="67" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="G16" s="65" t="inlineStr">
         <is>
@@ -1295,7 +1311,7 @@
         </is>
       </c>
       <c r="H16" s="68" t="n">
-        <v>38</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="I16" s="69">
         <f>IF(AND(F16&lt;&gt;"",H16&lt;&gt;""),F16*H16,"")</f>
@@ -1309,50 +1325,56 @@
       <c r="K16" s="66" t="n"/>
       <c r="L16" s="66" t="inlineStr">
         <is>
-          <t>Podea casuta + terasa</t>
+          <t>Podea casuta + balcon</t>
         </is>
       </c>
     </row>
     <row r="17" ht="21.75" customHeight="1" s="48">
-      <c r="A17" s="58" t="inlineStr">
-        <is>
-          <t>Terasa</t>
-        </is>
-      </c>
-      <c r="B17" s="59" t="inlineStr">
-        <is>
-          <t>Grinzi suport terasa</t>
-        </is>
-      </c>
-      <c r="C17" s="58" t="inlineStr">
-        <is>
-          <t>80x100 mm</t>
-        </is>
-      </c>
-      <c r="D17" s="58" t="n"/>
-      <c r="E17" s="58" t="n"/>
+      <c r="A17" s="94" t="inlineStr">
+        <is>
+          <t>Cadru</t>
+        </is>
+      </c>
+      <c r="B17" s="95" t="inlineStr">
+        <is>
+          <t>Polita + blocaje + rama gaura copac</t>
+        </is>
+      </c>
+      <c r="C17" s="94" t="inlineStr">
+        <is>
+          <t>din offcut 100x100</t>
+        </is>
+      </c>
+      <c r="D17" s="94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" s="94" t="n"/>
       <c r="F17" s="60" t="n">
-        <v>3</v>
-      </c>
-      <c r="G17" s="58" t="inlineStr">
-        <is>
-          <t>buc</t>
-        </is>
-      </c>
-      <c r="H17" s="61" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="G17" s="94" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="H17" s="61" t="n">
+        <v>0</v>
+      </c>
       <c r="I17" s="62">
         <f>IF(AND(F17&lt;&gt;"",H17&lt;&gt;""),F17*H17,"")</f>
         <v/>
       </c>
       <c r="J17" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
-        </is>
-      </c>
-      <c r="K17" s="59" t="n"/>
-      <c r="L17" s="59" t="inlineStr">
-        <is>
-          <t>Nivel mai jos, in jurul copacului — decupaj trunchi</t>
+          <t>Din offcut</t>
+        </is>
+      </c>
+      <c r="K17" s="95" t="n"/>
+      <c r="L17" s="95" t="inlineStr">
+        <is>
+          <t>Sub grinda spate + blocaje + incadrare gaura. Gratis din offcut.</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1401,7 @@
       </c>
       <c r="E18" s="65" t="n"/>
       <c r="F18" s="67" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G18" s="65" t="inlineStr">
         <is>
@@ -1401,36 +1423,36 @@
       <c r="K18" s="66" t="n"/>
       <c r="L18" s="66" t="inlineStr">
         <is>
-          <t>Obligatoriu la 2m inaltime</t>
+          <t>Balustrada balcon, 3 laturi, inclusiv nasul consolei</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="48">
-      <c r="A19" s="58" t="inlineStr">
+      <c r="A19" s="94" t="inlineStr">
         <is>
           <t>Balustrada</t>
         </is>
       </c>
-      <c r="B19" s="59" t="inlineStr">
+      <c r="B19" s="95" t="inlineStr">
         <is>
           <t>Sipci umplutura</t>
         </is>
       </c>
-      <c r="C19" s="58" t="inlineStr">
+      <c r="C19" s="94" t="inlineStr">
         <is>
           <t>18x18 / sipca</t>
         </is>
       </c>
-      <c r="D19" s="58" t="inlineStr">
+      <c r="D19" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="E19" s="58" t="n"/>
+      <c r="E19" s="94" t="n"/>
       <c r="F19" s="60" t="n">
         <v>24</v>
       </c>
-      <c r="G19" s="58" t="inlineStr">
+      <c r="G19" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -1447,8 +1469,8 @@
           <t>De cumparat</t>
         </is>
       </c>
-      <c r="K19" s="59" t="n"/>
-      <c r="L19" s="59" t="inlineStr">
+      <c r="K19" s="95" t="n"/>
+      <c r="L19" s="95" t="inlineStr">
         <is>
           <t>Goluri &lt;9 cm (siguranta copil)</t>
         </is>
@@ -1500,27 +1522,27 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="48">
-      <c r="A21" s="58" t="inlineStr">
+      <c r="A21" s="94" t="inlineStr">
         <is>
           <t>Acoperis</t>
         </is>
       </c>
-      <c r="B21" s="59" t="inlineStr">
+      <c r="B21" s="95" t="inlineStr">
         <is>
           <t>Capriori acoperis</t>
         </is>
       </c>
-      <c r="C21" s="58" t="inlineStr">
-        <is>
-          <t>60x80 mm</t>
-        </is>
-      </c>
-      <c r="D21" s="58" t="n"/>
-      <c r="E21" s="58" t="n"/>
+      <c r="C21" s="94" t="inlineStr">
+        <is>
+          <t>60x100 mm</t>
+        </is>
+      </c>
+      <c r="D21" s="94" t="n"/>
+      <c r="E21" s="94" t="n"/>
       <c r="F21" s="60" t="n">
         <v>4</v>
       </c>
-      <c r="G21" s="58" t="inlineStr">
+      <c r="G21" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -1537,8 +1559,8 @@
           <t>De cumparat</t>
         </is>
       </c>
-      <c r="K21" s="59" t="n"/>
-      <c r="L21" s="59" t="inlineStr">
+      <c r="K21" s="95" t="n"/>
+      <c r="L21" s="95" t="inlineStr">
         <is>
           <t>Structura acoperis inclinat</t>
         </is>
@@ -1588,27 +1610,27 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="48">
-      <c r="A23" s="58" t="inlineStr">
+      <c r="A23" s="94" t="inlineStr">
         <is>
           <t>Scara</t>
         </is>
       </c>
-      <c r="B23" s="59" t="inlineStr">
+      <c r="B23" s="95" t="inlineStr">
         <is>
           <t>Scara fixa + balustrada</t>
         </is>
       </c>
-      <c r="C23" s="58" t="inlineStr">
+      <c r="C23" s="94" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D23" s="58" t="n"/>
-      <c r="E23" s="58" t="n"/>
+      <c r="D23" s="94" t="n"/>
+      <c r="E23" s="94" t="n"/>
       <c r="F23" s="60" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="58" t="inlineStr">
+      <c r="G23" s="94" t="inlineStr">
         <is>
           <t>set</t>
         </is>
@@ -1623,8 +1645,8 @@
           <t>De cumparat</t>
         </is>
       </c>
-      <c r="K23" s="59" t="n"/>
-      <c r="L23" s="59" t="inlineStr">
+      <c r="K23" s="95" t="n"/>
+      <c r="L23" s="95" t="inlineStr">
         <is>
           <t>Cu balustrada, NU franghie</t>
         </is>
@@ -1638,12 +1660,12 @@
       </c>
       <c r="B24" s="66" t="inlineStr">
         <is>
-          <t>Suruburi structurale Torx</t>
+          <t>Suruburi structurale Heco (set)</t>
         </is>
       </c>
       <c r="C24" s="65" t="inlineStr">
         <is>
-          <t>6x200 mm, pac 100</t>
+          <t>8x200 + 6x100 + 6x80, 3 pac</t>
         </is>
       </c>
       <c r="D24" s="65" t="inlineStr">
@@ -1651,21 +1673,22 @@
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="E24" s="65" t="n"/>
+      <c r="E24" s="65" t="inlineStr">
+        <is>
+          <t>10434633/398/139</t>
+        </is>
+      </c>
       <c r="F24" s="67" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G24" s="65" t="inlineStr">
         <is>
           <t>pac</t>
         </is>
       </c>
-      <c r="H24" s="68" t="n">
-        <v>274</v>
-      </c>
-      <c r="I24" s="69">
-        <f>IF(AND(F24&lt;&gt;"",H24&lt;&gt;""),F24*H24,"")</f>
-        <v/>
+      <c r="H24" s="68" t="n"/>
+      <c r="I24" s="69" t="n">
+        <v>536.77</v>
       </c>
       <c r="J24" s="73" t="inlineStr">
         <is>
@@ -1675,37 +1698,47 @@
       <c r="K24" s="66" t="n"/>
       <c r="L24" s="66" t="inlineStr">
         <is>
-          <t>Imbinari grinzi/stalpi</t>
+          <t>Imbinari grinzi/stalpi/contrafise/blocaje</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="48">
-      <c r="A25" s="58" t="inlineStr">
+      <c r="A25" s="94" t="inlineStr">
         <is>
           <t>Feronerie</t>
         </is>
       </c>
-      <c r="B25" s="59" t="inlineStr">
-        <is>
-          <t>Suruburi podea/terasa</t>
-        </is>
-      </c>
-      <c r="C25" s="58" t="inlineStr">
-        <is>
-          <t>5x70 mm</t>
-        </is>
-      </c>
-      <c r="D25" s="58" t="n"/>
-      <c r="E25" s="58" t="n"/>
+      <c r="B25" s="95" t="inlineStr">
+        <is>
+          <t>Suruburi dusumea inox</t>
+        </is>
+      </c>
+      <c r="C25" s="94" t="inlineStr">
+        <is>
+          <t>A2 5x60, 2 pac (100)</t>
+        </is>
+      </c>
+      <c r="D25" s="94" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="E25" s="94" t="inlineStr">
+        <is>
+          <t>10528829</t>
+        </is>
+      </c>
       <c r="F25" s="60" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="58" t="inlineStr">
+      <c r="G25" s="94" t="inlineStr">
         <is>
           <t>pac</t>
         </is>
       </c>
-      <c r="H25" s="61" t="n"/>
+      <c r="H25" s="61" t="n">
+        <v>55.82</v>
+      </c>
       <c r="I25" s="62">
         <f>IF(AND(F25&lt;&gt;"",H25&lt;&gt;""),F25*H25,"")</f>
         <v/>
@@ -1715,10 +1748,10 @@
           <t>De cumparat</t>
         </is>
       </c>
-      <c r="K25" s="59" t="n"/>
-      <c r="L25" s="59" t="inlineStr">
-        <is>
-          <t>Prindere dusumea</t>
+      <c r="K25" s="95" t="n"/>
+      <c r="L25" s="95" t="inlineStr">
+        <is>
+          <t>Prindere larice (~204 buc)</t>
         </is>
       </c>
     </row>
@@ -1730,12 +1763,12 @@
       </c>
       <c r="B26" s="66" t="inlineStr">
         <is>
-          <t>Coltare metalice imbinare</t>
+          <t>Coltare imbinare C1 + C2</t>
         </is>
       </c>
       <c r="C26" s="65" t="inlineStr">
         <is>
-          <t>Alberts</t>
+          <t>4x 100x100x90 + 12x 90x90x65</t>
         </is>
       </c>
       <c r="D26" s="65" t="inlineStr">
@@ -1743,21 +1776,22 @@
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="E26" s="65" t="n"/>
+      <c r="E26" s="65" t="inlineStr">
+        <is>
+          <t>738965 / 738910</t>
+        </is>
+      </c>
       <c r="F26" s="67" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G26" s="65" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
       </c>
-      <c r="H26" s="68" t="n">
-        <v>28.37</v>
-      </c>
-      <c r="I26" s="69">
-        <f>IF(AND(F26&lt;&gt;"",H26&lt;&gt;""),F26*H26,"")</f>
-        <v/>
+      <c r="H26" s="68" t="n"/>
+      <c r="I26" s="69" t="n">
+        <v>95.36</v>
       </c>
       <c r="J26" s="73" t="inlineStr">
         <is>
@@ -1767,50 +1801,57 @@
       <c r="K26" s="66" t="n"/>
       <c r="L26" s="66" t="inlineStr">
         <is>
-          <t>Intarire colturi cadru</t>
+          <t>C1 grinda fata-&gt;stalp (4); C2 anti-ridicare joiste (12)</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="48">
-      <c r="A27" s="58" t="inlineStr">
+      <c r="A27" s="94" t="inlineStr">
         <is>
           <t>Feronerie</t>
         </is>
       </c>
-      <c r="B27" s="59" t="inlineStr">
-        <is>
-          <t>Buloane M10 + piulite autoblocante</t>
-        </is>
-      </c>
-      <c r="C27" s="58" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D27" s="58" t="n"/>
-      <c r="E27" s="58" t="n"/>
+      <c r="B27" s="95" t="inlineStr">
+        <is>
+          <t>Buloane M12 (baza + polita) + saibe</t>
+        </is>
+      </c>
+      <c r="C27" s="94" t="inlineStr">
+        <is>
+          <t>8x M12x120 baza + 4x M12 lung polita</t>
+        </is>
+      </c>
+      <c r="D27" s="94" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="E27" s="94" t="inlineStr">
+        <is>
+          <t>6834285 + set polita</t>
+        </is>
+      </c>
       <c r="F27" s="60" t="n">
-        <v>8</v>
-      </c>
-      <c r="G27" s="58" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="G27" s="94" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
       <c r="H27" s="61" t="n"/>
-      <c r="I27" s="62">
-        <f>IF(AND(F27&lt;&gt;"",H27&lt;&gt;""),F27*H27,"")</f>
-        <v/>
+      <c r="I27" s="62" t="n">
+        <v>231.99</v>
       </c>
       <c r="J27" s="74" t="inlineStr">
         <is>
           <t>De cumparat</t>
         </is>
       </c>
-      <c r="K27" s="59" t="n"/>
-      <c r="L27" s="59" t="inlineStr">
-        <is>
-          <t>Fixare grinzi principale pe stalpi</t>
+      <c r="K27" s="95" t="n"/>
+      <c r="L27" s="95" t="inlineStr">
+        <is>
+          <t>Baza papuc + polita grinda spate (vezi Comanda Hornbach)</t>
         </is>
       </c>
     </row>
@@ -1822,12 +1863,12 @@
       </c>
       <c r="B28" s="66" t="inlineStr">
         <is>
-          <t>Vopsea protectie lemn exterior</t>
+          <t>Ulei lemn tec (dusumea larice)</t>
         </is>
       </c>
       <c r="C28" s="65" t="inlineStr">
         <is>
-          <t>Wetterschutz 6 l</t>
+          <t>Hornbach Plus 2,5 l</t>
         </is>
       </c>
       <c r="D28" s="65" t="inlineStr">
@@ -1835,7 +1876,11 @@
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="E28" s="65" t="n"/>
+      <c r="E28" s="65" t="inlineStr">
+        <is>
+          <t>5509678</t>
+        </is>
+      </c>
       <c r="F28" s="67" t="n">
         <v>2</v>
       </c>
@@ -1845,7 +1890,7 @@
         </is>
       </c>
       <c r="H28" s="68" t="n">
-        <v>183</v>
+        <v>144.39</v>
       </c>
       <c r="I28" s="69">
         <f>IF(AND(F28&lt;&gt;"",H28&lt;&gt;""),F28*H28,"")</f>
@@ -1859,42 +1904,46 @@
       <c r="K28" s="66" t="n"/>
       <c r="L28" s="66" t="inlineStr">
         <is>
-          <t>Protectie intemperii</t>
+          <t>Finisaj larice + lemn expus</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="48">
-      <c r="A29" s="58" t="inlineStr">
+      <c r="A29" s="94" t="inlineStr">
         <is>
           <t>Finisaj</t>
         </is>
       </c>
-      <c r="B29" s="59" t="inlineStr">
-        <is>
-          <t>Grund izolare lemn</t>
-        </is>
-      </c>
-      <c r="C29" s="58" t="inlineStr">
-        <is>
-          <t>2,5 l</t>
-        </is>
-      </c>
-      <c r="D29" s="58" t="inlineStr">
+      <c r="B29" s="95" t="inlineStr">
+        <is>
+          <t>Lazura impregnare (grund structura)</t>
+        </is>
+      </c>
+      <c r="C29" s="94" t="inlineStr">
+        <is>
+          <t>Hornbach exterior 2,5 l</t>
+        </is>
+      </c>
+      <c r="D29" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="E29" s="58" t="n"/>
+      <c r="E29" s="94" t="inlineStr">
+        <is>
+          <t>12469765</t>
+        </is>
+      </c>
       <c r="F29" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="58" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="G29" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
       </c>
       <c r="H29" s="61" t="n">
-        <v>95.5</v>
+        <v>92.5</v>
       </c>
       <c r="I29" s="62">
         <f>IF(AND(F29&lt;&gt;"",H29&lt;&gt;""),F29*H29,"")</f>
@@ -1905,10 +1954,10 @@
           <t>De cumparat</t>
         </is>
       </c>
-      <c r="K29" s="59" t="n"/>
-      <c r="L29" s="59" t="inlineStr">
-        <is>
-          <t>Strat de baza inainte de vopsea</t>
+      <c r="K29" s="95" t="n"/>
+      <c r="L29" s="95" t="inlineStr">
+        <is>
+          <t>Strat de baza structura</t>
         </is>
       </c>
     </row>
@@ -1956,27 +2005,27 @@
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="48">
-      <c r="A31" s="58" t="inlineStr">
+      <c r="A31" s="94" t="inlineStr">
         <is>
           <t>Joaca</t>
         </is>
       </c>
-      <c r="B31" s="59" t="inlineStr">
+      <c r="B31" s="95" t="inlineStr">
         <is>
           <t>Tobogan</t>
         </is>
       </c>
-      <c r="C31" s="58" t="inlineStr">
+      <c r="C31" s="94" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D31" s="58" t="n"/>
-      <c r="E31" s="58" t="n"/>
+      <c r="D31" s="94" t="n"/>
+      <c r="E31" s="94" t="n"/>
       <c r="F31" s="60" t="n">
         <v>1</v>
       </c>
-      <c r="G31" s="58" t="inlineStr">
+      <c r="G31" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -1991,8 +2040,8 @@
           <t>De decis</t>
         </is>
       </c>
-      <c r="K31" s="59" t="n"/>
-      <c r="L31" s="59" t="inlineStr">
+      <c r="K31" s="95" t="n"/>
+      <c r="L31" s="95" t="inlineStr">
         <is>
           <t>Extra, optional</t>
         </is>
@@ -2038,6 +2087,51 @@
       <c r="L32" s="66" t="inlineStr">
         <is>
           <t>Extra, optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="65" t="inlineStr">
+        <is>
+          <t>Finisaj</t>
+        </is>
+      </c>
+      <c r="B33" s="66" t="inlineStr">
+        <is>
+          <t>Topcoat colorat exterior</t>
+        </is>
+      </c>
+      <c r="C33" s="65" t="inlineStr">
+        <is>
+          <t>alegerea ta de culoare</t>
+        </is>
+      </c>
+      <c r="D33" s="65" t="n"/>
+      <c r="E33" s="65" t="n"/>
+      <c r="F33" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="65" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="H33" s="68" t="n">
+        <v>170</v>
+      </c>
+      <c r="I33" s="69">
+        <f>IF(AND(F33&lt;&gt;"",H33&lt;&gt;""),F33*H33,"")</f>
+        <v/>
+      </c>
+      <c r="J33" s="75" t="inlineStr">
+        <is>
+          <t>De decis</t>
+        </is>
+      </c>
+      <c r="K33" s="66" t="n"/>
+      <c r="L33" s="66" t="inlineStr">
+        <is>
+          <t>Culoarea finala; il alegi tu</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2208,7 @@
     <row r="2" ht="15" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Structura blocata: stalpi spate 4m continui · stalpi fata taiati la podea +2200 · joiste Leroy fata-spate (consola 700) · pereti imbracati (bracaj) · acoperis 1 apa doar peste casuta</t>
+          <t>Structura blocata: stalpi spate 4m continui · stalpi fata taiati la +1872 (328 sub podea) · joiste Leroy fata-spate (consola 700) · pereti imbracati (bracaj) · acoperis 1 apa doar peste casuta</t>
         </is>
       </c>
     </row>
@@ -2180,37 +2274,37 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="95" t="inlineStr">
         <is>
           <t>Stalpi spate (inalti)</t>
         </is>
       </c>
-      <c r="C6" s="59" t="inlineStr">
+      <c r="C6" s="95" t="inlineStr">
         <is>
           <t>KVH 100×100</t>
         </is>
       </c>
-      <c r="D6" s="85" t="inlineStr">
+      <c r="D6" s="97" t="inlineStr">
         <is>
           <t>~3800</t>
         </is>
       </c>
-      <c r="E6" s="85" t="inlineStr">
+      <c r="E6" s="97" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F6" s="63" t="inlineStr">
+      <c r="F6" s="96" t="inlineStr">
         <is>
           <t>AVEM</t>
         </is>
       </c>
-      <c r="G6" s="58" t="inlineStr">
+      <c r="G6" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="H6" s="59" t="inlineStr">
+      <c r="H6" s="95" t="inlineStr">
         <is>
           <t>Continui pamant→acoperis; dau coama (latura inalta). Taiere finala pe loc.</t>
         </is>
@@ -2222,39 +2316,39 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="B7" s="59" t="inlineStr">
+      <c r="B7" s="95" t="inlineStr">
         <is>
           <t>Stalpi fata (la podea)</t>
         </is>
       </c>
-      <c r="C7" s="59" t="inlineStr">
+      <c r="C7" s="95" t="inlineStr">
         <is>
           <t>KVH 100×100</t>
         </is>
       </c>
-      <c r="D7" s="85" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="E7" s="85" t="inlineStr">
+      <c r="D7" s="97" t="inlineStr">
+        <is>
+          <t>1872</t>
+        </is>
+      </c>
+      <c r="E7" s="97" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F7" s="63" t="inlineStr">
+      <c r="F7" s="96" t="inlineStr">
         <is>
           <t>AVEM</t>
         </is>
       </c>
-      <c r="G7" s="58" t="inlineStr">
+      <c r="G7" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="H7" s="59" t="inlineStr">
-        <is>
-          <t>Taiati la nivel podea. Offcut ~1800×2 il pastram pentru contrafise/blocuri.</t>
+      <c r="H7" s="95" t="inlineStr">
+        <is>
+          <t>Taiati la +1872 (sub podea: grinda 200 + joista 100 + dusumea 28 = 2200). Offcut ~2128 pt contrafise/blocuri.</t>
         </is>
       </c>
     </row>
@@ -2264,24 +2358,24 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="B8" s="59" t="inlineStr">
+      <c r="B8" s="95" t="inlineStr">
         <is>
           <t>Grinzi principale (fata+spate)</t>
         </is>
       </c>
-      <c r="C8" s="59" t="inlineStr">
-        <is>
-          <t>KVH 80×140 DUBLAT</t>
-        </is>
-      </c>
-      <c r="D8" s="85" t="inlineStr">
+      <c r="C8" s="95" t="inlineStr">
+        <is>
+          <t>Glulam 90x200</t>
+        </is>
+      </c>
+      <c r="D8" s="97" t="inlineStr">
         <is>
           <t>~2300</t>
         </is>
       </c>
-      <c r="E8" s="85" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="E8" s="97" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
       <c r="F8" s="74" t="inlineStr">
@@ -2289,14 +2383,14 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G8" s="58" t="inlineStr">
+      <c r="G8" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="H8" s="59" t="inlineStr">
-        <is>
-          <t>2 grinzi, fiecare dublata. Bulonate M12 in stalpi. Componenta critica.</t>
+      <c r="H8" s="95" t="inlineStr">
+        <is>
+          <t>2 grinzi glulam. Fata pe varful stalpului + C1; spate pe polita + 2x M12. Componenta critica.</t>
         </is>
       </c>
     </row>
@@ -2306,22 +2400,22 @@
           <t>P4</t>
         </is>
       </c>
-      <c r="B9" s="59" t="inlineStr">
+      <c r="B9" s="95" t="inlineStr">
         <is>
           <t>Joiste podea</t>
         </is>
       </c>
-      <c r="C9" s="59" t="inlineStr">
+      <c r="C9" s="95" t="inlineStr">
         <is>
           <t>100×100</t>
         </is>
       </c>
-      <c r="D9" s="85" t="inlineStr">
+      <c r="D9" s="97" t="inlineStr">
         <is>
           <t>~2550</t>
         </is>
       </c>
-      <c r="E9" s="85" t="inlineStr">
+      <c r="E9" s="97" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -2331,14 +2425,14 @@
           <t>4 AVEM + 2 NOU</t>
         </is>
       </c>
-      <c r="G9" s="58" t="inlineStr">
+      <c r="G9" s="94" t="inlineStr">
         <is>
           <t>Leroy</t>
         </is>
       </c>
-      <c r="H9" s="59" t="inlineStr">
-        <is>
-          <t>Fata-spate (consola 700), CONTINUE. Pozitii de la S4: 0/360/660/1100/1575/2100 — ocolesc trunchiul.</t>
+      <c r="H9" s="95" t="inlineStr">
+        <is>
+          <t>Fata-spate (consola 700), CONTINUE. Pozitii de la S4: 100/280/720/1120/1550/1980 — ocolesc trunchiul.</t>
         </is>
       </c>
     </row>
@@ -2348,39 +2442,39 @@
           <t>P4b</t>
         </is>
       </c>
-      <c r="B10" s="59" t="inlineStr">
+      <c r="B10" s="95" t="inlineStr">
         <is>
           <t>Rama gaura copac (headers)</t>
         </is>
       </c>
-      <c r="C10" s="59" t="inlineStr">
+      <c r="C10" s="95" t="inlineStr">
         <is>
           <t>din offcut 100×100</t>
         </is>
       </c>
-      <c r="D10" s="85" t="inlineStr">
+      <c r="D10" s="97" t="inlineStr">
         <is>
           <t>~300</t>
         </is>
       </c>
-      <c r="E10" s="85" t="inlineStr">
+      <c r="E10" s="97" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F10" s="63" t="inlineStr">
+      <c r="F10" s="96" t="inlineStr">
         <is>
           <t>DIN OFFCUT</t>
         </is>
       </c>
-      <c r="G10" s="58" t="inlineStr">
+      <c r="G10" s="94" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H10" s="59" t="inlineStr">
-        <is>
-          <t>Doua traverse scurte intre joistele de la 360 si 660, sus+jos in jurul gaurii. Sustin capetele dusumelei.</t>
+      <c r="H10" s="95" t="inlineStr">
+        <is>
+          <t>Doua traverse scurte intre joistele de la 280 si 720, sus+jos in jurul gaurii. Sustin capetele dusumelei.</t>
         </is>
       </c>
     </row>
@@ -2446,22 +2540,22 @@
           <t>P7</t>
         </is>
       </c>
-      <c r="B15" s="59" t="inlineStr">
+      <c r="B15" s="95" t="inlineStr">
         <is>
           <t>Talpi + coronament pereti</t>
         </is>
       </c>
-      <c r="C15" s="59" t="inlineStr">
+      <c r="C15" s="95" t="inlineStr">
         <is>
           <t>50×80</t>
         </is>
       </c>
-      <c r="D15" s="85" t="inlineStr">
+      <c r="D15" s="97" t="inlineStr">
         <is>
           <t>var</t>
         </is>
       </c>
-      <c r="E15" s="85" t="inlineStr">
+      <c r="E15" s="97" t="inlineStr">
         <is>
           <t>~6</t>
         </is>
@@ -2471,12 +2565,12 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G15" s="58" t="inlineStr">
+      <c r="G15" s="94" t="inlineStr">
         <is>
           <t>oricare</t>
         </is>
       </c>
-      <c r="H15" s="59" t="inlineStr">
+      <c r="H15" s="95" t="inlineStr">
         <is>
           <t>Plate sus/jos pe cele 4 laturi (gol usa spre balcon).</t>
         </is>
@@ -2488,22 +2582,22 @@
           <t>P8</t>
         </is>
       </c>
-      <c r="B16" s="59" t="inlineStr">
+      <c r="B16" s="95" t="inlineStr">
         <is>
           <t>Montanti pereti</t>
         </is>
       </c>
-      <c r="C16" s="59" t="inlineStr">
+      <c r="C16" s="95" t="inlineStr">
         <is>
           <t>50×80</t>
         </is>
       </c>
-      <c r="D16" s="85" t="inlineStr">
+      <c r="D16" s="97" t="inlineStr">
         <is>
           <t>~1400</t>
         </is>
       </c>
-      <c r="E16" s="85" t="inlineStr">
+      <c r="E16" s="97" t="inlineStr">
         <is>
           <t>~14</t>
         </is>
@@ -2513,12 +2607,12 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G16" s="58" t="inlineStr">
+      <c r="G16" s="94" t="inlineStr">
         <is>
           <t>oricare</t>
         </is>
       </c>
-      <c r="H16" s="59" t="inlineStr">
+      <c r="H16" s="95" t="inlineStr">
         <is>
           <t>Interax 600 mm. Mai inalti in spate (latura coamei).</t>
         </is>
@@ -2558,22 +2652,22 @@
           <t>P10</t>
         </is>
       </c>
-      <c r="B19" s="59" t="inlineStr">
+      <c r="B19" s="95" t="inlineStr">
         <is>
           <t>Capriori</t>
         </is>
       </c>
-      <c r="C19" s="59" t="inlineStr">
+      <c r="C19" s="95" t="inlineStr">
         <is>
           <t>60×100</t>
         </is>
       </c>
-      <c r="D19" s="85" t="inlineStr">
+      <c r="D19" s="97" t="inlineStr">
         <is>
           <t>~1400</t>
         </is>
       </c>
-      <c r="E19" s="85" t="inlineStr">
+      <c r="E19" s="97" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -2583,12 +2677,12 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G19" s="58" t="inlineStr">
+      <c r="G19" s="94" t="inlineStr">
         <is>
           <t>oricare</t>
         </is>
       </c>
-      <c r="H19" s="59" t="inlineStr">
+      <c r="H19" s="95" t="inlineStr">
         <is>
           <t>Panta spre gradina, mic streasin in spate.</t>
         </is>
@@ -2600,22 +2694,22 @@
           <t>P11</t>
         </is>
       </c>
-      <c r="B20" s="59" t="inlineStr">
+      <c r="B20" s="95" t="inlineStr">
         <is>
           <t>Astereala acoperis</t>
         </is>
       </c>
-      <c r="C20" s="59" t="inlineStr">
+      <c r="C20" s="95" t="inlineStr">
         <is>
           <t>OSB3 / scandura</t>
         </is>
       </c>
-      <c r="D20" s="85" t="inlineStr">
+      <c r="D20" s="97" t="inlineStr">
         <is>
           <t>2500×1250</t>
         </is>
       </c>
-      <c r="E20" s="85" t="inlineStr">
+      <c r="E20" s="97" t="inlineStr">
         <is>
           <t>1 placa</t>
         </is>
@@ -2625,12 +2719,12 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G20" s="58" t="inlineStr">
+      <c r="G20" s="94" t="inlineStr">
         <is>
           <t>oricare</t>
         </is>
       </c>
-      <c r="H20" s="59" t="inlineStr">
+      <c r="H20" s="95" t="inlineStr">
         <is>
           <t>Suport invelitoare.</t>
         </is>
@@ -2670,22 +2764,22 @@
           <t>P13</t>
         </is>
       </c>
-      <c r="B23" s="59" t="inlineStr">
+      <c r="B23" s="95" t="inlineStr">
         <is>
           <t>Stalpisori balustrada</t>
         </is>
       </c>
-      <c r="C23" s="59" t="inlineStr">
+      <c r="C23" s="95" t="inlineStr">
         <is>
           <t>58×58</t>
         </is>
       </c>
-      <c r="D23" s="85" t="inlineStr">
+      <c r="D23" s="97" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="E23" s="85" t="inlineStr">
+      <c r="E23" s="97" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -2695,12 +2789,12 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G23" s="58" t="inlineStr">
+      <c r="G23" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="H23" s="59" t="inlineStr">
+      <c r="H23" s="95" t="inlineStr">
         <is>
           <t>Interax ~900 mm, inclusiv pe nasul consolei.</t>
         </is>
@@ -2712,22 +2806,22 @@
           <t>P14</t>
         </is>
       </c>
-      <c r="B24" s="59" t="inlineStr">
+      <c r="B24" s="95" t="inlineStr">
         <is>
           <t>Mana curenta + rigla jos</t>
         </is>
       </c>
-      <c r="C24" s="59" t="inlineStr">
+      <c r="C24" s="95" t="inlineStr">
         <is>
           <t>45×70</t>
         </is>
       </c>
-      <c r="D24" s="85" t="inlineStr">
+      <c r="D24" s="97" t="inlineStr">
         <is>
           <t>~9 m total</t>
         </is>
       </c>
-      <c r="E24" s="85" t="inlineStr">
+      <c r="E24" s="97" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -2737,12 +2831,12 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G24" s="58" t="inlineStr">
+      <c r="G24" s="94" t="inlineStr">
         <is>
           <t>oricare</t>
         </is>
       </c>
-      <c r="H24" s="59" t="inlineStr">
+      <c r="H24" s="95" t="inlineStr">
         <is>
           <t>Sus si jos, jur-imprejur.</t>
         </is>
@@ -2782,22 +2876,22 @@
           <t>P16</t>
         </is>
       </c>
-      <c r="B27" s="59" t="inlineStr">
+      <c r="B27" s="95" t="inlineStr">
         <is>
           <t>Coarde scara</t>
         </is>
       </c>
-      <c r="C27" s="59" t="inlineStr">
-        <is>
-          <t>50×150</t>
-        </is>
-      </c>
-      <c r="D27" s="85" t="inlineStr">
-        <is>
-          <t>~2900</t>
-        </is>
-      </c>
-      <c r="E27" s="85" t="inlineStr">
+      <c r="C27" s="95" t="inlineStr">
+        <is>
+          <t>60x140</t>
+        </is>
+      </c>
+      <c r="D27" s="97" t="inlineStr">
+        <is>
+          <t>~3000</t>
+        </is>
+      </c>
+      <c r="E27" s="97" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -2807,12 +2901,12 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G27" s="58" t="inlineStr">
+      <c r="G27" s="94" t="inlineStr">
         <is>
           <t>oricare</t>
         </is>
       </c>
-      <c r="H27" s="59" t="inlineStr">
+      <c r="H27" s="95" t="inlineStr">
         <is>
           <t>Panta de la sol/balcon la podea.</t>
         </is>
@@ -2824,24 +2918,24 @@
           <t>P17</t>
         </is>
       </c>
-      <c r="B28" s="59" t="inlineStr">
+      <c r="B28" s="95" t="inlineStr">
         <is>
           <t>Trepte</t>
         </is>
       </c>
-      <c r="C28" s="59" t="inlineStr">
-        <is>
-          <t>40×200</t>
-        </is>
-      </c>
-      <c r="D28" s="85" t="inlineStr">
+      <c r="C28" s="95" t="inlineStr">
+        <is>
+          <t>45x190</t>
+        </is>
+      </c>
+      <c r="D28" s="97" t="inlineStr">
         <is>
           <t>600</t>
         </is>
       </c>
-      <c r="E28" s="85" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="E28" s="97" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="F28" s="74" t="inlineStr">
@@ -2849,12 +2943,12 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G28" s="58" t="inlineStr">
+      <c r="G28" s="94" t="inlineStr">
         <is>
           <t>oricare</t>
         </is>
       </c>
-      <c r="H28" s="59" t="inlineStr">
+      <c r="H28" s="95" t="inlineStr">
         <is>
           <t>Trepte solide.</t>
         </is>
@@ -2894,22 +2988,22 @@
           <t>P19</t>
         </is>
       </c>
-      <c r="B31" s="59" t="inlineStr">
+      <c r="B31" s="95" t="inlineStr">
         <is>
           <t>Blat masa</t>
         </is>
       </c>
-      <c r="C31" s="59" t="inlineStr">
+      <c r="C31" s="95" t="inlineStr">
         <is>
           <t>panou / scandura lipita ~Ø500</t>
         </is>
       </c>
-      <c r="D31" s="85" t="inlineStr">
+      <c r="D31" s="97" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E31" s="85" t="inlineStr">
+      <c r="E31" s="97" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -2919,12 +3013,12 @@
           <t>NOU/offcut</t>
         </is>
       </c>
-      <c r="G31" s="58" t="inlineStr">
+      <c r="G31" s="94" t="inlineStr">
         <is>
           <t>oricare</t>
         </is>
       </c>
-      <c r="H31" s="59" t="inlineStr">
+      <c r="H31" s="95" t="inlineStr">
         <is>
           <t>Fixat de PODEA prin cadru propriu, NU de copac. Capat trunchi tesit+capac.</t>
         </is>
@@ -2964,24 +3058,24 @@
           <t>P21</t>
         </is>
       </c>
-      <c r="B34" s="59" t="inlineStr">
+      <c r="B34" s="95" t="inlineStr">
         <is>
           <t>Buloane M12 + piulite + saibe</t>
         </is>
       </c>
-      <c r="C34" s="59" t="inlineStr">
-        <is>
-          <t>M12 ×~180</t>
-        </is>
-      </c>
-      <c r="D34" s="85" t="inlineStr">
+      <c r="C34" s="95" t="inlineStr">
+        <is>
+          <t>M12: 8x120 + 4x~200</t>
+        </is>
+      </c>
+      <c r="D34" s="97" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E34" s="85" t="inlineStr">
-        <is>
-          <t>16</t>
+      <c r="E34" s="97" t="inlineStr">
+        <is>
+          <t>12</t>
         </is>
       </c>
       <c r="F34" s="74" t="inlineStr">
@@ -2989,14 +3083,14 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G34" s="58" t="inlineStr">
+      <c r="G34" s="94" t="inlineStr">
         <is>
           <t>oricare</t>
         </is>
       </c>
-      <c r="H34" s="59" t="inlineStr">
-        <is>
-          <t>Grinzi → stalpi. Traseu principal de greutate.</t>
+      <c r="H34" s="95" t="inlineStr">
+        <is>
+          <t>4x polita (lung ~200) + 8x baza papuc (M12x120). Traseu principal de greutate.</t>
         </is>
       </c>
     </row>
@@ -3006,24 +3100,24 @@
           <t>P22</t>
         </is>
       </c>
-      <c r="B35" s="59" t="inlineStr">
-        <is>
-          <t>Coltare metalice</t>
-        </is>
-      </c>
-      <c r="C35" s="59" t="inlineStr">
-        <is>
-          <t>intariri imbinari</t>
-        </is>
-      </c>
-      <c r="D35" s="85" t="inlineStr">
+      <c r="B35" s="95" t="inlineStr">
+        <is>
+          <t>Coltare metalice C1 + C2</t>
+        </is>
+      </c>
+      <c r="C35" s="95" t="inlineStr">
+        <is>
+          <t>C1 100x100x90 (4) + C2 90x90x65 (12)</t>
+        </is>
+      </c>
+      <c r="D35" s="97" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E35" s="85" t="inlineStr">
-        <is>
-          <t>12</t>
+      <c r="E35" s="97" t="inlineStr">
+        <is>
+          <t>16</t>
         </is>
       </c>
       <c r="F35" s="74" t="inlineStr">
@@ -3031,14 +3125,14 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G35" s="58" t="inlineStr">
+      <c r="G35" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="H35" s="59" t="inlineStr">
-        <is>
-          <t>Joiste → grinzi, colturi cadru.</t>
+      <c r="H35" s="95" t="inlineStr">
+        <is>
+          <t>C1 grinda fata-&gt;stalp (4); C2 joiste anti-ridicare (12).</t>
         </is>
       </c>
     </row>
@@ -3048,22 +3142,22 @@
           <t>P23</t>
         </is>
       </c>
-      <c r="B36" s="59" t="inlineStr">
-        <is>
-          <t>Suruburi structurale Torx</t>
-        </is>
-      </c>
-      <c r="C36" s="59" t="inlineStr">
-        <is>
-          <t>6×200, pac 100</t>
-        </is>
-      </c>
-      <c r="D36" s="85" t="inlineStr">
+      <c r="B36" s="95" t="inlineStr">
+        <is>
+          <t>Suruburi structurale Heco</t>
+        </is>
+      </c>
+      <c r="C36" s="95" t="inlineStr">
+        <is>
+          <t>Heco 8x200, pac 100</t>
+        </is>
+      </c>
+      <c r="D36" s="97" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E36" s="85" t="inlineStr">
+      <c r="E36" s="97" t="inlineStr">
         <is>
           <t>1 pac</t>
         </is>
@@ -3073,14 +3167,14 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G36" s="58" t="inlineStr">
+      <c r="G36" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="H36" s="59" t="inlineStr">
-        <is>
-          <t>Imbinari lemn-lemn.</t>
+      <c r="H36" s="95" t="inlineStr">
+        <is>
+          <t>Imbinari lemn-lemn (cod 10434633). Fara pre-gaurire.</t>
         </is>
       </c>
     </row>
@@ -3118,22 +3212,22 @@
           <t>P25</t>
         </is>
       </c>
-      <c r="B39" s="59" t="inlineStr">
+      <c r="B39" s="95" t="inlineStr">
         <is>
           <t>Grund izolare lemn</t>
         </is>
       </c>
-      <c r="C39" s="59" t="inlineStr">
+      <c r="C39" s="95" t="inlineStr">
         <is>
           <t>2,5 l</t>
         </is>
       </c>
-      <c r="D39" s="85" t="inlineStr">
+      <c r="D39" s="97" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E39" s="85" t="inlineStr">
+      <c r="E39" s="97" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3143,12 +3237,12 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G39" s="58" t="inlineStr">
+      <c r="G39" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="H39" s="59" t="inlineStr">
+      <c r="H39" s="95" t="inlineStr">
         <is>
           <t>Strat de baza.</t>
         </is>
@@ -3160,22 +3254,22 @@
           <t>P26</t>
         </is>
       </c>
-      <c r="B40" s="59" t="inlineStr">
+      <c r="B40" s="95" t="inlineStr">
         <is>
           <t>Vopsea protectie exterior</t>
         </is>
       </c>
-      <c r="C40" s="59" t="inlineStr">
+      <c r="C40" s="95" t="inlineStr">
         <is>
           <t>6 l</t>
         </is>
       </c>
-      <c r="D40" s="85" t="inlineStr">
+      <c r="D40" s="97" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E40" s="85" t="inlineStr">
+      <c r="E40" s="97" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -3185,12 +3279,12 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G40" s="58" t="inlineStr">
+      <c r="G40" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="H40" s="59" t="inlineStr">
+      <c r="H40" s="95" t="inlineStr">
         <is>
           <t>Wetterschutz sau similar.</t>
         </is>
@@ -3202,22 +3296,22 @@
           <t>P27</t>
         </is>
       </c>
-      <c r="B41" s="59" t="inlineStr">
+      <c r="B41" s="95" t="inlineStr">
         <is>
           <t>Sol moale sub platforma</t>
         </is>
       </c>
-      <c r="C41" s="59" t="inlineStr">
+      <c r="C41" s="95" t="inlineStr">
         <is>
           <t>scoarta / nisip</t>
         </is>
       </c>
-      <c r="D41" s="85" t="inlineStr">
+      <c r="D41" s="97" t="inlineStr">
         <is>
           <t>~5 m²</t>
         </is>
       </c>
-      <c r="E41" s="85" t="inlineStr">
+      <c r="E41" s="97" t="inlineStr">
         <is>
           <t>1 lot</t>
         </is>
@@ -3227,12 +3321,12 @@
           <t>NOU</t>
         </is>
       </c>
-      <c r="G41" s="58" t="inlineStr">
+      <c r="G41" s="94" t="inlineStr">
         <is>
           <t>oricare</t>
         </is>
       </c>
-      <c r="H41" s="59" t="inlineStr">
+      <c r="H41" s="95" t="inlineStr">
         <is>
           <t>Amortizare cadere. NU beton/piatra dedesubt.</t>
         </is>
@@ -3371,17 +3465,17 @@
       <c r="I5" s="84" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="48">
-      <c r="A6" s="58" t="inlineStr">
+      <c r="A6" s="94" t="inlineStr">
         <is>
           <t>Stalpi</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="95" t="inlineStr">
         <is>
           <t>Stalpi KVH 100×100×4000 (AVEM)</t>
         </is>
       </c>
-      <c r="C6" s="58" t="inlineStr">
+      <c r="C6" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -3392,7 +3486,7 @@
       <c r="E6" s="60" t="n">
         <v>4</v>
       </c>
-      <c r="F6" s="58" t="inlineStr">
+      <c r="F6" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -3401,29 +3495,29 @@
         <f>IF(AND(D6&lt;&gt;"",E6&lt;&gt;""),D6*E6,"")</f>
         <v/>
       </c>
-      <c r="H6" s="59" t="inlineStr">
+      <c r="H6" s="95" t="inlineStr">
         <is>
           <t>Stalpi spate (4m) + fata (taiati 1872)</t>
         </is>
       </c>
-      <c r="I6" s="63" t="inlineStr">
+      <c r="I6" s="96" t="inlineStr">
         <is>
           <t>AVEM</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="48">
-      <c r="A7" s="58" t="inlineStr">
+      <c r="A7" s="94" t="inlineStr">
         <is>
           <t>Baza</t>
         </is>
       </c>
-      <c r="B7" s="59" t="inlineStr">
+      <c r="B7" s="95" t="inlineStr">
         <is>
           <t>Papuc reazem U 101×100, otel 4 mm (in beton)</t>
         </is>
       </c>
-      <c r="C7" s="58" t="inlineStr">
+      <c r="C7" s="94" t="inlineStr">
         <is>
           <t>Leroy</t>
         </is>
@@ -3434,7 +3528,7 @@
       <c r="E7" s="60" t="n">
         <v>4</v>
       </c>
-      <c r="F7" s="58" t="inlineStr">
+      <c r="F7" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -3443,29 +3537,29 @@
         <f>IF(AND(D7&lt;&gt;"",E7&lt;&gt;""),D7*E7,"")</f>
         <v/>
       </c>
-      <c r="H7" s="59" t="inlineStr">
+      <c r="H7" s="95" t="inlineStr">
         <is>
           <t>Baza stalpilor; stalpul intra in U</t>
         </is>
       </c>
-      <c r="I7" s="63" t="inlineStr">
+      <c r="I7" s="96" t="inlineStr">
         <is>
           <t>AVEM</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="48">
-      <c r="A8" s="58" t="inlineStr">
+      <c r="A8" s="94" t="inlineStr">
         <is>
           <t>Baza</t>
         </is>
       </c>
-      <c r="B8" s="59" t="inlineStr">
+      <c r="B8" s="95" t="inlineStr">
         <is>
           <t>Buloane M12×180 + piulita + saiba</t>
         </is>
       </c>
-      <c r="C8" s="58" t="inlineStr">
+      <c r="C8" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -3476,7 +3570,7 @@
       <c r="E8" s="60" t="n">
         <v>12</v>
       </c>
-      <c r="F8" s="58" t="inlineStr">
+      <c r="F8" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -3485,7 +3579,7 @@
         <f>IF(AND(D8&lt;&gt;"",E8&lt;&gt;""),D8*E8,"")</f>
         <v/>
       </c>
-      <c r="H8" s="59" t="inlineStr">
+      <c r="H8" s="95" t="inlineStr">
         <is>
           <t>4× polita grinda spate + 8× baza stalpi (2/papuc)</t>
         </is>
@@ -3497,17 +3591,17 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="48">
-      <c r="A9" s="58" t="inlineStr">
+      <c r="A9" s="94" t="inlineStr">
         <is>
           <t>Joiste</t>
         </is>
       </c>
-      <c r="B9" s="59" t="inlineStr">
+      <c r="B9" s="95" t="inlineStr">
         <is>
           <t>Grinda 100×100×4000 (AVEM)</t>
         </is>
       </c>
-      <c r="C9" s="58" t="inlineStr">
+      <c r="C9" s="94" t="inlineStr">
         <is>
           <t>Leroy</t>
         </is>
@@ -3518,7 +3612,7 @@
       <c r="E9" s="60" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="58" t="inlineStr">
+      <c r="F9" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -3527,29 +3621,29 @@
         <f>IF(AND(D9&lt;&gt;"",E9&lt;&gt;""),D9*E9,"")</f>
         <v/>
       </c>
-      <c r="H9" s="59" t="inlineStr">
+      <c r="H9" s="95" t="inlineStr">
         <is>
           <t>Joiste podea fata-spate (consola 700)</t>
         </is>
       </c>
-      <c r="I9" s="63" t="inlineStr">
+      <c r="I9" s="96" t="inlineStr">
         <is>
           <t>AVEM</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="48">
-      <c r="A10" s="58" t="inlineStr">
+      <c r="A10" s="94" t="inlineStr">
         <is>
           <t>Joiste</t>
         </is>
       </c>
-      <c r="B10" s="59" t="inlineStr">
+      <c r="B10" s="95" t="inlineStr">
         <is>
           <t>KVH 100×100×4000 — inca 2 joiste</t>
         </is>
       </c>
-      <c r="C10" s="58" t="inlineStr">
+      <c r="C10" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -3560,7 +3654,7 @@
       <c r="E10" s="60" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="58" t="inlineStr">
+      <c r="F10" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -3569,7 +3663,7 @@
         <f>IF(AND(D10&lt;&gt;"",E10&lt;&gt;""),D10*E10,"")</f>
         <v/>
       </c>
-      <c r="H10" s="59" t="inlineStr">
+      <c r="H10" s="95" t="inlineStr">
         <is>
           <t>Completare la 6 joiste (interax ~430)</t>
         </is>
@@ -3581,17 +3675,17 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="48">
-      <c r="A11" s="58" t="inlineStr">
+      <c r="A11" s="94" t="inlineStr">
         <is>
           <t>Grinzi</t>
         </is>
       </c>
-      <c r="B11" s="59" t="inlineStr">
+      <c r="B11" s="95" t="inlineStr">
         <is>
           <t>Grinda lamelara Glulam 90×200×4000</t>
         </is>
       </c>
-      <c r="C11" s="58" t="inlineStr">
+      <c r="C11" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -3602,7 +3696,7 @@
       <c r="E11" s="60" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="58" t="inlineStr">
+      <c r="F11" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -3611,7 +3705,7 @@
         <f>IF(AND(D11&lt;&gt;"",E11&lt;&gt;""),D11*E11,"")</f>
         <v/>
       </c>
-      <c r="H11" s="59" t="inlineStr">
+      <c r="H11" s="95" t="inlineStr">
         <is>
           <t>Grinzi principale; fata pe varf, spate pe POLITA</t>
         </is>
@@ -3623,17 +3717,17 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="48">
-      <c r="A12" s="58" t="inlineStr">
+      <c r="A12" s="94" t="inlineStr">
         <is>
           <t>Grinzi</t>
         </is>
       </c>
-      <c r="B12" s="59" t="inlineStr">
+      <c r="B12" s="95" t="inlineStr">
         <is>
           <t>Polita lemn (din offcut 100×100)</t>
         </is>
       </c>
-      <c r="C12" s="58" t="inlineStr">
+      <c r="C12" s="94" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3644,7 +3738,7 @@
       <c r="E12" s="60" t="n">
         <v>2</v>
       </c>
-      <c r="F12" s="58" t="inlineStr">
+      <c r="F12" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -3653,12 +3747,12 @@
         <f>IF(AND(D12&lt;&gt;"",E12&lt;&gt;""),D12*E12,"")</f>
         <v/>
       </c>
-      <c r="H12" s="59" t="inlineStr">
+      <c r="H12" s="95" t="inlineStr">
         <is>
           <t>Sub grinda spate, bulonata cu M12</t>
         </is>
       </c>
-      <c r="I12" s="63" t="inlineStr">
+      <c r="I12" s="96" t="inlineStr">
         <is>
           <t>OFFCUT</t>
         </is>
@@ -3680,17 +3774,17 @@
       <c r="I13" s="84" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="48">
-      <c r="A14" s="58" t="inlineStr">
+      <c r="A14" s="94" t="inlineStr">
         <is>
           <t>Dusumea</t>
         </is>
       </c>
-      <c r="B14" s="59" t="inlineStr">
+      <c r="B14" s="95" t="inlineStr">
         <is>
           <t>Lemn terasa larice Konsta 28×145×3000</t>
         </is>
       </c>
-      <c r="C14" s="58" t="inlineStr">
+      <c r="C14" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -3701,7 +3795,7 @@
       <c r="E14" s="60" t="n">
         <v>17</v>
       </c>
-      <c r="F14" s="58" t="inlineStr">
+      <c r="F14" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -3710,7 +3804,7 @@
         <f>IF(AND(D14&lt;&gt;"",E14&lt;&gt;""),D14*E14,"")</f>
         <v/>
       </c>
-      <c r="H14" s="59" t="inlineStr">
+      <c r="H14" s="95" t="inlineStr">
         <is>
           <t>Dusumea premium 28mm</t>
         </is>
@@ -3737,17 +3831,17 @@
       <c r="I15" s="84" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="48">
-      <c r="A16" s="58" t="inlineStr">
+      <c r="A16" s="94" t="inlineStr">
         <is>
           <t>Conectori</t>
         </is>
       </c>
-      <c r="B16" s="59" t="inlineStr">
+      <c r="B16" s="95" t="inlineStr">
         <is>
           <t>Coltar rigidizat Alberts 100×100×90×3</t>
         </is>
       </c>
-      <c r="C16" s="58" t="inlineStr">
+      <c r="C16" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -3758,7 +3852,7 @@
       <c r="E16" s="60" t="n">
         <v>4</v>
       </c>
-      <c r="F16" s="58" t="inlineStr">
+      <c r="F16" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -3767,7 +3861,7 @@
         <f>IF(AND(D16&lt;&gt;"",E16&lt;&gt;""),D16*E16,"")</f>
         <v/>
       </c>
-      <c r="H16" s="59" t="inlineStr">
+      <c r="H16" s="95" t="inlineStr">
         <is>
           <t>Grinda FATA → stalp (pe varf)</t>
         </is>
@@ -3779,17 +3873,17 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="48">
-      <c r="A17" s="58" t="inlineStr">
+      <c r="A17" s="94" t="inlineStr">
         <is>
           <t>Conectori</t>
         </is>
       </c>
-      <c r="B17" s="59" t="inlineStr">
+      <c r="B17" s="95" t="inlineStr">
         <is>
           <t>Coltar rigidizat Alberts 90×90×65</t>
         </is>
       </c>
-      <c r="C17" s="58" t="inlineStr">
+      <c r="C17" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -3800,7 +3894,7 @@
       <c r="E17" s="60" t="n">
         <v>12</v>
       </c>
-      <c r="F17" s="58" t="inlineStr">
+      <c r="F17" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -3809,7 +3903,7 @@
         <f>IF(AND(D17&lt;&gt;"",E17&lt;&gt;""),D17*E17,"")</f>
         <v/>
       </c>
-      <c r="H17" s="59" t="inlineStr">
+      <c r="H17" s="95" t="inlineStr">
         <is>
           <t>Joiste → grinda, anti-ridicare</t>
         </is>
@@ -3821,17 +3915,17 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="48">
-      <c r="A18" s="58" t="inlineStr">
+      <c r="A18" s="94" t="inlineStr">
         <is>
           <t>Suruburi</t>
         </is>
       </c>
-      <c r="B18" s="59" t="inlineStr">
+      <c r="B18" s="95" t="inlineStr">
         <is>
           <t>Heco Topix-Plus 8×200 Torx (100 buc)</t>
         </is>
       </c>
-      <c r="C18" s="58" t="inlineStr">
+      <c r="C18" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -3842,7 +3936,7 @@
       <c r="E18" s="60" t="n">
         <v>1</v>
       </c>
-      <c r="F18" s="58" t="inlineStr">
+      <c r="F18" s="94" t="inlineStr">
         <is>
           <t>pac</t>
         </is>
@@ -3851,7 +3945,7 @@
         <f>IF(AND(D18&lt;&gt;"",E18&lt;&gt;""),D18*E18,"")</f>
         <v/>
       </c>
-      <c r="H18" s="59" t="inlineStr">
+      <c r="H18" s="95" t="inlineStr">
         <is>
           <t>Imbinari structurale, fara pre-gaurire</t>
         </is>
@@ -3863,28 +3957,28 @@
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="48">
-      <c r="A19" s="58" t="inlineStr">
+      <c r="A19" s="94" t="inlineStr">
         <is>
           <t>Suruburi</t>
         </is>
       </c>
-      <c r="B19" s="59" t="inlineStr">
-        <is>
-          <t>Heco Topix-Plus 6×100 inox A2 (100 buc)</t>
-        </is>
-      </c>
-      <c r="C19" s="58" t="inlineStr">
+      <c r="B19" s="95" t="inlineStr">
+        <is>
+          <t>Heco Topix-Plus 6x100 zincat (100 buc)</t>
+        </is>
+      </c>
+      <c r="C19" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
       <c r="D19" s="88" t="n">
-        <v>228.78</v>
+        <v>94.87</v>
       </c>
       <c r="E19" s="60" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="58" t="inlineStr">
+      <c r="F19" s="94" t="inlineStr">
         <is>
           <t>pac</t>
         </is>
@@ -3893,7 +3987,7 @@
         <f>IF(AND(D19&lt;&gt;"",E19&lt;&gt;""),D19*E19,"")</f>
         <v/>
       </c>
-      <c r="H19" s="59" t="inlineStr">
+      <c r="H19" s="95" t="inlineStr">
         <is>
           <t>Coltare, conectori, contrafise</t>
         </is>
@@ -3905,17 +3999,17 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="48">
-      <c r="A20" s="58" t="inlineStr">
+      <c r="A20" s="94" t="inlineStr">
         <is>
           <t>Suruburi</t>
         </is>
       </c>
-      <c r="B20" s="59" t="inlineStr">
+      <c r="B20" s="95" t="inlineStr">
         <is>
           <t>Heco Topix-Plus 6×80 (100 buc)</t>
         </is>
       </c>
-      <c r="C20" s="58" t="inlineStr">
+      <c r="C20" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -3926,7 +4020,7 @@
       <c r="E20" s="60" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="58" t="inlineStr">
+      <c r="F20" s="94" t="inlineStr">
         <is>
           <t>pac</t>
         </is>
@@ -3935,7 +4029,7 @@
         <f>IF(AND(D20&lt;&gt;"",E20&lt;&gt;""),D20*E20,"")</f>
         <v/>
       </c>
-      <c r="H20" s="59" t="inlineStr">
+      <c r="H20" s="95" t="inlineStr">
         <is>
           <t>Blocaje, prinderi generale</t>
         </is>
@@ -3947,28 +4041,28 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="48">
-      <c r="A21" s="58" t="inlineStr">
+      <c r="A21" s="94" t="inlineStr">
         <is>
           <t>Suruburi</t>
         </is>
       </c>
-      <c r="B21" s="59" t="inlineStr">
-        <is>
-          <t>Suruburi inox A2 5×60 dusumea (200)</t>
-        </is>
-      </c>
-      <c r="C21" s="58" t="inlineStr">
+      <c r="B21" s="95" t="inlineStr">
+        <is>
+          <t>Suruburi inox A2 5x60 dusumea (100 buc)</t>
+        </is>
+      </c>
+      <c r="C21" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
       <c r="D21" s="88" t="n">
-        <v>120</v>
+        <v>55.82</v>
       </c>
       <c r="E21" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="58" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="F21" s="94" t="inlineStr">
         <is>
           <t>pac</t>
         </is>
@@ -3977,14 +4071,14 @@
         <f>IF(AND(D21&lt;&gt;"",E21&lt;&gt;""),D21*E21,"")</f>
         <v/>
       </c>
-      <c r="H21" s="59" t="inlineStr">
+      <c r="H21" s="95" t="inlineStr">
         <is>
           <t>Prindere dusumea larice</t>
         </is>
       </c>
       <c r="I21" s="72" t="inlineStr">
         <is>
-          <t>De cumparat (est.)</t>
+          <t>De cumparat</t>
         </is>
       </c>
     </row>
@@ -4004,17 +4098,17 @@
       <c r="I22" s="84" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="48">
-      <c r="A23" s="58" t="inlineStr">
+      <c r="A23" s="94" t="inlineStr">
         <is>
           <t>Scara</t>
         </is>
       </c>
-      <c r="B23" s="59" t="inlineStr">
+      <c r="B23" s="95" t="inlineStr">
         <is>
           <t>Coarde scara KVH 60×140×3000</t>
         </is>
       </c>
-      <c r="C23" s="58" t="inlineStr">
+      <c r="C23" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -4025,7 +4119,7 @@
       <c r="E23" s="60" t="n">
         <v>2</v>
       </c>
-      <c r="F23" s="58" t="inlineStr">
+      <c r="F23" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -4034,7 +4128,7 @@
         <f>IF(AND(D23&lt;&gt;"",E23&lt;&gt;""),D23*E23,"")</f>
         <v/>
       </c>
-      <c r="H23" s="59" t="inlineStr">
+      <c r="H23" s="95" t="inlineStr">
         <is>
           <t>Cele 2 grinzi inclinate (~2,9 m)</t>
         </is>
@@ -4046,17 +4140,17 @@
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="48">
-      <c r="A24" s="58" t="inlineStr">
+      <c r="A24" s="94" t="inlineStr">
         <is>
           <t>Scara</t>
         </is>
       </c>
-      <c r="B24" s="59" t="inlineStr">
+      <c r="B24" s="95" t="inlineStr">
         <is>
           <t>Trepte larice/dulap 45×190 ~600 mm</t>
         </is>
       </c>
-      <c r="C24" s="58" t="inlineStr">
+      <c r="C24" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -4067,7 +4161,7 @@
       <c r="E24" s="60" t="n">
         <v>10</v>
       </c>
-      <c r="F24" s="58" t="inlineStr">
+      <c r="F24" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -4076,7 +4170,7 @@
         <f>IF(AND(D24&lt;&gt;"",E24&lt;&gt;""),D24*E24,"")</f>
         <v/>
       </c>
-      <c r="H24" s="59" t="inlineStr">
+      <c r="H24" s="95" t="inlineStr">
         <is>
           <t>11 trepte (riser 200, calcai 190)</t>
         </is>
@@ -4088,17 +4182,17 @@
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="48">
-      <c r="A25" s="58" t="inlineStr">
+      <c r="A25" s="94" t="inlineStr">
         <is>
           <t>Scara</t>
         </is>
       </c>
-      <c r="B25" s="59" t="inlineStr">
+      <c r="B25" s="95" t="inlineStr">
         <is>
           <t>Mana curenta + stalpisori (lemn)</t>
         </is>
       </c>
-      <c r="C25" s="58" t="inlineStr">
+      <c r="C25" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -4109,7 +4203,7 @@
       <c r="E25" s="60" t="n">
         <v>1</v>
       </c>
-      <c r="F25" s="58" t="inlineStr">
+      <c r="F25" s="94" t="inlineStr">
         <is>
           <t>set</t>
         </is>
@@ -4118,7 +4212,7 @@
         <f>IF(AND(D25&lt;&gt;"",E25&lt;&gt;""),D25*E25,"")</f>
         <v/>
       </c>
-      <c r="H25" s="59" t="inlineStr">
+      <c r="H25" s="95" t="inlineStr">
         <is>
           <t>Pe ambele parti</t>
         </is>
@@ -4130,17 +4224,17 @@
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="48">
-      <c r="A26" s="58" t="inlineStr">
+      <c r="A26" s="94" t="inlineStr">
         <is>
           <t>Scara</t>
         </is>
       </c>
-      <c r="B26" s="59" t="inlineStr">
+      <c r="B26" s="95" t="inlineStr">
         <is>
           <t>Feronerie scara (coltare + Heco + 2× M10)</t>
         </is>
       </c>
-      <c r="C26" s="58" t="inlineStr">
+      <c r="C26" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -4151,7 +4245,7 @@
       <c r="E26" s="60" t="n">
         <v>1</v>
       </c>
-      <c r="F26" s="58" t="inlineStr">
+      <c r="F26" s="94" t="inlineStr">
         <is>
           <t>set</t>
         </is>
@@ -4160,7 +4254,7 @@
         <f>IF(AND(D26&lt;&gt;"",E26&lt;&gt;""),D26*E26,"")</f>
         <v/>
       </c>
-      <c r="H26" s="59" t="inlineStr">
+      <c r="H26" s="95" t="inlineStr">
         <is>
           <t>Prindere de platforma + trepte</t>
         </is>
@@ -4172,17 +4266,17 @@
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="48">
-      <c r="A27" s="58" t="inlineStr">
+      <c r="A27" s="94" t="inlineStr">
         <is>
           <t>Scara</t>
         </is>
       </c>
-      <c r="B27" s="59" t="inlineStr">
+      <c r="B27" s="95" t="inlineStr">
         <is>
           <t>Dala/paver baza scara</t>
         </is>
       </c>
-      <c r="C27" s="58" t="inlineStr">
+      <c r="C27" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -4193,7 +4287,7 @@
       <c r="E27" s="60" t="n">
         <v>1</v>
       </c>
-      <c r="F27" s="58" t="inlineStr">
+      <c r="F27" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -4202,7 +4296,7 @@
         <f>IF(AND(D27&lt;&gt;"",E27&lt;&gt;""),D27*E27,"")</f>
         <v/>
       </c>
-      <c r="H27" s="59" t="inlineStr">
+      <c r="H27" s="95" t="inlineStr">
         <is>
           <t>Sub coarde, sa nu stea in pamant</t>
         </is>
@@ -4229,17 +4323,17 @@
       <c r="I28" s="84" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="48">
-      <c r="A29" s="58" t="inlineStr">
+      <c r="A29" s="94" t="inlineStr">
         <is>
           <t>Finisaj</t>
         </is>
       </c>
-      <c r="B29" s="59" t="inlineStr">
+      <c r="B29" s="95" t="inlineStr">
         <is>
           <t>Ulei lemn tec Hornbach Plus 2,5 l</t>
         </is>
       </c>
-      <c r="C29" s="58" t="inlineStr">
+      <c r="C29" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
@@ -4250,7 +4344,7 @@
       <c r="E29" s="60" t="n">
         <v>2</v>
       </c>
-      <c r="F29" s="58" t="inlineStr">
+      <c r="F29" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -4259,7 +4353,7 @@
         <f>IF(AND(D29&lt;&gt;"",E29&lt;&gt;""),D29*E29,"")</f>
         <v/>
       </c>
-      <c r="H29" s="59" t="inlineStr">
+      <c r="H29" s="95" t="inlineStr">
         <is>
           <t>Dusumea larice + grinzi/scara expuse</t>
         </is>
@@ -4271,28 +4365,28 @@
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="48">
-      <c r="A30" s="58" t="inlineStr">
+      <c r="A30" s="94" t="inlineStr">
         <is>
           <t>Finisaj</t>
         </is>
       </c>
-      <c r="B30" s="59" t="inlineStr">
-        <is>
-          <t>Lazura/protectie exterior structura</t>
-        </is>
-      </c>
-      <c r="C30" s="58" t="inlineStr">
+      <c r="B30" s="95" t="inlineStr">
+        <is>
+          <t>Lazura impregnare exterior 2,5 l (grund)</t>
+        </is>
+      </c>
+      <c r="C30" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
       <c r="D30" s="88" t="n">
-        <v>150</v>
+        <v>92.5</v>
       </c>
       <c r="E30" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="58" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="F30" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
@@ -4301,14 +4395,14 @@
         <f>IF(AND(D30&lt;&gt;"",E30&lt;&gt;""),D30*E30,"")</f>
         <v/>
       </c>
-      <c r="H30" s="59" t="inlineStr">
+      <c r="H30" s="95" t="inlineStr">
         <is>
           <t>Stalpi + joiste + capete</t>
         </is>
       </c>
       <c r="I30" s="72" t="inlineStr">
         <is>
-          <t>De cumparat (est.)</t>
+          <t>De cumparat</t>
         </is>
       </c>
     </row>
@@ -4440,12 +4534,12 @@
       <c r="G5" s="84" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="48">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="95" t="inlineStr">
         <is>
           <t>Grinda lamelara Glulam 90×200×4000</t>
         </is>
       </c>
-      <c r="B6" s="58" t="inlineStr">
+      <c r="B6" s="94" t="inlineStr">
         <is>
           <t>5483835</t>
         </is>
@@ -4460,24 +4554,24 @@
         <f>C6*D6</f>
         <v/>
       </c>
-      <c r="F6" s="63" t="inlineStr">
+      <c r="F6" s="96" t="inlineStr">
         <is>
           <t>IN COS</t>
         </is>
       </c>
-      <c r="G6" s="58" t="inlineStr">
+      <c r="G6" s="94" t="inlineStr">
         <is>
           <t>GR</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="48">
-      <c r="A7" s="59" t="inlineStr">
+      <c r="A7" s="95" t="inlineStr">
         <is>
           <t>KVH 100×100×4000 (joiste in plus)</t>
         </is>
       </c>
-      <c r="B7" s="58" t="inlineStr">
+      <c r="B7" s="94" t="inlineStr">
         <is>
           <t>7337253</t>
         </is>
@@ -4492,24 +4586,24 @@
         <f>C7*D7</f>
         <v/>
       </c>
-      <c r="F7" s="63" t="inlineStr">
+      <c r="F7" s="96" t="inlineStr">
         <is>
           <t>IN COS</t>
         </is>
       </c>
-      <c r="G7" s="58" t="inlineStr">
+      <c r="G7" s="94" t="inlineStr">
         <is>
           <t>JO</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="48">
-      <c r="A8" s="59" t="inlineStr">
+      <c r="A8" s="95" t="inlineStr">
         <is>
           <t>Lemn terasa larice Konsta 28×145×3000</t>
         </is>
       </c>
-      <c r="B8" s="58" t="inlineStr">
+      <c r="B8" s="94" t="inlineStr">
         <is>
           <t>6224073</t>
         </is>
@@ -4524,24 +4618,24 @@
         <f>C8*D8</f>
         <v/>
       </c>
-      <c r="F8" s="63" t="inlineStr">
+      <c r="F8" s="96" t="inlineStr">
         <is>
           <t>IN COS</t>
         </is>
       </c>
-      <c r="G8" s="58" t="inlineStr">
+      <c r="G8" s="94" t="inlineStr">
         <is>
           <t>DL</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="48">
-      <c r="A9" s="59" t="inlineStr">
+      <c r="A9" s="95" t="inlineStr">
         <is>
           <t>Coltar rigidizat Alberts 100×100×90×3</t>
         </is>
       </c>
-      <c r="B9" s="58" t="inlineStr">
+      <c r="B9" s="94" t="inlineStr">
         <is>
           <t>738965</t>
         </is>
@@ -4556,24 +4650,24 @@
         <f>C9*D9</f>
         <v/>
       </c>
-      <c r="F9" s="63" t="inlineStr">
+      <c r="F9" s="96" t="inlineStr">
         <is>
           <t>IN COS</t>
         </is>
       </c>
-      <c r="G9" s="58" t="inlineStr">
+      <c r="G9" s="94" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="48">
-      <c r="A10" s="59" t="inlineStr">
+      <c r="A10" s="95" t="inlineStr">
         <is>
           <t>Coltar rigidizat Alberts 90×90×65×2,5</t>
         </is>
       </c>
-      <c r="B10" s="58" t="inlineStr">
+      <c r="B10" s="94" t="inlineStr">
         <is>
           <t>738910</t>
         </is>
@@ -4588,24 +4682,24 @@
         <f>C10*D10</f>
         <v/>
       </c>
-      <c r="F10" s="63" t="inlineStr">
+      <c r="F10" s="96" t="inlineStr">
         <is>
           <t>IN COS</t>
         </is>
       </c>
-      <c r="G10" s="58" t="inlineStr">
+      <c r="G10" s="94" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="48">
-      <c r="A11" s="59" t="inlineStr">
+      <c r="A11" s="95" t="inlineStr">
         <is>
           <t>Heco Topix-Plus 8×200 zincat (100 buc)</t>
         </is>
       </c>
-      <c r="B11" s="58" t="inlineStr">
+      <c r="B11" s="94" t="inlineStr">
         <is>
           <t>10434633</t>
         </is>
@@ -4620,24 +4714,24 @@
         <f>C11*D11</f>
         <v/>
       </c>
-      <c r="F11" s="63" t="inlineStr">
+      <c r="F11" s="96" t="inlineStr">
         <is>
           <t>IN COS</t>
         </is>
       </c>
-      <c r="G11" s="58" t="inlineStr">
+      <c r="G11" s="94" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="48">
-      <c r="A12" s="59" t="inlineStr">
+      <c r="A12" s="95" t="inlineStr">
         <is>
           <t>Heco Topix-Plus 6×100 ZINCAT albastru (100 buc)</t>
         </is>
       </c>
-      <c r="B12" s="58" t="inlineStr">
+      <c r="B12" s="94" t="inlineStr">
         <is>
           <t>10434398</t>
         </is>
@@ -4652,24 +4746,24 @@
         <f>C12*D12</f>
         <v/>
       </c>
-      <c r="F12" s="63" t="inlineStr">
+      <c r="F12" s="96" t="inlineStr">
         <is>
           <t>IN COS</t>
         </is>
       </c>
-      <c r="G12" s="58" t="inlineStr">
+      <c r="G12" s="94" t="inlineStr">
         <is>
           <t>H2</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="48">
-      <c r="A13" s="59" t="inlineStr">
+      <c r="A13" s="95" t="inlineStr">
         <is>
           <t>Heco Topix-Plus 6×80 zincat (100 buc)</t>
         </is>
       </c>
-      <c r="B13" s="58" t="inlineStr">
+      <c r="B13" s="94" t="inlineStr">
         <is>
           <t>10434139</t>
         </is>
@@ -4684,24 +4778,24 @@
         <f>C13*D13</f>
         <v/>
       </c>
-      <c r="F13" s="63" t="inlineStr">
+      <c r="F13" s="96" t="inlineStr">
         <is>
           <t>IN COS</t>
         </is>
       </c>
-      <c r="G13" s="58" t="inlineStr">
+      <c r="G13" s="94" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="48">
-      <c r="A14" s="59" t="inlineStr">
+      <c r="A14" s="95" t="inlineStr">
         <is>
           <t>Suruburi terasa inox A2 5×60 (100 buc)</t>
         </is>
       </c>
-      <c r="B14" s="58" t="inlineStr">
+      <c r="B14" s="94" t="inlineStr">
         <is>
           <t>10528829</t>
         </is>
@@ -4716,24 +4810,24 @@
         <f>C14*D14</f>
         <v/>
       </c>
-      <c r="F14" s="63" t="inlineStr">
+      <c r="F14" s="96" t="inlineStr">
         <is>
           <t>IN COS</t>
         </is>
       </c>
-      <c r="G14" s="58" t="inlineStr">
+      <c r="G14" s="94" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="48">
-      <c r="A15" s="59" t="inlineStr">
+      <c r="A15" s="95" t="inlineStr">
         <is>
           <t>Surub hexagonal M12×120 inox A2 (25 buc) — baza papuc</t>
         </is>
       </c>
-      <c r="B15" s="58" t="inlineStr">
+      <c r="B15" s="94" t="inlineStr">
         <is>
           <t>6834285</t>
         </is>
@@ -4748,24 +4842,24 @@
         <f>C15*D15</f>
         <v/>
       </c>
-      <c r="F15" s="63" t="inlineStr">
+      <c r="F15" s="96" t="inlineStr">
         <is>
           <t>IN COS</t>
         </is>
       </c>
-      <c r="G15" s="58" t="inlineStr">
+      <c r="G15" s="94" t="inlineStr">
         <is>
           <t>B2</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="48">
-      <c r="A16" s="59" t="inlineStr">
+      <c r="A16" s="95" t="inlineStr">
         <is>
           <t>Ulei lemn tec Hornbach Plus 2,5 l (dusumea)</t>
         </is>
       </c>
-      <c r="B16" s="58" t="inlineStr">
+      <c r="B16" s="94" t="inlineStr">
         <is>
           <t>5509678</t>
         </is>
@@ -4780,24 +4874,24 @@
         <f>C16*D16</f>
         <v/>
       </c>
-      <c r="F16" s="63" t="inlineStr">
+      <c r="F16" s="96" t="inlineStr">
         <is>
           <t>IN COS</t>
         </is>
       </c>
-      <c r="G16" s="58" t="inlineStr">
+      <c r="G16" s="94" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16.5" customHeight="1" s="48">
-      <c r="A17" s="59" t="inlineStr">
+      <c r="A17" s="95" t="inlineStr">
         <is>
           <t>Saibe late M12 13×30 zincat (100 buc)</t>
         </is>
       </c>
-      <c r="B17" s="58" t="inlineStr">
+      <c r="B17" s="94" t="inlineStr">
         <is>
           <t>3840897</t>
         </is>
@@ -4812,24 +4906,24 @@
         <f>C17*D17</f>
         <v/>
       </c>
-      <c r="F17" s="63" t="inlineStr">
+      <c r="F17" s="96" t="inlineStr">
         <is>
           <t>IN COS</t>
         </is>
       </c>
-      <c r="G17" s="58" t="inlineStr">
+      <c r="G17" s="94" t="inlineStr">
         <is>
           <t>B3</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="48">
-      <c r="A18" s="59" t="inlineStr">
+      <c r="A18" s="95" t="inlineStr">
         <is>
           <t>Lazura impregnare Hornbach exterior 2,5 l (grund)</t>
         </is>
       </c>
-      <c r="B18" s="58" t="inlineStr">
+      <c r="B18" s="94" t="inlineStr">
         <is>
           <t>12469765</t>
         </is>
@@ -4844,12 +4938,12 @@
         <f>C18*D18</f>
         <v/>
       </c>
-      <c r="F18" s="63" t="inlineStr">
+      <c r="F18" s="96" t="inlineStr">
         <is>
           <t>IN COS</t>
         </is>
       </c>
-      <c r="G18" s="58" t="inlineStr">
+      <c r="G18" s="94" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
@@ -4869,12 +4963,12 @@
       <c r="G19" s="84" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="48">
-      <c r="A20" s="59" t="inlineStr">
+      <c r="A20" s="95" t="inlineStr">
         <is>
           <t>Bulon M12 POLITA lung ~200 (set cu piulita, 25 buc)</t>
         </is>
       </c>
-      <c r="B20" s="58" t="inlineStr">
+      <c r="B20" s="94" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4889,24 +4983,24 @@
         <f>C20*D20</f>
         <v/>
       </c>
-      <c r="F20" s="63" t="inlineStr">
+      <c r="F20" s="96" t="inlineStr">
         <is>
           <t>de confirmat</t>
         </is>
       </c>
-      <c r="G20" s="58" t="inlineStr">
+      <c r="G20" s="94" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="48">
-      <c r="A21" s="59" t="inlineStr">
+      <c r="A21" s="95" t="inlineStr">
         <is>
           <t>Piulite M12 — din raft la magazin</t>
         </is>
       </c>
-      <c r="B21" s="58" t="inlineStr">
+      <c r="B21" s="94" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4921,24 +5015,24 @@
         <f>C21*D21</f>
         <v/>
       </c>
-      <c r="F21" s="63" t="inlineStr">
+      <c r="F21" s="96" t="inlineStr">
         <is>
           <t>de confirmat</t>
         </is>
       </c>
-      <c r="G21" s="58" t="inlineStr">
+      <c r="G21" s="94" t="inlineStr">
         <is>
           <t>B4</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="48">
-      <c r="A22" s="59" t="inlineStr">
+      <c r="A22" s="95" t="inlineStr">
         <is>
           <t>Topcoat: lazura colorata / vopsea exterior (culoarea ta)</t>
         </is>
       </c>
-      <c r="B22" s="58" t="inlineStr">
+      <c r="B22" s="94" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4953,24 +5047,24 @@
         <f>C22*D22</f>
         <v/>
       </c>
-      <c r="F22" s="63" t="inlineStr">
+      <c r="F22" s="96" t="inlineStr">
         <is>
           <t>de confirmat</t>
         </is>
       </c>
-      <c r="G22" s="58" t="inlineStr">
+      <c r="G22" s="94" t="inlineStr">
         <is>
           <t>F3</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="48">
-      <c r="A23" s="59" t="inlineStr">
+      <c r="A23" s="95" t="inlineStr">
         <is>
           <t>KVH coarde scara ~60×140×3000 (Faza 2)</t>
         </is>
       </c>
-      <c r="B23" s="58" t="inlineStr">
+      <c r="B23" s="94" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4985,24 +5079,24 @@
         <f>C23*D23</f>
         <v/>
       </c>
-      <c r="F23" s="63" t="inlineStr">
+      <c r="F23" s="96" t="inlineStr">
         <is>
           <t>de confirmat</t>
         </is>
       </c>
-      <c r="G23" s="58" t="inlineStr">
+      <c r="G23" s="94" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="48">
-      <c r="A24" s="59" t="inlineStr">
+      <c r="A24" s="95" t="inlineStr">
         <is>
           <t>Trepte larice/dulap ~45×190, ~600 mm (Faza 2)</t>
         </is>
       </c>
-      <c r="B24" s="58" t="inlineStr">
+      <c r="B24" s="94" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5017,24 +5111,24 @@
         <f>C24*D24</f>
         <v/>
       </c>
-      <c r="F24" s="63" t="inlineStr">
+      <c r="F24" s="96" t="inlineStr">
         <is>
           <t>de confirmat</t>
         </is>
       </c>
-      <c r="G24" s="58" t="inlineStr">
+      <c r="G24" s="94" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="48">
-      <c r="A25" s="59" t="inlineStr">
+      <c r="A25" s="95" t="inlineStr">
         <is>
           <t>Lemn mana curenta + stalpisori scara (Faza 2)</t>
         </is>
       </c>
-      <c r="B25" s="58" t="inlineStr">
+      <c r="B25" s="94" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5049,24 +5143,24 @@
         <f>C25*D25</f>
         <v/>
       </c>
-      <c r="F25" s="63" t="inlineStr">
+      <c r="F25" s="96" t="inlineStr">
         <is>
           <t>de confirmat</t>
         </is>
       </c>
-      <c r="G25" s="58" t="inlineStr">
+      <c r="G25" s="94" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="48">
-      <c r="A26" s="59" t="inlineStr">
+      <c r="A26" s="95" t="inlineStr">
         <is>
           <t>Dala/paver baza scara (Faza 2)</t>
         </is>
       </c>
-      <c r="B26" s="58" t="inlineStr">
+      <c r="B26" s="94" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5081,12 +5175,12 @@
         <f>C26*D26</f>
         <v/>
       </c>
-      <c r="F26" s="63" t="inlineStr">
+      <c r="F26" s="96" t="inlineStr">
         <is>
           <t>de confirmat</t>
         </is>
       </c>
-      <c r="G26" s="58" t="inlineStr">
+      <c r="G26" s="94" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5243,12 +5337,12 @@
       <c r="H5" s="84" t="n"/>
     </row>
     <row r="6" ht="21.75" customHeight="1" s="48">
-      <c r="A6" s="58" t="inlineStr">
+      <c r="A6" s="94" t="inlineStr">
         <is>
           <t>Electrice</t>
         </is>
       </c>
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="95" t="inlineStr">
         <is>
           <t>Masina de insurubat cu impact + biti Torx TX40 &amp; TX30</t>
         </is>
@@ -5258,23 +5352,23 @@
           <t>Esential</t>
         </is>
       </c>
-      <c r="D6" s="85" t="n"/>
-      <c r="E6" s="85" t="n"/>
-      <c r="F6" s="85" t="n"/>
-      <c r="G6" s="85" t="n"/>
-      <c r="H6" s="59" t="inlineStr">
+      <c r="D6" s="97" t="n"/>
+      <c r="E6" s="97" t="n"/>
+      <c r="F6" s="97" t="n"/>
+      <c r="G6" s="97" t="n"/>
+      <c r="H6" s="95" t="inlineStr">
         <is>
           <t>Inima montajului — pt suruburile Heco</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="48">
-      <c r="A7" s="58" t="inlineStr">
+      <c r="A7" s="94" t="inlineStr">
         <is>
           <t>Electrice</t>
         </is>
       </c>
-      <c r="B7" s="59" t="inlineStr">
+      <c r="B7" s="95" t="inlineStr">
         <is>
           <t>Bormasina + burghie de lemn</t>
         </is>
@@ -5284,41 +5378,41 @@
           <t>Esential</t>
         </is>
       </c>
-      <c r="D7" s="85" t="n"/>
-      <c r="E7" s="85" t="n"/>
-      <c r="F7" s="85" t="n"/>
-      <c r="G7" s="85" t="n"/>
-      <c r="H7" s="59" t="inlineStr">
+      <c r="D7" s="97" t="n"/>
+      <c r="E7" s="97" t="n"/>
+      <c r="F7" s="97" t="n"/>
+      <c r="G7" s="97" t="n"/>
+      <c r="H7" s="95" t="inlineStr">
         <is>
           <t>Pregaurit DOAR la buloanele M12</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="48">
-      <c r="A8" s="58" t="inlineStr">
+      <c r="A8" s="94" t="inlineStr">
         <is>
           <t>Electrice</t>
         </is>
       </c>
-      <c r="B8" s="59" t="inlineStr">
+      <c r="B8" s="95" t="inlineStr">
         <is>
           <t>Fierastrau de retezat glisant</t>
         </is>
       </c>
-      <c r="C8" s="63" t="inlineStr">
+      <c r="C8" s="96" t="inlineStr">
         <is>
           <t>Esential</t>
         </is>
       </c>
-      <c r="D8" s="85" t="n"/>
-      <c r="E8" s="85" t="n"/>
-      <c r="F8" s="85" t="n"/>
-      <c r="G8" s="85" t="inlineStr">
+      <c r="D8" s="97" t="n"/>
+      <c r="E8" s="97" t="n"/>
+      <c r="F8" s="97" t="n"/>
+      <c r="G8" s="97" t="inlineStr">
         <is>
           <t>80–120/zi</t>
         </is>
       </c>
-      <c r="H8" s="59" t="inlineStr">
+      <c r="H8" s="95" t="inlineStr">
         <is>
           <t>SCULA PRINCIPALA de taiat — singura cu taietura perfect dreapta pe stalpi 100x100 si glulam. Capul stalpilor e portant.</t>
         </is>
@@ -5360,33 +5454,21 @@
           <t>Electrice</t>
         </is>
       </c>
-      <c r="B10" s="95" t="inlineStr">
-        <is>
-          <t>Panza de mana (coada de vulpe)</t>
-        </is>
-      </c>
-      <c r="C10" s="96" t="inlineStr">
-        <is>
-          <t>Esential</t>
-        </is>
-      </c>
-      <c r="D10" s="97" t="n"/>
-      <c r="E10" s="97" t="n"/>
-      <c r="F10" s="97" t="n"/>
-      <c r="G10" s="97" t="n"/>
-      <c r="H10" s="95" t="inlineStr">
-        <is>
-          <t>Backup fara curent + finisat miezul. Varianta ieftina: circular pe 4 fete cu echer, finisezi miezul cu panza.</t>
-        </is>
-      </c>
+      <c r="B10" s="83" t="n"/>
+      <c r="C10" s="83" t="n"/>
+      <c r="D10" s="83" t="n"/>
+      <c r="E10" s="83" t="n"/>
+      <c r="F10" s="83" t="n"/>
+      <c r="G10" s="83" t="n"/>
+      <c r="H10" s="84" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="48">
-      <c r="A11" s="58" t="inlineStr">
+      <c r="A11" s="94" t="inlineStr">
         <is>
           <t>Electrice</t>
         </is>
       </c>
-      <c r="B11" s="59" t="inlineStr">
+      <c r="B11" s="95" t="inlineStr">
         <is>
           <t>Fierastrau pendular</t>
         </is>
@@ -5396,11 +5478,11 @@
           <t>Optional</t>
         </is>
       </c>
-      <c r="D11" s="85" t="n"/>
-      <c r="E11" s="85" t="n"/>
-      <c r="F11" s="85" t="n"/>
-      <c r="G11" s="85" t="n"/>
-      <c r="H11" s="59" t="inlineStr">
+      <c r="D11" s="97" t="n"/>
+      <c r="E11" s="97" t="n"/>
+      <c r="F11" s="97" t="n"/>
+      <c r="G11" s="97" t="n"/>
+      <c r="H11" s="95" t="inlineStr">
         <is>
           <t>Decupajul gaurii pentru copac</t>
         </is>
@@ -5421,12 +5503,12 @@
       <c r="H12" s="84" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="48">
-      <c r="A13" s="58" t="inlineStr">
+      <c r="A13" s="94" t="inlineStr">
         <is>
           <t>Masurat</t>
         </is>
       </c>
-      <c r="B13" s="59" t="inlineStr">
+      <c r="B13" s="95" t="inlineStr">
         <is>
           <t>Nivela laser (sau nivela lunga 1–2 m)</t>
         </is>
@@ -5436,23 +5518,23 @@
           <t>Esential</t>
         </is>
       </c>
-      <c r="D13" s="85" t="n"/>
-      <c r="E13" s="85" t="n"/>
-      <c r="F13" s="85" t="n"/>
-      <c r="G13" s="85" t="n"/>
-      <c r="H13" s="59" t="inlineStr">
+      <c r="D13" s="97" t="n"/>
+      <c r="E13" s="97" t="n"/>
+      <c r="F13" s="97" t="n"/>
+      <c r="G13" s="97" t="n"/>
+      <c r="H13" s="95" t="inlineStr">
         <is>
           <t>Transfer nivel pe toti 4 stalpii</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="48">
-      <c r="A14" s="58" t="inlineStr">
+      <c r="A14" s="94" t="inlineStr">
         <is>
           <t>Masurat</t>
         </is>
       </c>
-      <c r="B14" s="59" t="inlineStr">
+      <c r="B14" s="95" t="inlineStr">
         <is>
           <t>Nivela cu bula mica</t>
         </is>
@@ -5462,23 +5544,23 @@
           <t>Esential</t>
         </is>
       </c>
-      <c r="D14" s="85" t="n"/>
-      <c r="E14" s="85" t="n"/>
-      <c r="F14" s="85" t="n"/>
-      <c r="G14" s="85" t="n"/>
-      <c r="H14" s="59" t="inlineStr">
+      <c r="D14" s="97" t="n"/>
+      <c r="E14" s="97" t="n"/>
+      <c r="F14" s="97" t="n"/>
+      <c r="G14" s="97" t="n"/>
+      <c r="H14" s="95" t="inlineStr">
         <is>
           <t>Verticalitatea stalpilor</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="48">
-      <c r="A15" s="58" t="inlineStr">
+      <c r="A15" s="94" t="inlineStr">
         <is>
           <t>Masurat</t>
         </is>
       </c>
-      <c r="B15" s="59" t="inlineStr">
+      <c r="B15" s="95" t="inlineStr">
         <is>
           <t>Ruleta 5 m + creion de tamplarie</t>
         </is>
@@ -5488,45 +5570,33 @@
           <t>Esential</t>
         </is>
       </c>
-      <c r="D15" s="85" t="n"/>
-      <c r="E15" s="85" t="n"/>
-      <c r="F15" s="85" t="n"/>
-      <c r="G15" s="85" t="n"/>
-      <c r="H15" s="59" t="n"/>
+      <c r="D15" s="97" t="n"/>
+      <c r="E15" s="97" t="n"/>
+      <c r="F15" s="97" t="n"/>
+      <c r="G15" s="97" t="n"/>
+      <c r="H15" s="95" t="n"/>
     </row>
     <row r="16" ht="16.5" customHeight="1" s="48">
-      <c r="A16" s="58" t="inlineStr">
+      <c r="A16" s="94" t="inlineStr">
         <is>
           <t>Masurat</t>
         </is>
       </c>
-      <c r="B16" s="59" t="inlineStr">
-        <is>
-          <t>Sfoara de trasat (chalk line)</t>
-        </is>
-      </c>
-      <c r="C16" s="72" t="inlineStr">
-        <is>
-          <t>Util</t>
-        </is>
-      </c>
-      <c r="D16" s="85" t="n"/>
-      <c r="E16" s="85" t="n"/>
-      <c r="F16" s="85" t="n"/>
-      <c r="G16" s="85" t="n"/>
-      <c r="H16" s="59" t="inlineStr">
-        <is>
-          <t>Linii lungi drepte</t>
-        </is>
-      </c>
+      <c r="B16" s="83" t="n"/>
+      <c r="C16" s="83" t="n"/>
+      <c r="D16" s="83" t="n"/>
+      <c r="E16" s="83" t="n"/>
+      <c r="F16" s="83" t="n"/>
+      <c r="G16" s="83" t="n"/>
+      <c r="H16" s="84" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="48">
-      <c r="A17" s="58" t="inlineStr">
+      <c r="A17" s="94" t="inlineStr">
         <is>
           <t>Masurat</t>
         </is>
       </c>
-      <c r="B17" s="59" t="inlineStr">
+      <c r="B17" s="95" t="inlineStr">
         <is>
           <t>Echer mare (vinclu)</t>
         </is>
@@ -5536,11 +5606,11 @@
           <t>Esential</t>
         </is>
       </c>
-      <c r="D17" s="85" t="n"/>
-      <c r="E17" s="85" t="n"/>
-      <c r="F17" s="85" t="n"/>
-      <c r="G17" s="85" t="n"/>
-      <c r="H17" s="59" t="inlineStr">
+      <c r="D17" s="97" t="n"/>
+      <c r="E17" s="97" t="n"/>
+      <c r="F17" s="97" t="n"/>
+      <c r="G17" s="97" t="n"/>
+      <c r="H17" s="95" t="inlineStr">
         <is>
           <t>Taieturi la 90°, colturi drepte</t>
         </is>
@@ -5561,12 +5631,12 @@
       <c r="H18" s="84" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="48">
-      <c r="A19" s="58" t="inlineStr">
+      <c r="A19" s="94" t="inlineStr">
         <is>
           <t>Mana</t>
         </is>
       </c>
-      <c r="B19" s="59" t="inlineStr">
+      <c r="B19" s="95" t="inlineStr">
         <is>
           <t>Cheie cu clichet + tubulara 17/19</t>
         </is>
@@ -5576,23 +5646,23 @@
           <t>Esential</t>
         </is>
       </c>
-      <c r="D19" s="85" t="n"/>
-      <c r="E19" s="85" t="n"/>
-      <c r="F19" s="85" t="n"/>
-      <c r="G19" s="85" t="n"/>
-      <c r="H19" s="59" t="inlineStr">
+      <c r="D19" s="97" t="n"/>
+      <c r="E19" s="97" t="n"/>
+      <c r="F19" s="97" t="n"/>
+      <c r="G19" s="97" t="n"/>
+      <c r="H19" s="95" t="inlineStr">
         <is>
           <t>Buloanele M12 (polita)</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="48">
-      <c r="A20" s="58" t="inlineStr">
+      <c r="A20" s="94" t="inlineStr">
         <is>
           <t>Mana</t>
         </is>
       </c>
-      <c r="B20" s="59" t="inlineStr">
+      <c r="B20" s="95" t="inlineStr">
         <is>
           <t>Ciocan</t>
         </is>
@@ -5602,19 +5672,19 @@
           <t>Esential</t>
         </is>
       </c>
-      <c r="D20" s="85" t="n"/>
-      <c r="E20" s="85" t="n"/>
-      <c r="F20" s="85" t="n"/>
-      <c r="G20" s="85" t="n"/>
-      <c r="H20" s="59" t="n"/>
+      <c r="D20" s="97" t="n"/>
+      <c r="E20" s="97" t="n"/>
+      <c r="F20" s="97" t="n"/>
+      <c r="G20" s="97" t="n"/>
+      <c r="H20" s="95" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="48">
-      <c r="A21" s="58" t="inlineStr">
+      <c r="A21" s="94" t="inlineStr">
         <is>
           <t>Mana</t>
         </is>
       </c>
-      <c r="B21" s="59" t="inlineStr">
+      <c r="B21" s="95" t="inlineStr">
         <is>
           <t>Set biti / surubelnite</t>
         </is>
@@ -5624,59 +5694,47 @@
           <t>Esential</t>
         </is>
       </c>
-      <c r="D21" s="85" t="n"/>
-      <c r="E21" s="85" t="n"/>
-      <c r="F21" s="85" t="n"/>
-      <c r="G21" s="85" t="n"/>
-      <c r="H21" s="59" t="n"/>
+      <c r="D21" s="97" t="n"/>
+      <c r="E21" s="97" t="n"/>
+      <c r="F21" s="97" t="n"/>
+      <c r="G21" s="97" t="n"/>
+      <c r="H21" s="95" t="n"/>
     </row>
     <row r="22" ht="16.5" customHeight="1" s="48">
-      <c r="A22" s="58" t="inlineStr">
+      <c r="A22" s="94" t="inlineStr">
         <is>
           <t>Mana</t>
         </is>
       </c>
-      <c r="B22" s="59" t="inlineStr">
-        <is>
-          <t>Dalta de lemn</t>
-        </is>
-      </c>
-      <c r="C22" s="72" t="inlineStr">
+      <c r="B22" s="83" t="n"/>
+      <c r="C22" s="83" t="n"/>
+      <c r="D22" s="83" t="n"/>
+      <c r="E22" s="83" t="n"/>
+      <c r="F22" s="83" t="n"/>
+      <c r="G22" s="83" t="n"/>
+      <c r="H22" s="84" t="n"/>
+    </row>
+    <row r="23" ht="15" customHeight="1" s="48">
+      <c r="A23" s="94" t="inlineStr">
+        <is>
+          <t>Mana</t>
+        </is>
+      </c>
+      <c r="B23" s="95" t="inlineStr">
+        <is>
+          <t>Cleste</t>
+        </is>
+      </c>
+      <c r="C23" s="72" t="inlineStr">
         <is>
           <t>Util</t>
         </is>
       </c>
-      <c r="D22" s="85" t="n"/>
-      <c r="E22" s="85" t="n"/>
-      <c r="F22" s="85" t="n"/>
-      <c r="G22" s="85" t="n"/>
-      <c r="H22" s="59" t="inlineStr">
-        <is>
-          <t>Ajustari, decupaje</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="48">
-      <c r="A23" s="58" t="inlineStr">
-        <is>
-          <t>Mana</t>
-        </is>
-      </c>
-      <c r="B23" s="59" t="inlineStr">
-        <is>
-          <t>Cleste</t>
-        </is>
-      </c>
-      <c r="C23" s="72" t="inlineStr">
-        <is>
-          <t>Util</t>
-        </is>
-      </c>
-      <c r="D23" s="85" t="n"/>
-      <c r="E23" s="85" t="n"/>
-      <c r="F23" s="85" t="n"/>
-      <c r="G23" s="85" t="n"/>
-      <c r="H23" s="59" t="n"/>
+      <c r="D23" s="97" t="n"/>
+      <c r="E23" s="97" t="n"/>
+      <c r="F23" s="97" t="n"/>
+      <c r="G23" s="97" t="n"/>
+      <c r="H23" s="95" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="48">
       <c r="A24" s="82" t="inlineStr">
@@ -5693,12 +5751,12 @@
       <c r="H24" s="84" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="48">
-      <c r="A25" s="58" t="inlineStr">
+      <c r="A25" s="94" t="inlineStr">
         <is>
           <t>Prindere</t>
         </is>
       </c>
-      <c r="B25" s="59" t="inlineStr">
+      <c r="B25" s="95" t="inlineStr">
         <is>
           <t>Cleme / menghine (clamps) — 2 pana la 4 buc</t>
         </is>
@@ -5708,49 +5766,37 @@
           <t>Esential</t>
         </is>
       </c>
-      <c r="D25" s="85" t="n"/>
-      <c r="E25" s="85" t="n"/>
-      <c r="F25" s="85" t="n"/>
-      <c r="G25" s="85" t="n"/>
-      <c r="H25" s="59" t="inlineStr">
+      <c r="D25" s="97" t="n"/>
+      <c r="E25" s="97" t="n"/>
+      <c r="F25" s="97" t="n"/>
+      <c r="G25" s="97" t="n"/>
+      <c r="H25" s="95" t="inlineStr">
         <is>
           <t>Tin piesele fixe cat insurubezi (vital in doi)</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16.5" customHeight="1" s="48">
-      <c r="A26" s="58" t="inlineStr">
+      <c r="A26" s="94" t="inlineStr">
         <is>
           <t>Acces</t>
         </is>
       </c>
-      <c r="B26" s="59" t="inlineStr">
-        <is>
-          <t>Scara / schela mica</t>
-        </is>
-      </c>
-      <c r="C26" s="74" t="inlineStr">
-        <is>
-          <t>Esential</t>
-        </is>
-      </c>
-      <c r="D26" s="85" t="n"/>
-      <c r="E26" s="85" t="n"/>
-      <c r="F26" s="85" t="n"/>
-      <c r="G26" s="85" t="n"/>
-      <c r="H26" s="59" t="inlineStr">
-        <is>
-          <t>Lucru la ~2 m</t>
-        </is>
-      </c>
+      <c r="B26" s="83" t="n"/>
+      <c r="C26" s="83" t="n"/>
+      <c r="D26" s="83" t="n"/>
+      <c r="E26" s="83" t="n"/>
+      <c r="F26" s="83" t="n"/>
+      <c r="G26" s="83" t="n"/>
+      <c r="H26" s="84" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="48">
-      <c r="A27" s="58" t="inlineStr">
+      <c r="A27" s="94" t="inlineStr">
         <is>
           <t>Acces</t>
         </is>
       </c>
-      <c r="B27" s="59" t="inlineStr">
+      <c r="B27" s="95" t="inlineStr">
         <is>
           <t>Capre de taiat (banc improvizat)</t>
         </is>
@@ -5760,11 +5806,11 @@
           <t>Util</t>
         </is>
       </c>
-      <c r="D27" s="85" t="n"/>
-      <c r="E27" s="85" t="n"/>
-      <c r="F27" s="85" t="n"/>
-      <c r="G27" s="85" t="n"/>
-      <c r="H27" s="59" t="inlineStr">
+      <c r="D27" s="97" t="n"/>
+      <c r="E27" s="97" t="n"/>
+      <c r="F27" s="97" t="n"/>
+      <c r="G27" s="97" t="n"/>
+      <c r="H27" s="95" t="inlineStr">
         <is>
           <t>Taiat comod la inaltime de lucru</t>
         </is>
@@ -5785,12 +5831,12 @@
       <c r="H28" s="84" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="48">
-      <c r="A29" s="58" t="inlineStr">
+      <c r="A29" s="94" t="inlineStr">
         <is>
           <t>Protectie</t>
         </is>
       </c>
-      <c r="B29" s="59" t="inlineStr">
+      <c r="B29" s="95" t="inlineStr">
         <is>
           <t>Ochelari de protectie</t>
         </is>
@@ -5800,19 +5846,19 @@
           <t>Esential</t>
         </is>
       </c>
-      <c r="D29" s="85" t="n"/>
-      <c r="E29" s="85" t="n"/>
-      <c r="F29" s="85" t="n"/>
-      <c r="G29" s="85" t="n"/>
-      <c r="H29" s="59" t="n"/>
+      <c r="D29" s="97" t="n"/>
+      <c r="E29" s="97" t="n"/>
+      <c r="F29" s="97" t="n"/>
+      <c r="G29" s="97" t="n"/>
+      <c r="H29" s="95" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="48">
-      <c r="A30" s="58" t="inlineStr">
+      <c r="A30" s="94" t="inlineStr">
         <is>
           <t>Protectie</t>
         </is>
       </c>
-      <c r="B30" s="59" t="inlineStr">
+      <c r="B30" s="95" t="inlineStr">
         <is>
           <t>Manusi de lucru</t>
         </is>
@@ -5822,45 +5868,33 @@
           <t>Esential</t>
         </is>
       </c>
-      <c r="D30" s="85" t="n"/>
-      <c r="E30" s="85" t="n"/>
-      <c r="F30" s="85" t="n"/>
-      <c r="G30" s="85" t="n"/>
-      <c r="H30" s="59" t="n"/>
+      <c r="D30" s="97" t="n"/>
+      <c r="E30" s="97" t="n"/>
+      <c r="F30" s="97" t="n"/>
+      <c r="G30" s="97" t="n"/>
+      <c r="H30" s="95" t="n"/>
     </row>
     <row r="31" ht="16.5" customHeight="1" s="48">
-      <c r="A31" s="58" t="inlineStr">
+      <c r="A31" s="94" t="inlineStr">
         <is>
           <t>Protectie</t>
         </is>
       </c>
-      <c r="B31" s="59" t="inlineStr">
-        <is>
-          <t>Antifoane</t>
-        </is>
-      </c>
-      <c r="C31" s="74" t="inlineStr">
-        <is>
-          <t>Esential</t>
-        </is>
-      </c>
-      <c r="D31" s="85" t="n"/>
-      <c r="E31" s="85" t="n"/>
-      <c r="F31" s="85" t="n"/>
-      <c r="G31" s="85" t="n"/>
-      <c r="H31" s="59" t="inlineStr">
-        <is>
-          <t>La circular/pendular</t>
-        </is>
-      </c>
+      <c r="B31" s="83" t="n"/>
+      <c r="C31" s="83" t="n"/>
+      <c r="D31" s="83" t="n"/>
+      <c r="E31" s="83" t="n"/>
+      <c r="F31" s="83" t="n"/>
+      <c r="G31" s="83" t="n"/>
+      <c r="H31" s="84" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1" s="48">
-      <c r="A32" s="58" t="inlineStr">
+      <c r="A32" s="94" t="inlineStr">
         <is>
           <t>Protectie</t>
         </is>
       </c>
-      <c r="B32" s="59" t="inlineStr">
+      <c r="B32" s="95" t="inlineStr">
         <is>
           <t>Masca de praf</t>
         </is>
@@ -5870,11 +5904,11 @@
           <t>Util</t>
         </is>
       </c>
-      <c r="D32" s="85" t="n"/>
-      <c r="E32" s="85" t="n"/>
-      <c r="F32" s="85" t="n"/>
-      <c r="G32" s="85" t="n"/>
-      <c r="H32" s="59" t="inlineStr">
+      <c r="D32" s="97" t="n"/>
+      <c r="E32" s="97" t="n"/>
+      <c r="F32" s="97" t="n"/>
+      <c r="G32" s="97" t="n"/>
+      <c r="H32" s="95" t="inlineStr">
         <is>
           <t>La taiat / slefuit</t>
         </is>
@@ -5895,12 +5929,12 @@
       <c r="H33" s="84" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="48">
-      <c r="A34" s="58" t="inlineStr">
+      <c r="A34" s="94" t="inlineStr">
         <is>
           <t>Finisaj</t>
         </is>
       </c>
-      <c r="B34" s="59" t="inlineStr">
+      <c r="B34" s="95" t="inlineStr">
         <is>
           <t>Pensula + trafalet</t>
         </is>
@@ -5910,65 +5944,56 @@
           <t>la finisaj</t>
         </is>
       </c>
-      <c r="D34" s="85" t="n"/>
-      <c r="E34" s="85" t="n"/>
-      <c r="F34" s="85" t="n"/>
-      <c r="G34" s="85" t="n"/>
-      <c r="H34" s="59" t="inlineStr">
+      <c r="D34" s="97" t="n"/>
+      <c r="E34" s="97" t="n"/>
+      <c r="F34" s="97" t="n"/>
+      <c r="G34" s="97" t="n"/>
+      <c r="H34" s="95" t="inlineStr">
         <is>
           <t>Ulei pe larice + protectie structura</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="58" t="inlineStr">
+      <c r="A35" s="94" t="inlineStr">
         <is>
           <t>Diverse</t>
         </is>
       </c>
-      <c r="B35" s="59" t="inlineStr">
+      <c r="B35" s="95" t="inlineStr">
         <is>
           <t>Distantier 5 mm (un cui)</t>
         </is>
       </c>
-      <c r="C35" s="63" t="inlineStr">
+      <c r="C35" s="96" t="inlineStr">
         <is>
           <t>gratis</t>
         </is>
       </c>
-      <c r="D35" s="85" t="n"/>
-      <c r="E35" s="85" t="n"/>
-      <c r="F35" s="85" t="n"/>
-      <c r="G35" s="85" t="n"/>
-      <c r="H35" s="59" t="inlineStr">
+      <c r="D35" s="97" t="n"/>
+      <c r="E35" s="97" t="n"/>
+      <c r="F35" s="97" t="n"/>
+      <c r="G35" s="97" t="n"/>
+      <c r="H35" s="95" t="inlineStr">
         <is>
           <t>Golul egal intre scandurile de dusumea</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="48">
-      <c r="A36" s="58" t="inlineStr">
+      <c r="A36" s="94" t="inlineStr">
         <is>
           <t>Diverse</t>
         </is>
       </c>
-      <c r="B36" s="59" t="inlineStr">
-        <is>
-          <t>Galeata, carpe, perie</t>
-        </is>
-      </c>
-      <c r="C36" s="72" t="inlineStr">
-        <is>
-          <t>Util</t>
-        </is>
-      </c>
-      <c r="D36" s="85" t="n"/>
-      <c r="E36" s="85" t="n"/>
-      <c r="F36" s="85" t="n"/>
-      <c r="G36" s="85" t="n"/>
-      <c r="H36" s="59" t="n"/>
-    </row>
-    <row r="37"/>
+      <c r="B36" s="83" t="n"/>
+      <c r="C36" s="83" t="n"/>
+      <c r="D36" s="83" t="n"/>
+      <c r="E36" s="83" t="n"/>
+      <c r="F36" s="83" t="n"/>
+      <c r="G36" s="83" t="n"/>
+      <c r="H36" s="84" t="n"/>
+    </row>
     <row r="38">
       <c r="A38" s="80" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Grund = Köber 4L (detinut): scos lazura Hornbach din cos, tracker + catalog + PDF sincronizate
</commit_message>
<xml_diff>
--- a/Tracker_materiale_casuta.xlsx
+++ b/Tracker_materiale_casuta.xlsx
@@ -1916,26 +1916,22 @@
       </c>
       <c r="B29" s="95" t="inlineStr">
         <is>
-          <t>Lazura impregnare (grund structura)</t>
+          <t>Grund impregnare lemn (AVEM)</t>
         </is>
       </c>
       <c r="C29" s="94" t="inlineStr">
         <is>
-          <t>Hornbach exterior 2,5 l</t>
+          <t>Köber pe baza de apa 4 L</t>
         </is>
       </c>
       <c r="D29" s="94" t="inlineStr">
         <is>
-          <t>Hornbach</t>
-        </is>
-      </c>
-      <c r="E29" s="94" t="inlineStr">
-        <is>
-          <t>12469765</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E29" s="94" t="n"/>
       <c r="F29" s="60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G29" s="94" t="inlineStr">
         <is>
@@ -1943,7 +1939,7 @@
         </is>
       </c>
       <c r="H29" s="61" t="n">
-        <v>92.5</v>
+        <v>0</v>
       </c>
       <c r="I29" s="62">
         <f>IF(AND(F29&lt;&gt;"",H29&lt;&gt;""),F29*H29,"")</f>
@@ -1951,13 +1947,13 @@
       </c>
       <c r="J29" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>Cumparat</t>
         </is>
       </c>
       <c r="K29" s="95" t="n"/>
       <c r="L29" s="95" t="inlineStr">
         <is>
-          <t>Strat de baza structura</t>
+          <t>Il avem deja; inlocuieste lazura Hornbach. Strat de baza structura.</t>
         </is>
       </c>
     </row>
@@ -4372,7 +4368,7 @@
       </c>
       <c r="B30" s="95" t="inlineStr">
         <is>
-          <t>Lazura impregnare exterior 2,5 l (grund)</t>
+          <t>Grund impregnare Köber 4 L (AVEM)</t>
         </is>
       </c>
       <c r="C30" s="94" t="inlineStr">
@@ -4381,10 +4377,10 @@
         </is>
       </c>
       <c r="D30" s="88" t="n">
-        <v>92.5</v>
+        <v>0</v>
       </c>
       <c r="E30" s="60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" s="94" t="inlineStr">
         <is>
@@ -4402,7 +4398,7 @@
       </c>
       <c r="I30" s="72" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>AVEM</t>
         </is>
       </c>
     </row>
@@ -4920,19 +4916,19 @@
     <row r="18" ht="15" customHeight="1" s="48">
       <c r="A18" s="95" t="inlineStr">
         <is>
-          <t>Lazura impregnare Hornbach exterior 2,5 l (grund)</t>
+          <t>Grund: AVEM Köber 4L — scos din cos (era lazura Hornbach)</t>
         </is>
       </c>
       <c r="B18" s="94" t="inlineStr">
         <is>
-          <t>12469765</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C18" s="88" t="n">
-        <v>92.5</v>
+        <v>0</v>
       </c>
       <c r="D18" s="60" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E18" s="62">
         <f>C18*D18</f>
@@ -4940,7 +4936,7 @@
       </c>
       <c r="F18" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>AVEM</t>
         </is>
       </c>
       <c r="G18" s="94" t="inlineStr">

</xml_diff>

<commit_message>
B1 polita: tija M12 + piulite in cos (cod 12130958, 3830642); tracker + catalog + PDF sincronizate, 18/21 acoperite
</commit_message>
<xml_diff>
--- a/Tracker_materiale_casuta.xlsx
+++ b/Tracker_materiale_casuta.xlsx
@@ -1813,12 +1813,12 @@
       </c>
       <c r="B27" s="95" t="inlineStr">
         <is>
-          <t>Buloane M12 (baza + polita) + saibe</t>
+          <t>Buloane M12: baza papuc + tija polita + piulite</t>
         </is>
       </c>
       <c r="C27" s="94" t="inlineStr">
         <is>
-          <t>8x M12x120 baza + 4x M12 lung polita</t>
+          <t>M12x120 (8) baza + tija M12 (4x~220) polita</t>
         </is>
       </c>
       <c r="D27" s="94" t="inlineStr">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="E27" s="94" t="inlineStr">
         <is>
-          <t>6834285 + set polita</t>
+          <t>6834285 / 12130958 / 3830642</t>
         </is>
       </c>
       <c r="F27" s="60" t="n">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="H27" s="61" t="n"/>
       <c r="I27" s="62" t="n">
-        <v>231.99</v>
+        <v>239.39</v>
       </c>
       <c r="J27" s="74" t="inlineStr">
         <is>
@@ -1851,7 +1851,7 @@
       <c r="K27" s="95" t="n"/>
       <c r="L27" s="95" t="inlineStr">
         <is>
-          <t>Baza papuc + polita grinda spate (vezi Comanda Hornbach)</t>
+          <t>Baza papuc (B2) + polita din tija taiata (B1) + piulite (B4) + saibe (B3). Toate in cos.</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="C34" s="95" t="inlineStr">
         <is>
-          <t>M12: 8x120 + 4x~200</t>
+          <t>M12: 8x120 baza + tija M12 polita</t>
         </is>
       </c>
       <c r="D34" s="97" t="inlineStr">
@@ -3086,7 +3086,7 @@
       </c>
       <c r="H34" s="95" t="inlineStr">
         <is>
-          <t>4x polita (lung ~200) + 8x baza papuc (M12x120). Traseu principal de greutate.</t>
+          <t>Baza papuc: 8x M12x120. Polita: tija filetata M12 1m taiata in 4x ~220 mm (cod 12130958) + piulite + saibe.</t>
         </is>
       </c>
     </row>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="H8" s="95" t="inlineStr">
         <is>
-          <t>4× polita grinda spate + 8× baza stalpi (2/papuc)</t>
+          <t>4x polita grinda spate (din tija M12 taiata) + 8x baza stalpi (2/papuc); piulite + saibe</t>
         </is>
       </c>
       <c r="I8" s="74" t="inlineStr">
@@ -4475,7 +4475,7 @@
     <row r="2" ht="15" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>13 produse in cos. Coloana 'Cod piesa' leaga fiecare linie de catalogul de piese. + livrare 215 lei.</t>
+          <t>14 produse in cos. Coloana 'Cod piesa' leaga fiecare linie de catalogul de piese. + livrare 215 lei.</t>
         </is>
       </c>
     </row>
@@ -4961,16 +4961,16 @@
     <row r="20" ht="15" customHeight="1" s="48">
       <c r="A20" s="95" t="inlineStr">
         <is>
-          <t>Bulon M12 POLITA lung ~200 (set cu piulita, 25 buc)</t>
+          <t>Tija filetata M12 1m DIN975 8.8 (se taie 4x ~220 pt polita)</t>
         </is>
       </c>
       <c r="B20" s="94" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12130958</t>
         </is>
       </c>
       <c r="C20" s="88" t="n">
-        <v>45</v>
+        <v>13.4</v>
       </c>
       <c r="D20" s="60" t="n">
         <v>1</v>
@@ -4981,7 +4981,7 @@
       </c>
       <c r="F20" s="96" t="inlineStr">
         <is>
-          <t>de confirmat</t>
+          <t>IN COS</t>
         </is>
       </c>
       <c r="G20" s="94" t="inlineStr">
@@ -4993,16 +4993,16 @@
     <row r="21" ht="15" customHeight="1" s="48">
       <c r="A21" s="95" t="inlineStr">
         <is>
-          <t>Piulite M12 — din raft la magazin</t>
+          <t>Piulite hexagonale M12 DIN934 zincat (100 buc)</t>
         </is>
       </c>
       <c r="B21" s="94" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3830642</t>
         </is>
       </c>
       <c r="C21" s="88" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D21" s="60" t="n">
         <v>1</v>
@@ -5013,7 +5013,7 @@
       </c>
       <c r="F21" s="96" t="inlineStr">
         <is>
-          <t>de confirmat</t>
+          <t>IN COS</t>
         </is>
       </c>
       <c r="G21" s="94" t="inlineStr">
@@ -5225,7 +5225,7 @@
     <row r="32" ht="15" customHeight="1" s="48">
       <c r="A32" s="80" t="inlineStr">
         <is>
-          <t>NOTA: Coloana 'Cod piesa' = legenda din catalogul de piese (catalog-piese.html). B1 = bulon M12 LUNG (~200) pt polita — masori grosimea reala inainte de comanda. B2 = M12×120 pt baza papuc (deja in cos). Piulitele M12 (B4) se iau din raft la magazin. Topcoatul colorat (F3) il alegi tu.</t>
+          <t>NOTA: B1 = tija filetata M12 (12130958) taiata in 4 bucati de ~220 mm pt polita; B4 = piulite M12 (3830642). Saibele = B3 (3840897, in cos). B2 = M12x120 baza papuc. Topcoatul (F3) si scara (Faza 2) raman de decis.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Comanda Faza 1 plasata 09.06.2026 (4101,24 lei): status COMANDAT in tracker + catalog + imbinari + PDF, plata inregistrata
</commit_message>
<xml_diff>
--- a/Tracker_materiale_casuta.xlsx
+++ b/Tracker_materiale_casuta.xlsx
@@ -893,7 +893,7 @@
     <row r="4" ht="15" customHeight="1" s="48">
       <c r="A4" s="51" t="inlineStr">
         <is>
-          <t>Cheltuit — cumparat</t>
+          <t>Cheltuit — cumparat (incl. comanda Faza 1 din 09.06.2026)</t>
         </is>
       </c>
       <c r="C4" s="53">
@@ -1213,13 +1213,13 @@
       </c>
       <c r="J14" s="73" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>Cumparat</t>
         </is>
       </c>
       <c r="K14" s="66" t="n"/>
       <c r="L14" s="66" t="inlineStr">
         <is>
-          <t>2 grinzi; fata pe varful stalpului, spate pe polita + 2x M12</t>
+          <t>2 grinzi; fata pe varful stalpului, spate pe polita + 2x M12 · comanda 09.06.2026</t>
         </is>
       </c>
     </row>
@@ -1266,13 +1266,13 @@
       </c>
       <c r="J15" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>Cumparat</t>
         </is>
       </c>
       <c r="K15" s="95" t="n"/>
       <c r="L15" s="95" t="inlineStr">
         <is>
-          <t>Inca 2 (la cele 4 Leroy) = 6 joiste, fata-spate</t>
+          <t>Inca 2 (la cele 4 Leroy) = 6 joiste, fata-spate · comanda 09.06.2026</t>
         </is>
       </c>
     </row>
@@ -1319,13 +1319,13 @@
       </c>
       <c r="J16" s="73" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>Cumparat</t>
         </is>
       </c>
       <c r="K16" s="66" t="n"/>
       <c r="L16" s="66" t="inlineStr">
         <is>
-          <t>Podea casuta + balcon</t>
+          <t>Podea casuta + balcon · comanda 09.06.2026</t>
         </is>
       </c>
     </row>
@@ -1692,13 +1692,13 @@
       </c>
       <c r="J24" s="73" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>Cumparat</t>
         </is>
       </c>
       <c r="K24" s="66" t="n"/>
       <c r="L24" s="66" t="inlineStr">
         <is>
-          <t>Imbinari grinzi/stalpi/contrafise/blocaje</t>
+          <t>Imbinari grinzi/stalpi/contrafise/blocaje · comanda 09.06.2026</t>
         </is>
       </c>
     </row>
@@ -1745,13 +1745,13 @@
       </c>
       <c r="J25" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>Cumparat</t>
         </is>
       </c>
       <c r="K25" s="95" t="n"/>
       <c r="L25" s="95" t="inlineStr">
         <is>
-          <t>Prindere larice (~204 buc)</t>
+          <t>Prindere larice (~204 buc) · comanda 09.06.2026</t>
         </is>
       </c>
     </row>
@@ -1795,13 +1795,13 @@
       </c>
       <c r="J26" s="73" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>Cumparat</t>
         </is>
       </c>
       <c r="K26" s="66" t="n"/>
       <c r="L26" s="66" t="inlineStr">
         <is>
-          <t>C1 grinda fata-&gt;stalp (4); C2 anti-ridicare joiste (12)</t>
+          <t>C1 grinda fata-&gt;stalp (4); C2 anti-ridicare joiste (12) · comanda 09.06.2026</t>
         </is>
       </c>
     </row>
@@ -1845,13 +1845,13 @@
       </c>
       <c r="J27" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>Cumparat</t>
         </is>
       </c>
       <c r="K27" s="95" t="n"/>
       <c r="L27" s="95" t="inlineStr">
         <is>
-          <t>Baza papuc (B2) + polita din tija taiata (B1) + piulite (B4) + saibe (B3). Toate in cos.</t>
+          <t>Baza papuc (B2) + polita din tija taiata (B1) + piulite (B4) + saibe (B3). Toate in cos. · comanda 09.06.2026</t>
         </is>
       </c>
     </row>
@@ -1898,13 +1898,13 @@
       </c>
       <c r="J28" s="73" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>Cumparat</t>
         </is>
       </c>
       <c r="K28" s="66" t="n"/>
       <c r="L28" s="66" t="inlineStr">
         <is>
-          <t>Finisaj larice + lemn expus</t>
+          <t>Finisaj larice + lemn expus · comanda 09.06.2026</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
     <row r="2" ht="15" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Sursa: HORNBACH (preferinta 1) + papuc/joiste Leroy. Grinzi glulam · suruburi Heco · grinda spate pe POLITA + M12 · baza pe papuc U · scara inclusa.</t>
+          <t>Sursa: HORNBACH (preferinta 1) + papuc/joiste Leroy. Grinzi glulam · suruburi Heco · grinda spate pe POLITA + M12 · baza pe papuc U · scara inclusa.  ·  COMANDA platforma plasata 09.06.2026 (4101,24 lei cu livrare).</t>
         </is>
       </c>
     </row>
@@ -4475,7 +4475,7 @@
     <row r="2" ht="15" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>14 produse in cos. Coloana 'Cod piesa' leaga fiecare linie de catalogul de piese. + livrare 215 lei.</t>
+          <t>COMANDA PLASATA 09.06.2026 · 14 produse · subtotal 3886,24 + livrare 215 = 4101,24 lei. Coloana 'Cod piesa' leaga de catalogul de piese.</t>
         </is>
       </c>
     </row>
@@ -4519,7 +4519,7 @@
     <row r="5" ht="16.5" customHeight="1" s="48">
       <c r="A5" s="82" t="inlineStr">
         <is>
-          <t>IN COS — adaugate</t>
+          <t>COMANDAT (09.06.2026)</t>
         </is>
       </c>
       <c r="B5" s="83" t="n"/>
@@ -4552,7 +4552,7 @@
       </c>
       <c r="F6" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G6" s="94" t="inlineStr">
@@ -4584,7 +4584,7 @@
       </c>
       <c r="F7" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G7" s="94" t="inlineStr">
@@ -4616,7 +4616,7 @@
       </c>
       <c r="F8" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G8" s="94" t="inlineStr">
@@ -4648,7 +4648,7 @@
       </c>
       <c r="F9" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G9" s="94" t="inlineStr">
@@ -4680,7 +4680,7 @@
       </c>
       <c r="F10" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G10" s="94" t="inlineStr">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="F11" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G11" s="94" t="inlineStr">
@@ -4744,7 +4744,7 @@
       </c>
       <c r="F12" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G12" s="94" t="inlineStr">
@@ -4776,7 +4776,7 @@
       </c>
       <c r="F13" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G13" s="94" t="inlineStr">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="F14" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G14" s="94" t="inlineStr">
@@ -4840,7 +4840,7 @@
       </c>
       <c r="F15" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G15" s="94" t="inlineStr">
@@ -4872,7 +4872,7 @@
       </c>
       <c r="F16" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G16" s="94" t="inlineStr">
@@ -4904,7 +4904,7 @@
       </c>
       <c r="F17" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G17" s="94" t="inlineStr">
@@ -4981,7 +4981,7 @@
       </c>
       <c r="F20" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G20" s="94" t="inlineStr">
@@ -5013,7 +5013,7 @@
       </c>
       <c r="F21" s="96" t="inlineStr">
         <is>
-          <t>IN COS</t>
+          <t>COMANDAT</t>
         </is>
       </c>
       <c r="G21" s="94" t="inlineStr">
@@ -5189,11 +5189,11 @@
     <row r="28" ht="15" customHeight="1" s="48">
       <c r="D28" s="92" t="inlineStr">
         <is>
-          <t>in cos:</t>
+          <t>comandat:</t>
         </is>
       </c>
       <c r="E28" s="93">
-        <f>SUMIF(F6:F26,"IN COS",E6:E26)</f>
+        <f>SUMIF(F6:F26,"COMANDAT",E6:E26)</f>
         <v/>
       </c>
     </row>
@@ -5221,6 +5221,15 @@
     </row>
     <row r="31" ht="15" customHeight="1" s="48">
       <c r="A31" s="80" t="n"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TOTAL PLATIT:</t>
+        </is>
+      </c>
+      <c r="E31">
+        <f>E28+E29</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="48">
       <c r="A32" s="80" t="inlineStr">

</xml_diff>

<commit_message>
Audit fixes F2/F4/F6/F7/F8/F10: stalpisor 58x58, corcodus +2780 de la sol, README structura, tracker 10 trepte, cod mort in _arhiva; regenerat fise HTML + toate PDF-urile; PROJ derivat din __file__
F1 (granita faza) si F3 (surub C1) raman pending aprobarea Vlad — vezi NEEDS-INPUT-audit-fixes.md.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tracker_materiale_casuta.xlsx
+++ b/Tracker_materiale_casuta.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materiale" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debitare" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platforma premium" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comanda Hornbach" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scule" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Materiale" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Debitare" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Platforma premium" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Comanda Hornbach" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Scule" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="H24" s="95" t="inlineStr">
         <is>
-          <t>11 trepte (riser 200, calcai 190)</t>
+          <t>10 trepte (11 niveluri) (riser 200, calcai 190)</t>
         </is>
       </c>
       <c r="I24" s="72" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="35" ht="15" customHeight="1" s="48">
       <c r="A35" s="80" t="inlineStr">
         <is>
-          <t>Scara: 11 trepte, riser 200 / calcai 190, ~49°, latime 600, mana curenta pe ambele parti, poarta la S3 (opus mesei de pe S4). Preturi 'est.' = de confirmat la magazin.</t>
+          <t>Scara: 10 trepte (11 niveluri), riser 200 / calcai 190, ~49°, latime 600, mana curenta pe ambele parti, poarta la S3 (opus mesei de pe S4). Preturi 'est.' = de confirmat la magazin.</t>
         </is>
       </c>
     </row>
@@ -5221,12 +5221,12 @@
     </row>
     <row r="31" ht="15" customHeight="1" s="48">
       <c r="A31" s="80" t="n"/>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="47" t="inlineStr">
         <is>
           <t>TOTAL PLATIT:</t>
         </is>
       </c>
-      <c r="E31">
+      <c r="E31" s="47">
         <f>E28+E29</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Manual upgrade: book.py fitz->pypdf (fix Builder crash), C2=14/H4=3pac/M10 in tracker, ghid pas4 H1+C2, fix orfani pagina; regenerat fise+toate PDF-urile
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tracker_materiale_casuta.xlsx
+++ b/Tracker_materiale_casuta.xlsx
@@ -851,7 +851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="47" min="1" max="1"/>
@@ -1477,610 +1477,620 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="48">
-      <c r="A20" s="65" t="inlineStr">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Balustrada</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Buloane M10 (balustrada)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>M10×120 + piulita + saiba</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>12</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I20">
+        <f>IF(AND(F20&lt;&gt;"",H20&lt;&gt;""),F20*H20,"")</f>
+        <v/>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>De cumparat</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Faza 1; prinde stalpisorii 58x58 de cadru</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="48">
+      <c r="A21" s="65" t="inlineStr">
         <is>
           <t>Pereti</t>
         </is>
       </c>
-      <c r="B20" s="66" t="inlineStr">
+      <c r="B21" s="66" t="inlineStr">
         <is>
           <t>Scanduri pereti partiali</t>
         </is>
       </c>
-      <c r="C20" s="65" t="inlineStr">
+      <c r="C21" s="65" t="inlineStr">
         <is>
           <t>28x90 mm</t>
         </is>
       </c>
-      <c r="D20" s="65" t="n"/>
-      <c r="E20" s="65" t="n"/>
-      <c r="F20" s="67" t="n">
+      <c r="D21" s="65" t="n"/>
+      <c r="E21" s="65" t="n"/>
+      <c r="F21" s="67" t="n">
         <v>16</v>
       </c>
-      <c r="G20" s="65" t="inlineStr">
+      <c r="G21" s="65" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
       </c>
-      <c r="H20" s="68" t="n">
+      <c r="H21" s="68" t="n">
         <v>38</v>
       </c>
-      <c r="I20" s="69">
-        <f>IF(AND(F20&lt;&gt;"",H20&lt;&gt;""),F20*H20,"")</f>
-        <v/>
-      </c>
-      <c r="J20" s="73" t="inlineStr">
+      <c r="I21" s="69">
+        <f>IF(AND(F21&lt;&gt;"",H21&lt;&gt;""),F21*H21,"")</f>
+        <v/>
+      </c>
+      <c r="J21" s="73" t="inlineStr">
         <is>
           <t>De cumparat</t>
         </is>
       </c>
-      <c r="K20" s="66" t="n"/>
-      <c r="L20" s="66" t="inlineStr">
+      <c r="K21" s="66" t="n"/>
+      <c r="L21" s="66" t="inlineStr">
         <is>
           <t>Pereti pana la jumatate + ferestre</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="48">
-      <c r="A21" s="94" t="inlineStr">
+    <row r="22" ht="21.75" customHeight="1" s="48">
+      <c r="A22" s="94" t="inlineStr">
         <is>
           <t>Acoperis</t>
         </is>
       </c>
-      <c r="B21" s="95" t="inlineStr">
+      <c r="B22" s="95" t="inlineStr">
         <is>
           <t>Capriori acoperis</t>
         </is>
       </c>
-      <c r="C21" s="94" t="inlineStr">
+      <c r="C22" s="94" t="inlineStr">
         <is>
           <t>60x100 mm</t>
         </is>
       </c>
-      <c r="D21" s="94" t="n"/>
-      <c r="E21" s="94" t="n"/>
-      <c r="F21" s="60" t="n">
+      <c r="D22" s="94" t="n"/>
+      <c r="E22" s="94" t="n"/>
+      <c r="F22" s="60" t="n">
         <v>4</v>
       </c>
-      <c r="G21" s="94" t="inlineStr">
+      <c r="G22" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
       </c>
-      <c r="H21" s="61" t="n">
+      <c r="H22" s="61" t="n">
         <v>39</v>
       </c>
-      <c r="I21" s="62">
-        <f>IF(AND(F21&lt;&gt;"",H21&lt;&gt;""),F21*H21,"")</f>
-        <v/>
-      </c>
-      <c r="J21" s="74" t="inlineStr">
+      <c r="I22" s="62">
+        <f>IF(AND(F22&lt;&gt;"",H22&lt;&gt;""),F22*H22,"")</f>
+        <v/>
+      </c>
+      <c r="J22" s="74" t="inlineStr">
         <is>
           <t>De cumparat</t>
         </is>
       </c>
-      <c r="K21" s="95" t="n"/>
-      <c r="L21" s="95" t="inlineStr">
+      <c r="K22" s="95" t="n"/>
+      <c r="L22" s="95" t="inlineStr">
         <is>
           <t>Structura acoperis inclinat</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="21.75" customHeight="1" s="48">
-      <c r="A22" s="65" t="inlineStr">
+    <row r="23" ht="15" customHeight="1" s="48">
+      <c r="A23" s="65" t="inlineStr">
         <is>
           <t>Acoperis</t>
         </is>
       </c>
-      <c r="B22" s="66" t="inlineStr">
+      <c r="B23" s="66" t="inlineStr">
         <is>
           <t>Invelitoare (policarbonat/scandura)</t>
         </is>
       </c>
-      <c r="C22" s="65" t="inlineStr">
+      <c r="C23" s="65" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D22" s="65" t="n"/>
-      <c r="E22" s="65" t="n"/>
-      <c r="F22" s="67" t="n">
+      <c r="D23" s="65" t="n"/>
+      <c r="E23" s="65" t="n"/>
+      <c r="F23" s="67" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="65" t="inlineStr">
+      <c r="G23" s="65" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="H22" s="68" t="n"/>
-      <c r="I22" s="69">
-        <f>IF(AND(F22&lt;&gt;"",H22&lt;&gt;""),F22*H22,"")</f>
-        <v/>
-      </c>
-      <c r="J22" s="75" t="inlineStr">
+      <c r="H23" s="68" t="n"/>
+      <c r="I23" s="69">
+        <f>IF(AND(F23&lt;&gt;"",H23&lt;&gt;""),F23*H23,"")</f>
+        <v/>
+      </c>
+      <c r="J23" s="75" t="inlineStr">
         <is>
           <t>De decis</t>
         </is>
       </c>
-      <c r="K22" s="66" t="n"/>
-      <c r="L22" s="66" t="inlineStr">
+      <c r="K23" s="66" t="n"/>
+      <c r="L23" s="66" t="inlineStr">
         <is>
           <t>Policarbonat ondulat sau sindrila bituminoasa</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="48">
-      <c r="A23" s="94" t="inlineStr">
+    <row r="24" ht="15" customHeight="1" s="48">
+      <c r="A24" s="94" t="inlineStr">
         <is>
           <t>Scara</t>
         </is>
       </c>
-      <c r="B23" s="95" t="inlineStr">
+      <c r="B24" s="95" t="inlineStr">
         <is>
           <t>Scara fixa + balustrada</t>
         </is>
       </c>
-      <c r="C23" s="94" t="inlineStr">
+      <c r="C24" s="94" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D23" s="94" t="n"/>
-      <c r="E23" s="94" t="n"/>
-      <c r="F23" s="60" t="n">
+      <c r="D24" s="94" t="n"/>
+      <c r="E24" s="94" t="n"/>
+      <c r="F24" s="60" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="94" t="inlineStr">
+      <c r="G24" s="94" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="H23" s="61" t="n"/>
-      <c r="I23" s="62">
-        <f>IF(AND(F23&lt;&gt;"",H23&lt;&gt;""),F23*H23,"")</f>
-        <v/>
-      </c>
-      <c r="J23" s="74" t="inlineStr">
+      <c r="H24" s="61" t="n"/>
+      <c r="I24" s="62">
+        <f>IF(AND(F24&lt;&gt;"",H24&lt;&gt;""),F24*H24,"")</f>
+        <v/>
+      </c>
+      <c r="J24" s="74" t="inlineStr">
         <is>
           <t>De cumparat</t>
         </is>
       </c>
-      <c r="K23" s="95" t="n"/>
-      <c r="L23" s="95" t="inlineStr">
+      <c r="K24" s="95" t="n"/>
+      <c r="L24" s="95" t="inlineStr">
         <is>
           <t>Cu balustrada, NU franghie</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="48">
-      <c r="A24" s="65" t="inlineStr">
+    <row r="25" ht="15" customHeight="1" s="48">
+      <c r="A25" s="65" t="inlineStr">
         <is>
           <t>Feronerie</t>
         </is>
       </c>
-      <c r="B24" s="66" t="inlineStr">
+      <c r="B25" s="66" t="inlineStr">
         <is>
           <t>Suruburi structurale Heco (set)</t>
         </is>
       </c>
-      <c r="C24" s="65" t="inlineStr">
+      <c r="C25" s="65" t="inlineStr">
         <is>
           <t>8x200 + 6x100 + 6x80, 3 pac</t>
         </is>
       </c>
-      <c r="D24" s="65" t="inlineStr">
+      <c r="D25" s="65" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="E24" s="65" t="inlineStr">
+      <c r="E25" s="65" t="inlineStr">
         <is>
           <t>10434633/398/139</t>
         </is>
       </c>
-      <c r="F24" s="67" t="n">
+      <c r="F25" s="67" t="n">
         <v>3</v>
       </c>
-      <c r="G24" s="65" t="inlineStr">
+      <c r="G25" s="65" t="inlineStr">
         <is>
           <t>pac</t>
         </is>
       </c>
-      <c r="H24" s="68" t="n"/>
-      <c r="I24" s="69" t="n">
+      <c r="H25" s="68" t="n"/>
+      <c r="I25" s="69" t="n">
         <v>536.77</v>
       </c>
-      <c r="J24" s="73" t="inlineStr">
+      <c r="J25" s="73" t="inlineStr">
         <is>
           <t>Cumparat</t>
         </is>
       </c>
-      <c r="K24" s="66" t="n"/>
-      <c r="L24" s="66" t="inlineStr">
+      <c r="K25" s="66" t="n"/>
+      <c r="L25" s="66" t="inlineStr">
         <is>
           <t>Imbinari grinzi/stalpi/contrafise/blocaje · comanda 09.06.2026</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="48">
-      <c r="A25" s="94" t="inlineStr">
+    <row r="26" ht="15" customHeight="1" s="48">
+      <c r="A26" s="94" t="inlineStr">
         <is>
           <t>Feronerie</t>
         </is>
       </c>
-      <c r="B25" s="95" t="inlineStr">
+      <c r="B26" s="95" t="inlineStr">
         <is>
           <t>Suruburi dusumea inox</t>
         </is>
       </c>
-      <c r="C25" s="94" t="inlineStr">
-        <is>
-          <t>A2 5x60, 2 pac (100)</t>
-        </is>
-      </c>
-      <c r="D25" s="94" t="inlineStr">
+      <c r="C26" s="94" t="inlineStr">
+        <is>
+          <t>A2 5x60, 3 pac (300)</t>
+        </is>
+      </c>
+      <c r="D26" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="E25" s="94" t="inlineStr">
+      <c r="E26" s="94" t="inlineStr">
         <is>
           <t>10528829</t>
         </is>
       </c>
-      <c r="F25" s="60" t="n">
+      <c r="F26" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="94" t="inlineStr">
+        <is>
+          <t>pac</t>
+        </is>
+      </c>
+      <c r="H26" s="61" t="n">
+        <v>55.82</v>
+      </c>
+      <c r="I26" s="62">
+        <f>IF(AND(F26&lt;&gt;"",H26&lt;&gt;""),F26*H26,"")</f>
+        <v/>
+      </c>
+      <c r="J26" s="74" t="inlineStr">
+        <is>
+          <t>Cumparat</t>
+        </is>
+      </c>
+      <c r="K26" s="95" t="n"/>
+      <c r="L26" s="95" t="inlineStr">
+        <is>
+          <t>Prindere larice (~204 buc necesare, 3 pachete) · comanda 09.06.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1" s="48">
+      <c r="A27" s="65" t="inlineStr">
+        <is>
+          <t>Feronerie</t>
+        </is>
+      </c>
+      <c r="B27" s="66" t="inlineStr">
+        <is>
+          <t>Coltare imbinare C1 + C2</t>
+        </is>
+      </c>
+      <c r="C27" s="65" t="inlineStr">
+        <is>
+          <t>4x 100x100x90 + 14x 90x90x65</t>
+        </is>
+      </c>
+      <c r="D27" s="65" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="E27" s="65" t="inlineStr">
+        <is>
+          <t>738965 / 738910</t>
+        </is>
+      </c>
+      <c r="F27" s="67" t="n">
+        <v>18</v>
+      </c>
+      <c r="G27" s="65" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="H27" s="68" t="n"/>
+      <c r="I27" s="69" t="n">
+        <v>95.36</v>
+      </c>
+      <c r="J27" s="73" t="inlineStr">
+        <is>
+          <t>Cumparat</t>
+        </is>
+      </c>
+      <c r="K27" s="66" t="n"/>
+      <c r="L27" s="66" t="inlineStr">
+        <is>
+          <t>C1 grinda fata-&gt;stalp (4); C2 anti-ridicare (12 joiste + 2 grinda spate = 14) · comanda 09.06.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="48">
+      <c r="A28" s="94" t="inlineStr">
+        <is>
+          <t>Feronerie</t>
+        </is>
+      </c>
+      <c r="B28" s="95" t="inlineStr">
+        <is>
+          <t>Buloane M12: baza papuc + tija polita + piulite</t>
+        </is>
+      </c>
+      <c r="C28" s="94" t="inlineStr">
+        <is>
+          <t>M12x120 (8) baza + tija M12 (4x~220) polita</t>
+        </is>
+      </c>
+      <c r="D28" s="94" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="E28" s="94" t="inlineStr">
+        <is>
+          <t>6834285 / 12130958 / 3830642</t>
+        </is>
+      </c>
+      <c r="F28" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="94" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="H28" s="61" t="n"/>
+      <c r="I28" s="62" t="n">
+        <v>239.39</v>
+      </c>
+      <c r="J28" s="74" t="inlineStr">
+        <is>
+          <t>Cumparat</t>
+        </is>
+      </c>
+      <c r="K28" s="95" t="n"/>
+      <c r="L28" s="95" t="inlineStr">
+        <is>
+          <t>Baza papuc (B2) + polita din tija taiata (B1) + piulite (B4) + saibe (B3). Toate in cos. · comanda 09.06.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1" s="48">
+      <c r="A29" s="65" t="inlineStr">
+        <is>
+          <t>Finisaj</t>
+        </is>
+      </c>
+      <c r="B29" s="66" t="inlineStr">
+        <is>
+          <t>Ulei lemn tec (dusumea larice)</t>
+        </is>
+      </c>
+      <c r="C29" s="65" t="inlineStr">
+        <is>
+          <t>Hornbach Plus 2,5 l</t>
+        </is>
+      </c>
+      <c r="D29" s="65" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="E29" s="65" t="inlineStr">
+        <is>
+          <t>5509678</t>
+        </is>
+      </c>
+      <c r="F29" s="67" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="94" t="inlineStr">
-        <is>
-          <t>pac</t>
-        </is>
-      </c>
-      <c r="H25" s="61" t="n">
-        <v>55.82</v>
-      </c>
-      <c r="I25" s="62">
-        <f>IF(AND(F25&lt;&gt;"",H25&lt;&gt;""),F25*H25,"")</f>
-        <v/>
-      </c>
-      <c r="J25" s="74" t="inlineStr">
+      <c r="G29" s="65" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="H29" s="68" t="n">
+        <v>144.39</v>
+      </c>
+      <c r="I29" s="69">
+        <f>IF(AND(F29&lt;&gt;"",H29&lt;&gt;""),F29*H29,"")</f>
+        <v/>
+      </c>
+      <c r="J29" s="73" t="inlineStr">
         <is>
           <t>Cumparat</t>
         </is>
       </c>
-      <c r="K25" s="95" t="n"/>
-      <c r="L25" s="95" t="inlineStr">
-        <is>
-          <t>Prindere larice (~204 buc) · comanda 09.06.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="48">
-      <c r="A26" s="65" t="inlineStr">
-        <is>
-          <t>Feronerie</t>
-        </is>
-      </c>
-      <c r="B26" s="66" t="inlineStr">
-        <is>
-          <t>Coltare imbinare C1 + C2</t>
-        </is>
-      </c>
-      <c r="C26" s="65" t="inlineStr">
-        <is>
-          <t>4x 100x100x90 + 12x 90x90x65</t>
-        </is>
-      </c>
-      <c r="D26" s="65" t="inlineStr">
-        <is>
-          <t>Hornbach</t>
-        </is>
-      </c>
-      <c r="E26" s="65" t="inlineStr">
-        <is>
-          <t>738965 / 738910</t>
-        </is>
-      </c>
-      <c r="F26" s="67" t="n">
-        <v>16</v>
-      </c>
-      <c r="G26" s="65" t="inlineStr">
+      <c r="K29" s="66" t="n"/>
+      <c r="L29" s="66" t="inlineStr">
+        <is>
+          <t>Finisaj larice + lemn expus · comanda 09.06.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="48">
+      <c r="A30" s="94" t="inlineStr">
+        <is>
+          <t>Finisaj</t>
+        </is>
+      </c>
+      <c r="B30" s="95" t="inlineStr">
+        <is>
+          <t>Grund impregnare lemn (AVEM)</t>
+        </is>
+      </c>
+      <c r="C30" s="94" t="inlineStr">
+        <is>
+          <t>Köber pe baza de apa 4 L</t>
+        </is>
+      </c>
+      <c r="D30" s="94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E30" s="94" t="n"/>
+      <c r="F30" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
       </c>
-      <c r="H26" s="68" t="n"/>
-      <c r="I26" s="69" t="n">
-        <v>95.36</v>
-      </c>
-      <c r="J26" s="73" t="inlineStr">
+      <c r="H30" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="62">
+        <f>IF(AND(F30&lt;&gt;"",H30&lt;&gt;""),F30*H30,"")</f>
+        <v/>
+      </c>
+      <c r="J30" s="74" t="inlineStr">
         <is>
           <t>Cumparat</t>
         </is>
       </c>
-      <c r="K26" s="66" t="n"/>
-      <c r="L26" s="66" t="inlineStr">
-        <is>
-          <t>C1 grinda fata-&gt;stalp (4); C2 anti-ridicare joiste (12) · comanda 09.06.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="48">
-      <c r="A27" s="94" t="inlineStr">
-        <is>
-          <t>Feronerie</t>
-        </is>
-      </c>
-      <c r="B27" s="95" t="inlineStr">
-        <is>
-          <t>Buloane M12: baza papuc + tija polita + piulite</t>
-        </is>
-      </c>
-      <c r="C27" s="94" t="inlineStr">
-        <is>
-          <t>M12x120 (8) baza + tija M12 (4x~220) polita</t>
-        </is>
-      </c>
-      <c r="D27" s="94" t="inlineStr">
-        <is>
-          <t>Hornbach</t>
-        </is>
-      </c>
-      <c r="E27" s="94" t="inlineStr">
-        <is>
-          <t>6834285 / 12130958 / 3830642</t>
-        </is>
-      </c>
-      <c r="F27" s="60" t="n">
+      <c r="K30" s="95" t="n"/>
+      <c r="L30" s="95" t="inlineStr">
+        <is>
+          <t>Il avem deja; inlocuieste lazura Hornbach. Strat de baza structura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="48">
+      <c r="A31" s="65" t="inlineStr">
+        <is>
+          <t>Siguranta</t>
+        </is>
+      </c>
+      <c r="B31" s="66" t="inlineStr">
+        <is>
+          <t>Material sol moale</t>
+        </is>
+      </c>
+      <c r="C31" s="65" t="inlineStr">
+        <is>
+          <t>scoarta/nisip</t>
+        </is>
+      </c>
+      <c r="D31" s="65" t="n"/>
+      <c r="E31" s="65" t="n"/>
+      <c r="F31" s="67" t="n">
         <v>1</v>
       </c>
-      <c r="G27" s="94" t="inlineStr">
-        <is>
-          <t>set</t>
-        </is>
-      </c>
-      <c r="H27" s="61" t="n"/>
-      <c r="I27" s="62" t="n">
-        <v>239.39</v>
-      </c>
-      <c r="J27" s="74" t="inlineStr">
-        <is>
-          <t>Cumparat</t>
-        </is>
-      </c>
-      <c r="K27" s="95" t="n"/>
-      <c r="L27" s="95" t="inlineStr">
-        <is>
-          <t>Baza papuc (B2) + polita din tija taiata (B1) + piulite (B4) + saibe (B3). Toate in cos. · comanda 09.06.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1" s="48">
-      <c r="A28" s="65" t="inlineStr">
-        <is>
-          <t>Finisaj</t>
-        </is>
-      </c>
-      <c r="B28" s="66" t="inlineStr">
-        <is>
-          <t>Ulei lemn tec (dusumea larice)</t>
-        </is>
-      </c>
-      <c r="C28" s="65" t="inlineStr">
-        <is>
-          <t>Hornbach Plus 2,5 l</t>
-        </is>
-      </c>
-      <c r="D28" s="65" t="inlineStr">
-        <is>
-          <t>Hornbach</t>
-        </is>
-      </c>
-      <c r="E28" s="65" t="inlineStr">
-        <is>
-          <t>5509678</t>
-        </is>
-      </c>
-      <c r="F28" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="G28" s="65" t="inlineStr">
+      <c r="G31" s="65" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="H31" s="68" t="n"/>
+      <c r="I31" s="69">
+        <f>IF(AND(F31&lt;&gt;"",H31&lt;&gt;""),F31*H31,"")</f>
+        <v/>
+      </c>
+      <c r="J31" s="73" t="inlineStr">
+        <is>
+          <t>De cumparat</t>
+        </is>
+      </c>
+      <c r="K31" s="66" t="n"/>
+      <c r="L31" s="66" t="inlineStr">
+        <is>
+          <t>Sub platforma — amortizare cadere</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="48">
+      <c r="A32" s="94" t="inlineStr">
+        <is>
+          <t>Joaca</t>
+        </is>
+      </c>
+      <c r="B32" s="95" t="inlineStr">
+        <is>
+          <t>Tobogan</t>
+        </is>
+      </c>
+      <c r="C32" s="94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D32" s="94" t="n"/>
+      <c r="E32" s="94" t="n"/>
+      <c r="F32" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
       </c>
-      <c r="H28" s="68" t="n">
-        <v>144.39</v>
-      </c>
-      <c r="I28" s="69">
-        <f>IF(AND(F28&lt;&gt;"",H28&lt;&gt;""),F28*H28,"")</f>
-        <v/>
-      </c>
-      <c r="J28" s="73" t="inlineStr">
-        <is>
-          <t>Cumparat</t>
-        </is>
-      </c>
-      <c r="K28" s="66" t="n"/>
-      <c r="L28" s="66" t="inlineStr">
-        <is>
-          <t>Finisaj larice + lemn expus · comanda 09.06.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="48">
-      <c r="A29" s="94" t="inlineStr">
-        <is>
-          <t>Finisaj</t>
-        </is>
-      </c>
-      <c r="B29" s="95" t="inlineStr">
-        <is>
-          <t>Grund impregnare lemn (AVEM)</t>
-        </is>
-      </c>
-      <c r="C29" s="94" t="inlineStr">
-        <is>
-          <t>Köber pe baza de apa 4 L</t>
-        </is>
-      </c>
-      <c r="D29" s="94" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E29" s="94" t="n"/>
-      <c r="F29" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="94" t="inlineStr">
-        <is>
-          <t>buc</t>
-        </is>
-      </c>
-      <c r="H29" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="62">
-        <f>IF(AND(F29&lt;&gt;"",H29&lt;&gt;""),F29*H29,"")</f>
-        <v/>
-      </c>
-      <c r="J29" s="74" t="inlineStr">
-        <is>
-          <t>Cumparat</t>
-        </is>
-      </c>
-      <c r="K29" s="95" t="n"/>
-      <c r="L29" s="95" t="inlineStr">
-        <is>
-          <t>Il avem deja; inlocuieste lazura Hornbach. Strat de baza structura.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="48">
-      <c r="A30" s="65" t="inlineStr">
-        <is>
-          <t>Siguranta</t>
-        </is>
-      </c>
-      <c r="B30" s="66" t="inlineStr">
-        <is>
-          <t>Material sol moale</t>
-        </is>
-      </c>
-      <c r="C30" s="65" t="inlineStr">
-        <is>
-          <t>scoarta/nisip</t>
-        </is>
-      </c>
-      <c r="D30" s="65" t="n"/>
-      <c r="E30" s="65" t="n"/>
-      <c r="F30" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="G30" s="65" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="H30" s="68" t="n"/>
-      <c r="I30" s="69">
-        <f>IF(AND(F30&lt;&gt;"",H30&lt;&gt;""),F30*H30,"")</f>
-        <v/>
-      </c>
-      <c r="J30" s="73" t="inlineStr">
-        <is>
-          <t>De cumparat</t>
-        </is>
-      </c>
-      <c r="K30" s="66" t="n"/>
-      <c r="L30" s="66" t="inlineStr">
-        <is>
-          <t>Sub platforma — amortizare cadere</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="48">
-      <c r="A31" s="94" t="inlineStr">
-        <is>
-          <t>Joaca</t>
-        </is>
-      </c>
-      <c r="B31" s="95" t="inlineStr">
-        <is>
-          <t>Tobogan</t>
-        </is>
-      </c>
-      <c r="C31" s="94" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D31" s="94" t="n"/>
-      <c r="E31" s="94" t="n"/>
-      <c r="F31" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" s="94" t="inlineStr">
-        <is>
-          <t>buc</t>
-        </is>
-      </c>
-      <c r="H31" s="61" t="n"/>
-      <c r="I31" s="62">
-        <f>IF(AND(F31&lt;&gt;"",H31&lt;&gt;""),F31*H31,"")</f>
-        <v/>
-      </c>
-      <c r="J31" s="72" t="inlineStr">
+      <c r="H32" s="61" t="n"/>
+      <c r="I32" s="62">
+        <f>IF(AND(F32&lt;&gt;"",H32&lt;&gt;""),F32*H32,"")</f>
+        <v/>
+      </c>
+      <c r="J32" s="72" t="inlineStr">
         <is>
           <t>De decis</t>
         </is>
       </c>
-      <c r="K31" s="95" t="n"/>
-      <c r="L31" s="95" t="inlineStr">
-        <is>
-          <t>Extra, optional</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="48">
-      <c r="A32" s="65" t="inlineStr">
-        <is>
-          <t>Joaca</t>
-        </is>
-      </c>
-      <c r="B32" s="66" t="inlineStr">
-        <is>
-          <t>Franghie catarare / scripete cu galeata</t>
-        </is>
-      </c>
-      <c r="C32" s="65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D32" s="65" t="n"/>
-      <c r="E32" s="65" t="n"/>
-      <c r="F32" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="G32" s="65" t="inlineStr">
-        <is>
-          <t>set</t>
-        </is>
-      </c>
-      <c r="H32" s="68" t="n"/>
-      <c r="I32" s="69">
-        <f>IF(AND(F32&lt;&gt;"",H32&lt;&gt;""),F32*H32,"")</f>
-        <v/>
-      </c>
-      <c r="J32" s="75" t="inlineStr">
-        <is>
-          <t>De decis</t>
-        </is>
-      </c>
-      <c r="K32" s="66" t="n"/>
-      <c r="L32" s="66" t="inlineStr">
+      <c r="K32" s="95" t="n"/>
+      <c r="L32" s="95" t="inlineStr">
         <is>
           <t>Extra, optional</t>
         </is>
@@ -2089,17 +2099,17 @@
     <row r="33">
       <c r="A33" s="65" t="inlineStr">
         <is>
-          <t>Finisaj</t>
+          <t>Joaca</t>
         </is>
       </c>
       <c r="B33" s="66" t="inlineStr">
         <is>
-          <t>Topcoat colorat exterior</t>
+          <t>Franghie catarare / scripete cu galeata</t>
         </is>
       </c>
       <c r="C33" s="65" t="inlineStr">
         <is>
-          <t>alegerea ta de culoare</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D33" s="65" t="n"/>
@@ -2109,12 +2119,10 @@
       </c>
       <c r="G33" s="65" t="inlineStr">
         <is>
-          <t>buc</t>
-        </is>
-      </c>
-      <c r="H33" s="68" t="n">
-        <v>170</v>
-      </c>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="H33" s="68" t="n"/>
       <c r="I33" s="69">
         <f>IF(AND(F33&lt;&gt;"",H33&lt;&gt;""),F33*H33,"")</f>
         <v/>
@@ -2127,34 +2135,79 @@
       <c r="K33" s="66" t="n"/>
       <c r="L33" s="66" t="inlineStr">
         <is>
+          <t>Extra, optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="48">
+      <c r="A34" s="65" t="inlineStr">
+        <is>
+          <t>Finisaj</t>
+        </is>
+      </c>
+      <c r="B34" s="66" t="inlineStr">
+        <is>
+          <t>Topcoat colorat exterior</t>
+        </is>
+      </c>
+      <c r="C34" s="65" t="inlineStr">
+        <is>
+          <t>alegerea ta de culoare</t>
+        </is>
+      </c>
+      <c r="D34" s="65" t="n"/>
+      <c r="E34" s="65" t="n"/>
+      <c r="F34" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="65" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="H34" s="68" t="n">
+        <v>170</v>
+      </c>
+      <c r="I34" s="69">
+        <f>IF(AND(F34&lt;&gt;"",H34&lt;&gt;""),F34*H34,"")</f>
+        <v/>
+      </c>
+      <c r="J34" s="75" t="inlineStr">
+        <is>
+          <t>De decis</t>
+        </is>
+      </c>
+      <c r="K34" s="66" t="n"/>
+      <c r="L34" s="66" t="inlineStr">
+        <is>
           <t>Culoarea finala; il alegi tu</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="48">
-      <c r="A34" s="76" t="inlineStr">
+    <row r="35" ht="15" customHeight="1" s="48">
+      <c r="A35" s="76" t="inlineStr">
         <is>
           <t>Legenda status:</t>
         </is>
       </c>
-      <c r="B34" s="77" t="inlineStr">
+      <c r="B35" s="77" t="inlineStr">
         <is>
           <t>Cumparat</t>
         </is>
       </c>
-      <c r="C34" s="78" t="inlineStr">
+      <c r="C35" s="78" t="inlineStr">
         <is>
           <t>De cumparat</t>
         </is>
       </c>
-      <c r="D34" s="79" t="inlineStr">
+      <c r="D35" s="79" t="inlineStr">
         <is>
           <t>De decis</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="48">
-      <c r="A35" s="80" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="80" t="inlineStr">
         <is>
           <t>Preturile goale se completeaza in magazin. Total se calculeaza automat (Cant. x Pret unitar).</t>
         </is>
@@ -3888,7 +3941,7 @@
         <v>4.83</v>
       </c>
       <c r="E17" s="60" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F17" s="94" t="inlineStr">
         <is>
@@ -3901,7 +3954,7 @@
       </c>
       <c r="H17" s="95" t="inlineStr">
         <is>
-          <t>Joiste → grinda, anti-ridicare</t>
+          <t>Joiste → grinda + grinda spate, anti-ridicare (12+2=14)</t>
         </is>
       </c>
       <c r="I17" s="74" t="inlineStr">
@@ -4056,7 +4109,7 @@
         <v>55.82</v>
       </c>
       <c r="E21" s="60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F21" s="94" t="inlineStr">
         <is>
@@ -4672,7 +4725,7 @@
         <v>4.83</v>
       </c>
       <c r="D10" s="60" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E10" s="62">
         <f>C10*D10</f>
@@ -4800,7 +4853,7 @@
         <v>55.82</v>
       </c>
       <c r="D14" s="60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E14" s="62">
         <f>C14*D14</f>
@@ -5183,8 +5236,36 @@
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="48">
-      <c r="D27" s="92" t="n"/>
-      <c r="E27" s="93" t="n"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Bulon M10×120 + piulita + saiba — balustrada (Faza 1)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D27" s="92" t="n">
+        <v>12</v>
+      </c>
+      <c r="E27" s="93">
+        <f>C27*D27</f>
+        <v/>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>de confirmat</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>BM</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="48">
       <c r="D28" s="92" t="inlineStr">

</xml_diff>

<commit_message>
Tidy: tracker 6x100 fara contrafise, materiale.html C2=14/H4=3pac COMANDAT
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tracker_materiale_casuta.xlsx
+++ b/Tracker_materiale_casuta.xlsx
@@ -1477,53 +1477,53 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="48">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="47" t="inlineStr">
         <is>
           <t>Balustrada</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="47" t="inlineStr">
         <is>
           <t>Buloane M10 (balustrada)</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="47" t="inlineStr">
         <is>
           <t>M10×120 + piulita + saiba</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="47" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="47" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" s="47" t="n">
         <v>12</v>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="47" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
       </c>
-      <c r="H20" t="n">
+      <c r="H20" s="47" t="n">
         <v>3.5</v>
       </c>
-      <c r="I20">
+      <c r="I20" s="47">
         <f>IF(AND(F20&lt;&gt;"",H20&lt;&gt;""),F20*H20,"")</f>
         <v/>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J20" s="47" t="inlineStr">
         <is>
           <t>De cumparat</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr">
+      <c r="K20" s="47" t="inlineStr"/>
+      <c r="L20" s="47" t="inlineStr">
         <is>
           <t>Faza 1; prinde stalpisorii 58x58 de cadru</t>
         </is>
@@ -3451,6 +3451,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="25.5" customHeight="1" s="48">
       <c r="A4" s="57" t="inlineStr">
         <is>
@@ -4038,7 +4039,7 @@
       </c>
       <c r="H19" s="95" t="inlineStr">
         <is>
-          <t>Coltare, conectori, contrafise</t>
+          <t>Coltare, conectori</t>
         </is>
       </c>
       <c r="I19" s="74" t="inlineStr">
@@ -4455,6 +4456,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32" ht="15" customHeight="1" s="48">
       <c r="F32" s="89" t="inlineStr">
         <is>
@@ -4477,6 +4479,7 @@
         <v/>
       </c>
     </row>
+    <row r="34"/>
     <row r="35" ht="15" customHeight="1" s="48">
       <c r="A35" s="80" t="inlineStr">
         <is>
@@ -5236,17 +5239,17 @@
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="48">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="47" t="inlineStr">
         <is>
           <t>Bulon M10×120 + piulita + saiba — balustrada (Faza 1)</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="47" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C27" t="n">
+      <c r="C27" s="47" t="n">
         <v>3.5</v>
       </c>
       <c r="D27" s="92" t="n">
@@ -5256,12 +5259,12 @@
         <f>C27*D27</f>
         <v/>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="47" t="inlineStr">
         <is>
           <t>de confirmat</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="47" t="inlineStr">
         <is>
           <t>BM</t>
         </is>

</xml_diff>

<commit_message>
Audit fixes 2026-06-18: 14 puncte aplicate
DOC: stalpisori balustrada x7, inventar ghid C2x14/qty18, Debitare P22 (14), tracker buget 8500, mana curenta + feronerie poarta adaugate, sectiune BALUSTRADA in Platforma premium, avertisment receptie C2/inox in Comanda Hornbach, balustrada scoasa din nota Faza 2.
PIPE: requirements.txt, README pipeline order, .gitignore ~$*.xlsx, book.html sters.
PDF: 02-Ghid-montaj + 06-Materiale regenerate.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tracker_materiale_casuta.xlsx
+++ b/Tracker_materiale_casuta.xlsx
@@ -851,7 +851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="47" min="1" max="1"/>
@@ -876,7 +876,7 @@
     <row r="2" ht="15.75" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Proiect cu Tudor (11 ani) · casuta pe 4 stalpi + balcon · buget = TOT proiectul (Faza 1 platforma ~5000 + Faza 2 pereti/acoperis/balustrada/scara). Doar platforma Faza 1: vezi foaia "Platforma premium" / "Comanda Hornbach". Ajusteaza C3 la plafonul tau real.</t>
+          <t>Proiect cu Tudor (11 ani) · casuta pe 4 stalpi + balcon · buget = TOT proiectul (Faza 1 platforma ~5000 + Faza 2 pereti/acoperis/scara). Doar platforma Faza 1: vezi foaia "Platforma premium" / "Comanda Hornbach". Ajusteaza C3 la plafonul tau real.</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="C3" s="52" t="n">
-        <v>6600</v>
+        <v>8500</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="48">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="J14" s="73" t="inlineStr">
         <is>
-          <t>Cumparat</t>
+          <t>Sosit 18.06</t>
         </is>
       </c>
       <c r="K14" s="66" t="n"/>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="J15" s="74" t="inlineStr">
         <is>
-          <t>Cumparat</t>
+          <t>Sosit 18.06</t>
         </is>
       </c>
       <c r="K15" s="95" t="n"/>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="J16" s="73" t="inlineStr">
         <is>
-          <t>Cumparat</t>
+          <t>Sosit 18.06</t>
         </is>
       </c>
       <c r="K16" s="66" t="n"/>
@@ -1745,7 +1745,7 @@
       </c>
       <c r="J25" s="73" t="inlineStr">
         <is>
-          <t>Cumparat</t>
+          <t>Sosit 18.06</t>
         </is>
       </c>
       <c r="K25" s="66" t="n"/>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="J26" s="74" t="inlineStr">
         <is>
-          <t>Cumparat</t>
+          <t>Sosit 18.06</t>
         </is>
       </c>
       <c r="K26" s="95" t="n"/>
@@ -1848,7 +1848,7 @@
       </c>
       <c r="J27" s="73" t="inlineStr">
         <is>
-          <t>Cumparat</t>
+          <t>Sosit 18.06</t>
         </is>
       </c>
       <c r="K27" s="66" t="n"/>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="J28" s="74" t="inlineStr">
         <is>
-          <t>Cumparat</t>
+          <t>Sosit 18.06</t>
         </is>
       </c>
       <c r="K28" s="95" t="n"/>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="J29" s="73" t="inlineStr">
         <is>
-          <t>Cumparat</t>
+          <t>Sosit 18.06</t>
         </is>
       </c>
       <c r="K29" s="66" t="n"/>
@@ -2185,29 +2185,112 @@
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="48">
-      <c r="A35" s="76" t="inlineStr">
+      <c r="A35" s="47" t="inlineStr">
+        <is>
+          <t>Balustrada</t>
+        </is>
+      </c>
+      <c r="B35" s="47" t="inlineStr">
+        <is>
+          <t>Mana curenta + rigla jos</t>
+        </is>
+      </c>
+      <c r="C35" s="47" t="inlineStr">
+        <is>
+          <t>45x70, ~9 m total</t>
+        </is>
+      </c>
+      <c r="D35" s="47" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="F35" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="G35" s="47" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="I35" s="47">
+        <f>IF(AND(F35&lt;&gt;"",H35&lt;&gt;""),F35*H35,"")</f>
+        <v/>
+      </c>
+      <c r="J35" s="47" t="inlineStr">
+        <is>
+          <t>De cumparat</t>
+        </is>
+      </c>
+      <c r="L35" s="47" t="inlineStr">
+        <is>
+          <t>Sus+jos pe 3 laturi; lipsea din tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="47" t="inlineStr">
+        <is>
+          <t>Balustrada</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="inlineStr">
+        <is>
+          <t>Feronerie poarta</t>
+        </is>
+      </c>
+      <c r="C36" s="47" t="inlineStr">
+        <is>
+          <t>2x balama cu arc (self-close) + zavor copil sus</t>
+        </is>
+      </c>
+      <c r="F36" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="47" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="I36" s="47">
+        <f>IF(AND(F36&lt;&gt;"",H36&lt;&gt;""),F36*H36,"")</f>
+        <v/>
+      </c>
+      <c r="J36" s="47" t="inlineStr">
+        <is>
+          <t>De cumparat</t>
+        </is>
+      </c>
+      <c r="L36" s="47" t="inlineStr">
+        <is>
+          <t>Poarta auto-inchidere la capul scarii (SIG-03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="76" t="inlineStr">
         <is>
           <t>Legenda status:</t>
         </is>
       </c>
-      <c r="B35" s="77" t="inlineStr">
+      <c r="B37" s="77" t="inlineStr">
         <is>
           <t>Cumparat</t>
         </is>
       </c>
-      <c r="C35" s="78" t="inlineStr">
+      <c r="C37" s="78" t="inlineStr">
         <is>
           <t>De cumparat</t>
         </is>
       </c>
-      <c r="D35" s="79" t="inlineStr">
+      <c r="D37" s="79" t="inlineStr">
         <is>
           <t>De decis</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="80" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="80" t="inlineStr">
         <is>
           <t>Preturile goale se completeaza in magazin. Total se calculeaza automat (Cant. x Pret unitar).</t>
         </is>
@@ -3156,7 +3239,7 @@
       </c>
       <c r="C35" s="95" t="inlineStr">
         <is>
-          <t>C1 100x100x90 (4) + C2 90x90x65 (12)</t>
+          <t>C1 100x100x90 (4) + C2 90x90x65 (14)</t>
         </is>
       </c>
       <c r="D35" s="97" t="inlineStr">
@@ -3166,7 +3249,7 @@
       </c>
       <c r="E35" s="97" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="F35" s="74" t="inlineStr">
@@ -3181,7 +3264,7 @@
       </c>
       <c r="H35" s="95" t="inlineStr">
         <is>
-          <t>C1 grinda fata-&gt;stalp (4); C2 joiste anti-ridicare (12).</t>
+          <t>C1 grinda fata-&gt;stalp (4); C2 joiste anti-ridicare (14).</t>
         </is>
       </c>
     </row>
@@ -3423,7 +3506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="47" min="1" max="1"/>
@@ -3451,7 +3534,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="25.5" customHeight="1" s="48">
       <c r="A4" s="57" t="inlineStr">
         <is>
@@ -4456,32 +4538,243 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
+    <row r="31">
+      <c r="A31" s="47" t="inlineStr">
+        <is>
+          <t>BALUSTRADA</t>
+        </is>
+      </c>
+    </row>
     <row r="32" ht="15" customHeight="1" s="48">
-      <c r="F32" s="89" t="inlineStr">
+      <c r="A32" s="47" t="inlineStr">
+        <is>
+          <t>Balustrada</t>
+        </is>
+      </c>
+      <c r="B32" s="47" t="inlineStr">
+        <is>
+          <t>Stalpisori 58x58, h=100 cm</t>
+        </is>
+      </c>
+      <c r="C32" s="47" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="D32" s="47" t="n">
+        <v>60.91</v>
+      </c>
+      <c r="E32" s="47" t="n">
+        <v>7</v>
+      </c>
+      <c r="F32" s="47" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="G32" s="47">
+        <f>IF(AND(D32&lt;&gt;"",E32&lt;&gt;""),D32*E32,"")</f>
+        <v/>
+      </c>
+      <c r="H32" s="47" t="inlineStr">
+        <is>
+          <t>Stalpisori balustrada, jur-imprejur</t>
+        </is>
+      </c>
+      <c r="I32" s="47" t="inlineStr">
+        <is>
+          <t>De cumparat (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="48">
+      <c r="A33" s="47" t="inlineStr">
+        <is>
+          <t>Balustrada</t>
+        </is>
+      </c>
+      <c r="B33" s="47" t="inlineStr">
+        <is>
+          <t>Sipci 18x18 umplutura goluri</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="D33" s="47" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E33" s="47" t="n">
+        <v>24</v>
+      </c>
+      <c r="F33" s="47" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="G33" s="47">
+        <f>IF(AND(D33&lt;&gt;"",E33&lt;&gt;""),D33*E33,"")</f>
+        <v/>
+      </c>
+      <c r="H33" s="47" t="inlineStr">
+        <is>
+          <t>Goluri sub 9 cm</t>
+        </is>
+      </c>
+      <c r="I33" s="47" t="inlineStr">
+        <is>
+          <t>De cumparat (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="47" t="inlineStr">
+        <is>
+          <t>Balustrada</t>
+        </is>
+      </c>
+      <c r="B34" s="47" t="inlineStr">
+        <is>
+          <t>Mana curenta + rigla jos 45x70</t>
+        </is>
+      </c>
+      <c r="C34" s="47" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="D34" s="47" t="inlineStr">
+        <is>
+          <t>est.</t>
+        </is>
+      </c>
+      <c r="E34" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="47" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="H34" s="47" t="inlineStr">
+        <is>
+          <t>Sus+jos, ~9 m total (3 laturi)</t>
+        </is>
+      </c>
+      <c r="I34" s="47" t="inlineStr">
+        <is>
+          <t>De cumparat (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1" s="48">
+      <c r="A35" s="47" t="inlineStr">
+        <is>
+          <t>Balustrada</t>
+        </is>
+      </c>
+      <c r="B35" s="47" t="inlineStr">
+        <is>
+          <t>Buloane M10x120 + piulita + saiba</t>
+        </is>
+      </c>
+      <c r="C35" s="47" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="D35" s="47" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E35" s="47" t="n">
+        <v>14</v>
+      </c>
+      <c r="F35" s="47" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="G35" s="47">
+        <f>IF(AND(D35&lt;&gt;"",E35&lt;&gt;""),D35*E35,"")</f>
+        <v/>
+      </c>
+      <c r="H35" s="47" t="inlineStr">
+        <is>
+          <t>Prindere stalpisori de cadru</t>
+        </is>
+      </c>
+      <c r="I35" s="47" t="inlineStr">
+        <is>
+          <t>De cumparat (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="47" t="inlineStr">
+        <is>
+          <t>Balustrada</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="inlineStr">
+        <is>
+          <t>Feronerie poarta (self-close)</t>
+        </is>
+      </c>
+      <c r="C36" s="47" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="D36" s="47" t="inlineStr">
+        <is>
+          <t>est.</t>
+        </is>
+      </c>
+      <c r="E36" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="47" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="H36" s="47" t="inlineStr">
+        <is>
+          <t>2x balama arc + zavor copil sus; de confirmat</t>
+        </is>
+      </c>
+      <c r="I36" s="47" t="inlineStr">
+        <is>
+          <t>De cumparat (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="F38" s="89" t="inlineStr">
         <is>
           <t>TOTAL platforma:</t>
         </is>
       </c>
-      <c r="G32" s="90">
-        <f>SUM(G5:G30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="48">
-      <c r="F33" s="76" t="inlineStr">
+      <c r="G38" s="90">
+        <f>SUM(G5:G36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="F39" s="76" t="inlineStr">
         <is>
           <t>din care DE CUMPARAT:</t>
         </is>
       </c>
-      <c r="G33" s="91">
-        <f>SUMIF(I5:I30,"De cumparat*",G5:G30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34"/>
-    <row r="35" ht="15" customHeight="1" s="48">
-      <c r="A35" s="80" t="inlineStr">
+      <c r="G39" s="91">
+        <f>SUMIF(I5:I36,"De cumparat*",G5:G36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="80" t="inlineStr">
         <is>
           <t>Scara: 10 trepte (11 niveluri), riser 200 / calcai 190, ~49°, latime 600, mana curenta pe ambele parti, poarta la S3 (opus mesei de pe S4). Preturi 'est.' = de confirmat la magazin.</t>
         </is>
@@ -4495,8 +4788,8 @@
     <mergeCell ref="A28:I28"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A31:I31"/>
     <mergeCell ref="A22:I22"/>
-    <mergeCell ref="A35:I35"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4524,14 +4817,14 @@
     <row r="1" ht="27.75" customHeight="1" s="48">
       <c r="A1" s="81" t="inlineStr">
         <is>
-          <t>CASUTA DIN COPAC  ·  COMANDA HORNBACH (in cos)</t>
+          <t>CASUTA DIN COPAC  ·  COMANDA HORNBACH (in cos) · SOSITA 18.06.2026</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="48">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>COMANDA PLASATA 09.06.2026 · 14 produse · subtotal 3886,24 + livrare 215 = 4101,24 lei. Coloana 'Cod piesa' leaga de catalogul de piese.</t>
+          <t>COMANDA PLASATA 09.06.2026 · 14 produse · subtotal 3886,24 + livrare 215 = 4101,24 lei. Coloana 'Cod piesa' leaga de catalogul de piese. · DE VERIFICAT LA RECEPTIE: C2 14 vs 12 platit, inox 3 vs 2 platit</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4901,7 @@
       </c>
       <c r="F6" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G6" s="94" t="inlineStr">
@@ -4640,7 +4933,7 @@
       </c>
       <c r="F7" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G7" s="94" t="inlineStr">
@@ -4672,7 +4965,7 @@
       </c>
       <c r="F8" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G8" s="94" t="inlineStr">
@@ -4704,7 +4997,7 @@
       </c>
       <c r="F9" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G9" s="94" t="inlineStr">
@@ -4736,7 +5029,7 @@
       </c>
       <c r="F10" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G10" s="94" t="inlineStr">
@@ -4768,7 +5061,7 @@
       </c>
       <c r="F11" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G11" s="94" t="inlineStr">
@@ -4800,7 +5093,7 @@
       </c>
       <c r="F12" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G12" s="94" t="inlineStr">
@@ -4832,7 +5125,7 @@
       </c>
       <c r="F13" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G13" s="94" t="inlineStr">
@@ -4864,7 +5157,7 @@
       </c>
       <c r="F14" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G14" s="94" t="inlineStr">
@@ -4896,7 +5189,7 @@
       </c>
       <c r="F15" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G15" s="94" t="inlineStr">
@@ -4928,7 +5221,7 @@
       </c>
       <c r="F16" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G16" s="94" t="inlineStr">
@@ -4960,7 +5253,7 @@
       </c>
       <c r="F17" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G17" s="94" t="inlineStr">
@@ -5037,7 +5330,7 @@
       </c>
       <c r="F20" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G20" s="94" t="inlineStr">
@@ -5069,7 +5362,7 @@
       </c>
       <c r="F21" s="96" t="inlineStr">
         <is>
-          <t>COMANDAT</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
       <c r="G21" s="94" t="inlineStr">

</xml_diff>

<commit_message>
talpic: bloc compresiune sub polita propagat in fise/ghid/3D/tracker + PDF regenerate
</commit_message>
<xml_diff>
--- a/Tracker_materiale_casuta.xlsx
+++ b/Tracker_materiale_casuta.xlsx
@@ -1337,7 +1337,7 @@
       </c>
       <c r="B17" s="95" t="inlineStr">
         <is>
-          <t>Polita + blocaje + rama gaura copac</t>
+          <t>Polita + talpic + blocaje + rama gaura copac</t>
         </is>
       </c>
       <c r="C17" s="94" t="inlineStr">
@@ -1374,7 +1374,7 @@
       <c r="K17" s="95" t="n"/>
       <c r="L17" s="95" t="inlineStr">
         <is>
-          <t>Sub grinda spate + blocaje + incadrare gaura. Gratis din offcut.</t>
+          <t>Sub grinda spate: polita + TALPICUL de sub ea (bloc ~180, reazem la compresiune) + blocaje + incadrare gaura. Gratis din offcut — nu se cumpara nimic in plus.</t>
         </is>
       </c>
     </row>
@@ -2317,7 +2317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="47" min="1" max="1"/>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="H7" s="95" t="inlineStr">
         <is>
-          <t>Taiati la +1872 (sub podea: grinda 200 + joista 100 + dusumea 28 = 2200). Offcut ~2128 pt contrafise/blocuri.</t>
+          <t>Taiati la +1872 (sub podea: grinda 200 + joista 100 + dusumea 28 = 2200). Offcut ~2128 pt polite, talpice, contrafise/blocuri.</t>
         </is>
       </c>
     </row>
@@ -2610,113 +2610,113 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" s="48">
+    <row r="11" ht="21.75" customHeight="1" s="48">
       <c r="A11" s="72" t="inlineStr">
         <is>
+          <t>P4c</t>
+        </is>
+      </c>
+      <c r="B11" s="95" t="inlineStr">
+        <is>
+          <t>Talpic sub polita (bloc compresiune)</t>
+        </is>
+      </c>
+      <c r="C11" s="95" t="inlineStr">
+        <is>
+          <t>din offcut 100×100</t>
+        </is>
+      </c>
+      <c r="D11" s="97" t="inlineStr">
+        <is>
+          <t>~180</t>
+        </is>
+      </c>
+      <c r="E11" s="97" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F11" s="96" t="inlineStr">
+        <is>
+          <t>DIN OFFCUT</t>
+        </is>
+      </c>
+      <c r="G11" s="94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" s="95" t="inlineStr">
+        <is>
+          <t>Cate unul sub fiecare polita, pe fata stalpului din spate. Polita reazema pe el (compresiune); buloanele M12 = doar pozitie + anti-smulgere. Confirma masura pe teren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="21.75" customHeight="1" s="48">
+      <c r="A12" s="72" t="inlineStr">
+        <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="B11" s="83" t="n"/>
-      <c r="C11" s="83" t="n"/>
-      <c r="D11" s="83" t="n"/>
-      <c r="E11" s="83" t="n"/>
-      <c r="F11" s="83" t="n"/>
-      <c r="G11" s="83" t="n"/>
-      <c r="H11" s="84" t="n"/>
-    </row>
-    <row r="12" ht="21.75" customHeight="1" s="48">
-      <c r="A12" s="82" t="inlineStr">
+      <c r="B12" s="83" t="n"/>
+      <c r="C12" s="83" t="n"/>
+      <c r="D12" s="83" t="n"/>
+      <c r="E12" s="83" t="n"/>
+      <c r="F12" s="83" t="n"/>
+      <c r="G12" s="83" t="n"/>
+      <c r="H12" s="84" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="48">
+      <c r="A13" s="82" t="inlineStr">
         <is>
           <t>PODEA</t>
         </is>
       </c>
-      <c r="B12" s="86" t="n"/>
-      <c r="C12" s="86" t="n"/>
-      <c r="D12" s="86" t="n"/>
-      <c r="E12" s="86" t="n"/>
-      <c r="F12" s="86" t="n"/>
-      <c r="G12" s="86" t="n"/>
-      <c r="H12" s="87" t="n"/>
-    </row>
-    <row r="13" ht="18" customHeight="1" s="48">
-      <c r="A13" s="72" t="inlineStr">
+      <c r="B13" s="86" t="n"/>
+      <c r="C13" s="86" t="n"/>
+      <c r="D13" s="86" t="n"/>
+      <c r="E13" s="86" t="n"/>
+      <c r="F13" s="86" t="n"/>
+      <c r="G13" s="86" t="n"/>
+      <c r="H13" s="87" t="n"/>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="48">
+      <c r="A14" s="72" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
       </c>
-      <c r="B13" s="83" t="n"/>
-      <c r="C13" s="83" t="n"/>
-      <c r="D13" s="83" t="n"/>
-      <c r="E13" s="83" t="n"/>
-      <c r="F13" s="83" t="n"/>
-      <c r="G13" s="83" t="n"/>
-      <c r="H13" s="84" t="n"/>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="48">
-      <c r="A14" s="82" t="inlineStr">
+      <c r="B14" s="83" t="n"/>
+      <c r="C14" s="83" t="n"/>
+      <c r="D14" s="83" t="n"/>
+      <c r="E14" s="83" t="n"/>
+      <c r="F14" s="83" t="n"/>
+      <c r="G14" s="83" t="n"/>
+      <c r="H14" s="84" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="48">
+      <c r="A15" s="82" t="inlineStr">
         <is>
           <t>PERETI CASUTA (bracaj)</t>
         </is>
       </c>
-      <c r="B14" s="86" t="n"/>
-      <c r="C14" s="86" t="n"/>
-      <c r="D14" s="86" t="n"/>
-      <c r="E14" s="86" t="n"/>
-      <c r="F14" s="86" t="n"/>
-      <c r="G14" s="86" t="n"/>
-      <c r="H14" s="87" t="n"/>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="48">
-      <c r="A15" s="72" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="B15" s="95" t="inlineStr">
-        <is>
-          <t>Talpi + coronament pereti</t>
-        </is>
-      </c>
-      <c r="C15" s="95" t="inlineStr">
-        <is>
-          <t>50×80</t>
-        </is>
-      </c>
-      <c r="D15" s="97" t="inlineStr">
-        <is>
-          <t>var</t>
-        </is>
-      </c>
-      <c r="E15" s="97" t="inlineStr">
-        <is>
-          <t>~6</t>
-        </is>
-      </c>
-      <c r="F15" s="74" t="inlineStr">
-        <is>
-          <t>NOU</t>
-        </is>
-      </c>
-      <c r="G15" s="94" t="inlineStr">
-        <is>
-          <t>oricare</t>
-        </is>
-      </c>
-      <c r="H15" s="95" t="inlineStr">
-        <is>
-          <t>Plate sus/jos pe cele 4 laturi (gol usa spre balcon).</t>
-        </is>
-      </c>
+      <c r="B15" s="86" t="n"/>
+      <c r="C15" s="86" t="n"/>
+      <c r="D15" s="86" t="n"/>
+      <c r="E15" s="86" t="n"/>
+      <c r="F15" s="86" t="n"/>
+      <c r="G15" s="86" t="n"/>
+      <c r="H15" s="87" t="n"/>
     </row>
     <row r="16" ht="21.75" customHeight="1" s="48">
       <c r="A16" s="72" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="B16" s="95" t="inlineStr">
         <is>
-          <t>Montanti pereti</t>
+          <t>Talpi + coronament pereti</t>
         </is>
       </c>
       <c r="C16" s="95" t="inlineStr">
@@ -2726,12 +2726,12 @@
       </c>
       <c r="D16" s="97" t="inlineStr">
         <is>
-          <t>~1400</t>
+          <t>var</t>
         </is>
       </c>
       <c r="E16" s="97" t="inlineStr">
         <is>
-          <t>~14</t>
+          <t>~6</t>
         </is>
       </c>
       <c r="F16" s="74" t="inlineStr">
@@ -2746,104 +2746,104 @@
       </c>
       <c r="H16" s="95" t="inlineStr">
         <is>
-          <t>Interax 600 mm. Mai inalti in spate (latura coamei).</t>
+          <t>Plate sus/jos pe cele 4 laturi (gol usa spre balcon).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" s="48">
       <c r="A17" s="72" t="inlineStr">
         <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B17" s="95" t="inlineStr">
+        <is>
+          <t>Montanti pereti</t>
+        </is>
+      </c>
+      <c r="C17" s="95" t="inlineStr">
+        <is>
+          <t>50×80</t>
+        </is>
+      </c>
+      <c r="D17" s="97" t="inlineStr">
+        <is>
+          <t>~1400</t>
+        </is>
+      </c>
+      <c r="E17" s="97" t="inlineStr">
+        <is>
+          <t>~14</t>
+        </is>
+      </c>
+      <c r="F17" s="74" t="inlineStr">
+        <is>
+          <t>NOU</t>
+        </is>
+      </c>
+      <c r="G17" s="94" t="inlineStr">
+        <is>
+          <t>oricare</t>
+        </is>
+      </c>
+      <c r="H17" s="95" t="inlineStr">
+        <is>
+          <t>Interax 600 mm. Mai inalti in spate (latura coamei).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="48">
+      <c r="A18" s="72" t="inlineStr">
+        <is>
           <t>P9</t>
         </is>
       </c>
-      <c r="B17" s="83" t="n"/>
-      <c r="C17" s="83" t="n"/>
-      <c r="D17" s="83" t="n"/>
-      <c r="E17" s="83" t="n"/>
-      <c r="F17" s="83" t="n"/>
-      <c r="G17" s="83" t="n"/>
-      <c r="H17" s="84" t="n"/>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="48">
-      <c r="A18" s="82" t="inlineStr">
+      <c r="B18" s="83" t="n"/>
+      <c r="C18" s="83" t="n"/>
+      <c r="D18" s="83" t="n"/>
+      <c r="E18" s="83" t="n"/>
+      <c r="F18" s="83" t="n"/>
+      <c r="G18" s="83" t="n"/>
+      <c r="H18" s="84" t="n"/>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="48">
+      <c r="A19" s="82" t="inlineStr">
         <is>
           <t>ACOPERIS (1 apa, doar casuta)</t>
         </is>
       </c>
-      <c r="B18" s="86" t="n"/>
-      <c r="C18" s="86" t="n"/>
-      <c r="D18" s="86" t="n"/>
-      <c r="E18" s="86" t="n"/>
-      <c r="F18" s="86" t="n"/>
-      <c r="G18" s="86" t="n"/>
-      <c r="H18" s="87" t="n"/>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="48">
-      <c r="A19" s="72" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="B19" s="95" t="inlineStr">
-        <is>
-          <t>Capriori</t>
-        </is>
-      </c>
-      <c r="C19" s="95" t="inlineStr">
-        <is>
-          <t>60×100</t>
-        </is>
-      </c>
-      <c r="D19" s="97" t="inlineStr">
-        <is>
-          <t>~1400</t>
-        </is>
-      </c>
-      <c r="E19" s="97" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F19" s="74" t="inlineStr">
-        <is>
-          <t>NOU</t>
-        </is>
-      </c>
-      <c r="G19" s="94" t="inlineStr">
-        <is>
-          <t>oricare</t>
-        </is>
-      </c>
-      <c r="H19" s="95" t="inlineStr">
-        <is>
-          <t>Panta spre gradina, mic streasin in spate.</t>
-        </is>
-      </c>
+      <c r="B19" s="86" t="n"/>
+      <c r="C19" s="86" t="n"/>
+      <c r="D19" s="86" t="n"/>
+      <c r="E19" s="86" t="n"/>
+      <c r="F19" s="86" t="n"/>
+      <c r="G19" s="86" t="n"/>
+      <c r="H19" s="87" t="n"/>
     </row>
     <row r="20" ht="21.75" customHeight="1" s="48">
       <c r="A20" s="72" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B20" s="95" t="inlineStr">
         <is>
-          <t>Astereala acoperis</t>
+          <t>Capriori</t>
         </is>
       </c>
       <c r="C20" s="95" t="inlineStr">
         <is>
-          <t>OSB3 / scandura</t>
+          <t>60×100</t>
         </is>
       </c>
       <c r="D20" s="97" t="inlineStr">
         <is>
-          <t>2500×1250</t>
+          <t>~1400</t>
         </is>
       </c>
       <c r="E20" s="97" t="inlineStr">
         <is>
-          <t>1 placa</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F20" s="74" t="inlineStr">
@@ -2858,104 +2858,104 @@
       </c>
       <c r="H20" s="95" t="inlineStr">
         <is>
-          <t>Suport invelitoare.</t>
+          <t>Panta spre gradina, mic streasin in spate.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1" s="48">
       <c r="A21" s="72" t="inlineStr">
         <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B21" s="95" t="inlineStr">
+        <is>
+          <t>Astereala acoperis</t>
+        </is>
+      </c>
+      <c r="C21" s="95" t="inlineStr">
+        <is>
+          <t>OSB3 / scandura</t>
+        </is>
+      </c>
+      <c r="D21" s="97" t="inlineStr">
+        <is>
+          <t>2500×1250</t>
+        </is>
+      </c>
+      <c r="E21" s="97" t="inlineStr">
+        <is>
+          <t>1 placa</t>
+        </is>
+      </c>
+      <c r="F21" s="74" t="inlineStr">
+        <is>
+          <t>NOU</t>
+        </is>
+      </c>
+      <c r="G21" s="94" t="inlineStr">
+        <is>
+          <t>oricare</t>
+        </is>
+      </c>
+      <c r="H21" s="95" t="inlineStr">
+        <is>
+          <t>Suport invelitoare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="48">
+      <c r="A22" s="72" t="inlineStr">
+        <is>
           <t>P12</t>
         </is>
       </c>
-      <c r="B21" s="83" t="n"/>
-      <c r="C21" s="83" t="n"/>
-      <c r="D21" s="83" t="n"/>
-      <c r="E21" s="83" t="n"/>
-      <c r="F21" s="83" t="n"/>
-      <c r="G21" s="83" t="n"/>
-      <c r="H21" s="84" t="n"/>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="48">
-      <c r="A22" s="82" t="inlineStr">
+      <c r="B22" s="83" t="n"/>
+      <c r="C22" s="83" t="n"/>
+      <c r="D22" s="83" t="n"/>
+      <c r="E22" s="83" t="n"/>
+      <c r="F22" s="83" t="n"/>
+      <c r="G22" s="83" t="n"/>
+      <c r="H22" s="84" t="n"/>
+    </row>
+    <row r="23" ht="15" customHeight="1" s="48">
+      <c r="A23" s="82" t="inlineStr">
         <is>
           <t>BALUSTRADA BALCON (3 laturi)</t>
         </is>
       </c>
-      <c r="B22" s="86" t="n"/>
-      <c r="C22" s="86" t="n"/>
-      <c r="D22" s="86" t="n"/>
-      <c r="E22" s="86" t="n"/>
-      <c r="F22" s="86" t="n"/>
-      <c r="G22" s="86" t="n"/>
-      <c r="H22" s="87" t="n"/>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="48">
-      <c r="A23" s="72" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="B23" s="95" t="inlineStr">
-        <is>
-          <t>Stalpisori balustrada</t>
-        </is>
-      </c>
-      <c r="C23" s="95" t="inlineStr">
-        <is>
-          <t>58×58</t>
-        </is>
-      </c>
-      <c r="D23" s="97" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="E23" s="97" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="F23" s="74" t="inlineStr">
-        <is>
-          <t>NOU</t>
-        </is>
-      </c>
-      <c r="G23" s="94" t="inlineStr">
-        <is>
-          <t>Hornbach</t>
-        </is>
-      </c>
-      <c r="H23" s="95" t="inlineStr">
-        <is>
-          <t>Interax ~900 mm, inclusiv pe nasul consolei.</t>
-        </is>
-      </c>
+      <c r="B23" s="86" t="n"/>
+      <c r="C23" s="86" t="n"/>
+      <c r="D23" s="86" t="n"/>
+      <c r="E23" s="86" t="n"/>
+      <c r="F23" s="86" t="n"/>
+      <c r="G23" s="86" t="n"/>
+      <c r="H23" s="87" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="48">
       <c r="A24" s="72" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B24" s="95" t="inlineStr">
         <is>
-          <t>Mana curenta + rigla jos</t>
+          <t>Stalpisori balustrada</t>
         </is>
       </c>
       <c r="C24" s="95" t="inlineStr">
         <is>
-          <t>45×70</t>
+          <t>58×58</t>
         </is>
       </c>
       <c r="D24" s="97" t="inlineStr">
         <is>
-          <t>~9 m total</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="E24" s="97" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F24" s="74" t="inlineStr">
@@ -2965,109 +2965,109 @@
       </c>
       <c r="G24" s="94" t="inlineStr">
         <is>
-          <t>oricare</t>
+          <t>Hornbach</t>
         </is>
       </c>
       <c r="H24" s="95" t="inlineStr">
         <is>
-          <t>Sus si jos, jur-imprejur.</t>
+          <t>Interax ~900 mm, inclusiv pe nasul consolei.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1" s="48">
       <c r="A25" s="72" t="inlineStr">
         <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B25" s="95" t="inlineStr">
+        <is>
+          <t>Mana curenta + rigla jos</t>
+        </is>
+      </c>
+      <c r="C25" s="95" t="inlineStr">
+        <is>
+          <t>45×70</t>
+        </is>
+      </c>
+      <c r="D25" s="97" t="inlineStr">
+        <is>
+          <t>~9 m total</t>
+        </is>
+      </c>
+      <c r="E25" s="97" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F25" s="74" t="inlineStr">
+        <is>
+          <t>NOU</t>
+        </is>
+      </c>
+      <c r="G25" s="94" t="inlineStr">
+        <is>
+          <t>oricare</t>
+        </is>
+      </c>
+      <c r="H25" s="95" t="inlineStr">
+        <is>
+          <t>Sus si jos, jur-imprejur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1" s="48">
+      <c r="A26" s="72" t="inlineStr">
+        <is>
           <t>P15</t>
         </is>
       </c>
-      <c r="B25" s="83" t="n"/>
-      <c r="C25" s="83" t="n"/>
-      <c r="D25" s="83" t="n"/>
-      <c r="E25" s="83" t="n"/>
-      <c r="F25" s="83" t="n"/>
-      <c r="G25" s="83" t="n"/>
-      <c r="H25" s="84" t="n"/>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="48">
-      <c r="A26" s="82" t="inlineStr">
+      <c r="B26" s="83" t="n"/>
+      <c r="C26" s="83" t="n"/>
+      <c r="D26" s="83" t="n"/>
+      <c r="E26" s="83" t="n"/>
+      <c r="F26" s="83" t="n"/>
+      <c r="G26" s="83" t="n"/>
+      <c r="H26" s="84" t="n"/>
+    </row>
+    <row r="27" ht="15" customHeight="1" s="48">
+      <c r="A27" s="82" t="inlineStr">
         <is>
           <t>SCARA</t>
         </is>
       </c>
-      <c r="B26" s="86" t="n"/>
-      <c r="C26" s="86" t="n"/>
-      <c r="D26" s="86" t="n"/>
-      <c r="E26" s="86" t="n"/>
-      <c r="F26" s="86" t="n"/>
-      <c r="G26" s="86" t="n"/>
-      <c r="H26" s="87" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="48">
-      <c r="A27" s="72" t="inlineStr">
-        <is>
-          <t>P16</t>
-        </is>
-      </c>
-      <c r="B27" s="95" t="inlineStr">
-        <is>
-          <t>Coarde scara</t>
-        </is>
-      </c>
-      <c r="C27" s="95" t="inlineStr">
-        <is>
-          <t>60x140</t>
-        </is>
-      </c>
-      <c r="D27" s="97" t="inlineStr">
-        <is>
-          <t>~3000</t>
-        </is>
-      </c>
-      <c r="E27" s="97" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F27" s="74" t="inlineStr">
-        <is>
-          <t>NOU</t>
-        </is>
-      </c>
-      <c r="G27" s="94" t="inlineStr">
-        <is>
-          <t>oricare</t>
-        </is>
-      </c>
-      <c r="H27" s="95" t="inlineStr">
-        <is>
-          <t>Panta de la sol/balcon la podea.</t>
-        </is>
-      </c>
+      <c r="B27" s="86" t="n"/>
+      <c r="C27" s="86" t="n"/>
+      <c r="D27" s="86" t="n"/>
+      <c r="E27" s="86" t="n"/>
+      <c r="F27" s="86" t="n"/>
+      <c r="G27" s="86" t="n"/>
+      <c r="H27" s="87" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="48">
       <c r="A28" s="72" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B28" s="95" t="inlineStr">
         <is>
-          <t>Trepte</t>
+          <t>Coarde scara</t>
         </is>
       </c>
       <c r="C28" s="95" t="inlineStr">
         <is>
-          <t>45x190</t>
+          <t>60x140</t>
         </is>
       </c>
       <c r="D28" s="97" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>~3000</t>
         </is>
       </c>
       <c r="E28" s="97" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F28" s="74" t="inlineStr">
@@ -3082,164 +3082,164 @@
       </c>
       <c r="H28" s="95" t="inlineStr">
         <is>
-          <t>Trepte solide.</t>
+          <t>Panta de la sol/balcon la podea.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1" s="48">
       <c r="A29" s="72" t="inlineStr">
         <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="B29" s="95" t="inlineStr">
+        <is>
+          <t>Trepte</t>
+        </is>
+      </c>
+      <c r="C29" s="95" t="inlineStr">
+        <is>
+          <t>45x190</t>
+        </is>
+      </c>
+      <c r="D29" s="97" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="E29" s="97" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F29" s="74" t="inlineStr">
+        <is>
+          <t>NOU</t>
+        </is>
+      </c>
+      <c r="G29" s="94" t="inlineStr">
+        <is>
+          <t>oricare</t>
+        </is>
+      </c>
+      <c r="H29" s="95" t="inlineStr">
+        <is>
+          <t>Trepte solide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="21.75" customHeight="1" s="48">
+      <c r="A30" s="72" t="inlineStr">
+        <is>
           <t>P18</t>
         </is>
       </c>
-      <c r="B29" s="83" t="n"/>
-      <c r="C29" s="83" t="n"/>
-      <c r="D29" s="83" t="n"/>
-      <c r="E29" s="83" t="n"/>
-      <c r="F29" s="83" t="n"/>
-      <c r="G29" s="83" t="n"/>
-      <c r="H29" s="84" t="n"/>
-    </row>
-    <row r="30" ht="21.75" customHeight="1" s="48">
-      <c r="A30" s="82" t="inlineStr">
+      <c r="B30" s="83" t="n"/>
+      <c r="C30" s="83" t="n"/>
+      <c r="D30" s="83" t="n"/>
+      <c r="E30" s="83" t="n"/>
+      <c r="F30" s="83" t="n"/>
+      <c r="G30" s="83" t="n"/>
+      <c r="H30" s="84" t="n"/>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="48">
+      <c r="A31" s="82" t="inlineStr">
         <is>
           <t>MASA-COPAC</t>
         </is>
       </c>
-      <c r="B30" s="86" t="n"/>
-      <c r="C30" s="86" t="n"/>
-      <c r="D30" s="86" t="n"/>
-      <c r="E30" s="86" t="n"/>
-      <c r="F30" s="86" t="n"/>
-      <c r="G30" s="86" t="n"/>
-      <c r="H30" s="87" t="n"/>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="48">
-      <c r="A31" s="72" t="inlineStr">
-        <is>
-          <t>P19</t>
-        </is>
-      </c>
-      <c r="B31" s="95" t="inlineStr">
-        <is>
-          <t>Blat masa</t>
-        </is>
-      </c>
-      <c r="C31" s="95" t="inlineStr">
-        <is>
-          <t>panou / scandura lipita ~Ø500</t>
-        </is>
-      </c>
-      <c r="D31" s="97" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E31" s="97" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F31" s="74" t="inlineStr">
-        <is>
-          <t>NOU/offcut</t>
-        </is>
-      </c>
-      <c r="G31" s="94" t="inlineStr">
-        <is>
-          <t>oricare</t>
-        </is>
-      </c>
-      <c r="H31" s="95" t="inlineStr">
-        <is>
-          <t>Fixat de PODEA prin cadru propriu, NU de copac. Capat trunchi tesit+capac.</t>
-        </is>
-      </c>
+      <c r="B31" s="86" t="n"/>
+      <c r="C31" s="86" t="n"/>
+      <c r="D31" s="86" t="n"/>
+      <c r="E31" s="86" t="n"/>
+      <c r="F31" s="86" t="n"/>
+      <c r="G31" s="86" t="n"/>
+      <c r="H31" s="87" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1" s="48">
       <c r="A32" s="72" t="inlineStr">
         <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="B32" s="95" t="inlineStr">
+        <is>
+          <t>Blat masa</t>
+        </is>
+      </c>
+      <c r="C32" s="95" t="inlineStr">
+        <is>
+          <t>panou / scandura lipita ~Ø500</t>
+        </is>
+      </c>
+      <c r="D32" s="97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E32" s="97" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F32" s="74" t="inlineStr">
+        <is>
+          <t>NOU/offcut</t>
+        </is>
+      </c>
+      <c r="G32" s="94" t="inlineStr">
+        <is>
+          <t>oricare</t>
+        </is>
+      </c>
+      <c r="H32" s="95" t="inlineStr">
+        <is>
+          <t>Fixat de PODEA prin cadru propriu, NU de copac. Capat trunchi tesit+capac.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="48">
+      <c r="A33" s="72" t="inlineStr">
+        <is>
           <t>P20</t>
         </is>
       </c>
-      <c r="B32" s="83" t="n"/>
-      <c r="C32" s="83" t="n"/>
-      <c r="D32" s="83" t="n"/>
-      <c r="E32" s="83" t="n"/>
-      <c r="F32" s="83" t="n"/>
-      <c r="G32" s="83" t="n"/>
-      <c r="H32" s="84" t="n"/>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="48">
-      <c r="A33" s="82" t="inlineStr">
+      <c r="B33" s="83" t="n"/>
+      <c r="C33" s="83" t="n"/>
+      <c r="D33" s="83" t="n"/>
+      <c r="E33" s="83" t="n"/>
+      <c r="F33" s="83" t="n"/>
+      <c r="G33" s="83" t="n"/>
+      <c r="H33" s="84" t="n"/>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="48">
+      <c r="A34" s="82" t="inlineStr">
         <is>
           <t>FERONERIE</t>
         </is>
       </c>
-      <c r="B33" s="86" t="n"/>
-      <c r="C33" s="86" t="n"/>
-      <c r="D33" s="86" t="n"/>
-      <c r="E33" s="86" t="n"/>
-      <c r="F33" s="86" t="n"/>
-      <c r="G33" s="86" t="n"/>
-      <c r="H33" s="87" t="n"/>
-    </row>
-    <row r="34" ht="15" customHeight="1" s="48">
-      <c r="A34" s="72" t="inlineStr">
-        <is>
-          <t>P21</t>
-        </is>
-      </c>
-      <c r="B34" s="95" t="inlineStr">
-        <is>
-          <t>Buloane M12 + piulite + saibe</t>
-        </is>
-      </c>
-      <c r="C34" s="95" t="inlineStr">
-        <is>
-          <t>M12: 8x120 baza + tija M12 polita</t>
-        </is>
-      </c>
-      <c r="D34" s="97" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E34" s="97" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="F34" s="74" t="inlineStr">
-        <is>
-          <t>NOU</t>
-        </is>
-      </c>
-      <c r="G34" s="94" t="inlineStr">
-        <is>
-          <t>oricare</t>
-        </is>
-      </c>
-      <c r="H34" s="95" t="inlineStr">
-        <is>
-          <t>Baza papuc: 8x M12x120. Polita: tija filetata M12 1m taiata in 4x ~220 mm (cod 12130958) + piulite + saibe.</t>
-        </is>
-      </c>
+      <c r="B34" s="86" t="n"/>
+      <c r="C34" s="86" t="n"/>
+      <c r="D34" s="86" t="n"/>
+      <c r="E34" s="86" t="n"/>
+      <c r="F34" s="86" t="n"/>
+      <c r="G34" s="86" t="n"/>
+      <c r="H34" s="87" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="48">
       <c r="A35" s="72" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="B35" s="95" t="inlineStr">
         <is>
-          <t>Coltare metalice C1 + C2</t>
+          <t>Buloane M12 + piulite + saibe</t>
         </is>
       </c>
       <c r="C35" s="95" t="inlineStr">
         <is>
-          <t>C1 100x100x90 (4) + C2 90x90x65 (14)</t>
+          <t>M12: 8x120 baza + tija M12 polita</t>
         </is>
       </c>
       <c r="D35" s="97" t="inlineStr">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="E35" s="97" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F35" s="74" t="inlineStr">
@@ -3259,29 +3259,29 @@
       </c>
       <c r="G35" s="94" t="inlineStr">
         <is>
-          <t>Hornbach</t>
+          <t>oricare</t>
         </is>
       </c>
       <c r="H35" s="95" t="inlineStr">
         <is>
-          <t>C1 grinda fata-&gt;stalp (4); C2 joiste anti-ridicare (14).</t>
+          <t>Baza papuc: 8x M12x120. Polita: tija filetata M12 1m taiata in 4x ~220 mm (cod 12130958) + piulite + saibe.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="48">
       <c r="A36" s="72" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="B36" s="95" t="inlineStr">
         <is>
-          <t>Suruburi structurale Heco</t>
+          <t>Coltare metalice C1 + C2</t>
         </is>
       </c>
       <c r="C36" s="95" t="inlineStr">
         <is>
-          <t>Heco 8x200, pac 100</t>
+          <t>C1 100x100x90 (4) + C2 90x90x65 (14)</t>
         </is>
       </c>
       <c r="D36" s="97" t="inlineStr">
@@ -3291,7 +3291,7 @@
       </c>
       <c r="E36" s="97" t="inlineStr">
         <is>
-          <t>1 pac</t>
+          <t>18</t>
         </is>
       </c>
       <c r="F36" s="74" t="inlineStr">
@@ -3306,94 +3306,94 @@
       </c>
       <c r="H36" s="95" t="inlineStr">
         <is>
-          <t>Imbinari lemn-lemn (cod 10434633). Fara pre-gaurire.</t>
+          <t>C1 grinda fata-&gt;stalp (4); C2 joiste anti-ridicare (14).</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1" s="48">
       <c r="A37" s="72" t="inlineStr">
         <is>
+          <t>P23</t>
+        </is>
+      </c>
+      <c r="B37" s="95" t="inlineStr">
+        <is>
+          <t>Suruburi structurale Heco</t>
+        </is>
+      </c>
+      <c r="C37" s="95" t="inlineStr">
+        <is>
+          <t>Heco 8x200, pac 100</t>
+        </is>
+      </c>
+      <c r="D37" s="97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E37" s="97" t="inlineStr">
+        <is>
+          <t>1 pac</t>
+        </is>
+      </c>
+      <c r="F37" s="74" t="inlineStr">
+        <is>
+          <t>NOU</t>
+        </is>
+      </c>
+      <c r="G37" s="94" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="H37" s="95" t="inlineStr">
+        <is>
+          <t>Imbinari lemn-lemn (cod 10434633). Fara pre-gaurire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15" customHeight="1" s="48">
+      <c r="A38" s="72" t="inlineStr">
+        <is>
           <t>P24</t>
         </is>
       </c>
-      <c r="B37" s="83" t="n"/>
-      <c r="C37" s="83" t="n"/>
-      <c r="D37" s="83" t="n"/>
-      <c r="E37" s="83" t="n"/>
-      <c r="F37" s="83" t="n"/>
-      <c r="G37" s="83" t="n"/>
-      <c r="H37" s="84" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1" s="48">
-      <c r="A38" s="82" t="inlineStr">
+      <c r="B38" s="83" t="n"/>
+      <c r="C38" s="83" t="n"/>
+      <c r="D38" s="83" t="n"/>
+      <c r="E38" s="83" t="n"/>
+      <c r="F38" s="83" t="n"/>
+      <c r="G38" s="83" t="n"/>
+      <c r="H38" s="84" t="n"/>
+    </row>
+    <row r="39" ht="15" customHeight="1" s="48">
+      <c r="A39" s="82" t="inlineStr">
         <is>
           <t>FINISAJ + SOL</t>
         </is>
       </c>
-      <c r="B38" s="86" t="n"/>
-      <c r="C38" s="86" t="n"/>
-      <c r="D38" s="86" t="n"/>
-      <c r="E38" s="86" t="n"/>
-      <c r="F38" s="86" t="n"/>
-      <c r="G38" s="86" t="n"/>
-      <c r="H38" s="87" t="n"/>
-    </row>
-    <row r="39" ht="15" customHeight="1" s="48">
-      <c r="A39" s="72" t="inlineStr">
-        <is>
-          <t>P25</t>
-        </is>
-      </c>
-      <c r="B39" s="95" t="inlineStr">
-        <is>
-          <t>Grund izolare lemn</t>
-        </is>
-      </c>
-      <c r="C39" s="95" t="inlineStr">
-        <is>
-          <t>2,5 l</t>
-        </is>
-      </c>
-      <c r="D39" s="97" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E39" s="97" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F39" s="74" t="inlineStr">
-        <is>
-          <t>NOU</t>
-        </is>
-      </c>
-      <c r="G39" s="94" t="inlineStr">
-        <is>
-          <t>Hornbach</t>
-        </is>
-      </c>
-      <c r="H39" s="95" t="inlineStr">
-        <is>
-          <t>Strat de baza.</t>
-        </is>
-      </c>
+      <c r="B39" s="86" t="n"/>
+      <c r="C39" s="86" t="n"/>
+      <c r="D39" s="86" t="n"/>
+      <c r="E39" s="86" t="n"/>
+      <c r="F39" s="86" t="n"/>
+      <c r="G39" s="86" t="n"/>
+      <c r="H39" s="87" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="48">
       <c r="A40" s="72" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="B40" s="95" t="inlineStr">
         <is>
-          <t>Vopsea protectie exterior</t>
+          <t>Grund izolare lemn</t>
         </is>
       </c>
       <c r="C40" s="95" t="inlineStr">
         <is>
-          <t>6 l</t>
+          <t>2,5 l</t>
         </is>
       </c>
       <c r="D40" s="97" t="inlineStr">
@@ -3403,7 +3403,7 @@
       </c>
       <c r="E40" s="97" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F40" s="74" t="inlineStr">
@@ -3418,62 +3418,104 @@
       </c>
       <c r="H40" s="95" t="inlineStr">
         <is>
-          <t>Wetterschutz sau similar.</t>
+          <t>Strat de baza.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="48">
       <c r="A41" s="72" t="inlineStr">
         <is>
+          <t>P26</t>
+        </is>
+      </c>
+      <c r="B41" s="95" t="inlineStr">
+        <is>
+          <t>Vopsea protectie exterior</t>
+        </is>
+      </c>
+      <c r="C41" s="95" t="inlineStr">
+        <is>
+          <t>6 l</t>
+        </is>
+      </c>
+      <c r="D41" s="97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E41" s="97" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F41" s="74" t="inlineStr">
+        <is>
+          <t>NOU</t>
+        </is>
+      </c>
+      <c r="G41" s="94" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="H41" s="95" t="inlineStr">
+        <is>
+          <t>Wetterschutz sau similar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="15" customHeight="1" s="48">
+      <c r="A42" s="72" t="inlineStr">
+        <is>
           <t>P27</t>
         </is>
       </c>
-      <c r="B41" s="95" t="inlineStr">
+      <c r="B42" s="95" t="inlineStr">
         <is>
           <t>Sol moale sub platforma</t>
         </is>
       </c>
-      <c r="C41" s="95" t="inlineStr">
+      <c r="C42" s="95" t="inlineStr">
         <is>
           <t>scoarta / nisip</t>
         </is>
       </c>
-      <c r="D41" s="97" t="inlineStr">
+      <c r="D42" s="97" t="inlineStr">
         <is>
           <t>~5 m²</t>
         </is>
       </c>
-      <c r="E41" s="97" t="inlineStr">
+      <c r="E42" s="97" t="inlineStr">
         <is>
           <t>1 lot</t>
         </is>
       </c>
-      <c r="F41" s="74" t="inlineStr">
+      <c r="F42" s="74" t="inlineStr">
         <is>
           <t>NOU</t>
         </is>
       </c>
-      <c r="G41" s="94" t="inlineStr">
+      <c r="G42" s="94" t="inlineStr">
         <is>
           <t>oricare</t>
         </is>
       </c>
-      <c r="H41" s="95" t="inlineStr">
+      <c r="H42" s="95" t="inlineStr">
         <is>
           <t>Amortizare cadere. NU beton/piatra dedesubt.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="15" customHeight="1" s="48"/>
-    <row r="43" ht="15" customHeight="1" s="48">
-      <c r="A43" s="76" t="inlineStr">
+    <row r="43" ht="15" customHeight="1" s="48"/>
+    <row r="44" ht="15" customHeight="1" s="48">
+      <c r="A44" s="76" t="inlineStr">
         <is>
           <t>Note:</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="15" customHeight="1" s="48">
-      <c r="A44" s="80" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="80" t="inlineStr">
         <is>
           <t>Ancorele de fundatie sunt deja in pamant → nu cumparam suporti de stalp. Cantitatile de dusumea/sipci/placaj sunt estimate; le confirmam la magazin dupa sectiunile finale de scandura.</t>
         </is>
@@ -3481,18 +3523,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A30:H30"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A29:H29"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A44:H44"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3506,7 +3548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="47" min="1" max="1"/>
@@ -3890,119 +3932,119 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="48">
-      <c r="A13" s="82" t="inlineStr">
+    <row r="13" ht="15" customHeight="1" s="48">
+      <c r="A13" s="94" t="inlineStr">
+        <is>
+          <t>Grinzi</t>
+        </is>
+      </c>
+      <c r="B13" s="95" t="inlineStr">
+        <is>
+          <t>Talpic sub polita (din offcut 100×100)</t>
+        </is>
+      </c>
+      <c r="C13" s="94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D13" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="94" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="G13" s="62">
+        <f>IF(AND(D13&lt;&gt;"",E13&lt;&gt;""),D13*E13,"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="95" t="inlineStr">
+        <is>
+          <t>Bloc ~180 sub fiecare polita: duce greutatea in compresiune. M12 = pozitie + anti-smulgere.</t>
+        </is>
+      </c>
+      <c r="I13" s="96" t="inlineStr">
+        <is>
+          <t>OFFCUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="48">
+      <c r="A14" s="82" t="inlineStr">
         <is>
           <t>PODEA</t>
         </is>
       </c>
-      <c r="B13" s="83" t="n"/>
-      <c r="C13" s="83" t="n"/>
-      <c r="D13" s="83" t="n"/>
-      <c r="E13" s="83" t="n"/>
-      <c r="F13" s="83" t="n"/>
-      <c r="G13" s="83" t="n"/>
-      <c r="H13" s="83" t="n"/>
-      <c r="I13" s="84" t="n"/>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="48">
-      <c r="A14" s="94" t="inlineStr">
+      <c r="B14" s="83" t="n"/>
+      <c r="C14" s="83" t="n"/>
+      <c r="D14" s="83" t="n"/>
+      <c r="E14" s="83" t="n"/>
+      <c r="F14" s="83" t="n"/>
+      <c r="G14" s="83" t="n"/>
+      <c r="H14" s="83" t="n"/>
+      <c r="I14" s="84" t="n"/>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="48">
+      <c r="A15" s="94" t="inlineStr">
         <is>
           <t>Dusumea</t>
         </is>
       </c>
-      <c r="B14" s="95" t="inlineStr">
+      <c r="B15" s="95" t="inlineStr">
         <is>
           <t>Lemn terasa larice Konsta 28×145×3000</t>
         </is>
       </c>
-      <c r="C14" s="94" t="inlineStr">
+      <c r="C15" s="94" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="D14" s="88" t="n">
+      <c r="D15" s="88" t="n">
         <v>79.90000000000001</v>
       </c>
-      <c r="E14" s="60" t="n">
+      <c r="E15" s="60" t="n">
         <v>17</v>
       </c>
-      <c r="F14" s="94" t="inlineStr">
+      <c r="F15" s="94" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
       </c>
-      <c r="G14" s="62">
-        <f>IF(AND(D14&lt;&gt;"",E14&lt;&gt;""),D14*E14,"")</f>
-        <v/>
-      </c>
-      <c r="H14" s="95" t="inlineStr">
+      <c r="G15" s="62">
+        <f>IF(AND(D15&lt;&gt;"",E15&lt;&gt;""),D15*E15,"")</f>
+        <v/>
+      </c>
+      <c r="H15" s="95" t="inlineStr">
         <is>
           <t>Dusumea premium 28mm</t>
         </is>
       </c>
-      <c r="I14" s="74" t="inlineStr">
+      <c r="I15" s="74" t="inlineStr">
         <is>
           <t>De cumparat</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="48">
-      <c r="A15" s="82" t="inlineStr">
+    <row r="16" ht="15" customHeight="1" s="48">
+      <c r="A16" s="82" t="inlineStr">
         <is>
           <t>IMBINARI</t>
         </is>
       </c>
-      <c r="B15" s="83" t="n"/>
-      <c r="C15" s="83" t="n"/>
-      <c r="D15" s="83" t="n"/>
-      <c r="E15" s="83" t="n"/>
-      <c r="F15" s="83" t="n"/>
-      <c r="G15" s="83" t="n"/>
-      <c r="H15" s="83" t="n"/>
-      <c r="I15" s="84" t="n"/>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="48">
-      <c r="A16" s="94" t="inlineStr">
-        <is>
-          <t>Conectori</t>
-        </is>
-      </c>
-      <c r="B16" s="95" t="inlineStr">
-        <is>
-          <t>Coltar rigidizat Alberts 100×100×90×3</t>
-        </is>
-      </c>
-      <c r="C16" s="94" t="inlineStr">
-        <is>
-          <t>Hornbach</t>
-        </is>
-      </c>
-      <c r="D16" s="88" t="n">
-        <v>9.35</v>
-      </c>
-      <c r="E16" s="60" t="n">
-        <v>4</v>
-      </c>
-      <c r="F16" s="94" t="inlineStr">
-        <is>
-          <t>buc</t>
-        </is>
-      </c>
-      <c r="G16" s="62">
-        <f>IF(AND(D16&lt;&gt;"",E16&lt;&gt;""),D16*E16,"")</f>
-        <v/>
-      </c>
-      <c r="H16" s="95" t="inlineStr">
-        <is>
-          <t>Grinda FATA → stalp (pe varf)</t>
-        </is>
-      </c>
-      <c r="I16" s="74" t="inlineStr">
-        <is>
-          <t>De cumparat</t>
-        </is>
-      </c>
+      <c r="B16" s="83" t="n"/>
+      <c r="C16" s="83" t="n"/>
+      <c r="D16" s="83" t="n"/>
+      <c r="E16" s="83" t="n"/>
+      <c r="F16" s="83" t="n"/>
+      <c r="G16" s="83" t="n"/>
+      <c r="H16" s="83" t="n"/>
+      <c r="I16" s="84" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="48">
       <c r="A17" s="94" t="inlineStr">
@@ -4012,7 +4054,7 @@
       </c>
       <c r="B17" s="95" t="inlineStr">
         <is>
-          <t>Coltar rigidizat Alberts 90×90×65</t>
+          <t>Coltar rigidizat Alberts 100×100×90×3</t>
         </is>
       </c>
       <c r="C17" s="94" t="inlineStr">
@@ -4021,10 +4063,10 @@
         </is>
       </c>
       <c r="D17" s="88" t="n">
-        <v>4.83</v>
+        <v>9.35</v>
       </c>
       <c r="E17" s="60" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="F17" s="94" t="inlineStr">
         <is>
@@ -4037,7 +4079,7 @@
       </c>
       <c r="H17" s="95" t="inlineStr">
         <is>
-          <t>Joiste → grinda + grinda spate, anti-ridicare (12+2=14)</t>
+          <t>Grinda FATA → stalp (pe varf)</t>
         </is>
       </c>
       <c r="I17" s="74" t="inlineStr">
@@ -4049,12 +4091,12 @@
     <row r="18" ht="15" customHeight="1" s="48">
       <c r="A18" s="94" t="inlineStr">
         <is>
-          <t>Suruburi</t>
+          <t>Conectori</t>
         </is>
       </c>
       <c r="B18" s="95" t="inlineStr">
         <is>
-          <t>Heco Topix-Plus 8×200 Torx (100 buc)</t>
+          <t>Coltar rigidizat Alberts 90×90×65</t>
         </is>
       </c>
       <c r="C18" s="94" t="inlineStr">
@@ -4063,14 +4105,14 @@
         </is>
       </c>
       <c r="D18" s="88" t="n">
-        <v>369.1</v>
+        <v>4.83</v>
       </c>
       <c r="E18" s="60" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F18" s="94" t="inlineStr">
         <is>
-          <t>pac</t>
+          <t>buc</t>
         </is>
       </c>
       <c r="G18" s="62">
@@ -4079,7 +4121,7 @@
       </c>
       <c r="H18" s="95" t="inlineStr">
         <is>
-          <t>Imbinari structurale, fara pre-gaurire</t>
+          <t>Joiste → grinda + grinda spate, anti-ridicare (12+2=14)</t>
         </is>
       </c>
       <c r="I18" s="74" t="inlineStr">
@@ -4096,7 +4138,7 @@
       </c>
       <c r="B19" s="95" t="inlineStr">
         <is>
-          <t>Heco Topix-Plus 6x100 zincat (100 buc)</t>
+          <t>Heco Topix-Plus 8×200 Torx (100 buc)</t>
         </is>
       </c>
       <c r="C19" s="94" t="inlineStr">
@@ -4105,7 +4147,7 @@
         </is>
       </c>
       <c r="D19" s="88" t="n">
-        <v>94.87</v>
+        <v>369.1</v>
       </c>
       <c r="E19" s="60" t="n">
         <v>1</v>
@@ -4121,7 +4163,7 @@
       </c>
       <c r="H19" s="95" t="inlineStr">
         <is>
-          <t>Coltare, conectori</t>
+          <t>Imbinari structurale, fara pre-gaurire</t>
         </is>
       </c>
       <c r="I19" s="74" t="inlineStr">
@@ -4138,7 +4180,7 @@
       </c>
       <c r="B20" s="95" t="inlineStr">
         <is>
-          <t>Heco Topix-Plus 6×80 (100 buc)</t>
+          <t>Heco Topix-Plus 6x100 zincat (100 buc)</t>
         </is>
       </c>
       <c r="C20" s="94" t="inlineStr">
@@ -4147,7 +4189,7 @@
         </is>
       </c>
       <c r="D20" s="88" t="n">
-        <v>72.8</v>
+        <v>94.87</v>
       </c>
       <c r="E20" s="60" t="n">
         <v>1</v>
@@ -4163,7 +4205,7 @@
       </c>
       <c r="H20" s="95" t="inlineStr">
         <is>
-          <t>Blocaje, prinderi generale</t>
+          <t>Coltare, conectori</t>
         </is>
       </c>
       <c r="I20" s="74" t="inlineStr">
@@ -4180,7 +4222,7 @@
       </c>
       <c r="B21" s="95" t="inlineStr">
         <is>
-          <t>Suruburi inox A2 5x60 dusumea (100 buc)</t>
+          <t>Heco Topix-Plus 6×80 (100 buc)</t>
         </is>
       </c>
       <c r="C21" s="94" t="inlineStr">
@@ -4189,10 +4231,10 @@
         </is>
       </c>
       <c r="D21" s="88" t="n">
-        <v>55.82</v>
+        <v>72.8</v>
       </c>
       <c r="E21" s="60" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F21" s="94" t="inlineStr">
         <is>
@@ -4205,71 +4247,71 @@
       </c>
       <c r="H21" s="95" t="inlineStr">
         <is>
+          <t>Blocaje, prinderi generale</t>
+        </is>
+      </c>
+      <c r="I21" s="74" t="inlineStr">
+        <is>
+          <t>De cumparat</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="48">
+      <c r="A22" s="94" t="inlineStr">
+        <is>
+          <t>Suruburi</t>
+        </is>
+      </c>
+      <c r="B22" s="95" t="inlineStr">
+        <is>
+          <t>Suruburi inox A2 5x60 dusumea (100 buc)</t>
+        </is>
+      </c>
+      <c r="C22" s="94" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="D22" s="88" t="n">
+        <v>55.82</v>
+      </c>
+      <c r="E22" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="F22" s="94" t="inlineStr">
+        <is>
+          <t>pac</t>
+        </is>
+      </c>
+      <c r="G22" s="62">
+        <f>IF(AND(D22&lt;&gt;"",E22&lt;&gt;""),D22*E22,"")</f>
+        <v/>
+      </c>
+      <c r="H22" s="95" t="inlineStr">
+        <is>
           <t>Prindere dusumea larice</t>
         </is>
       </c>
-      <c r="I21" s="72" t="inlineStr">
+      <c r="I22" s="72" t="inlineStr">
         <is>
           <t>De cumparat</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="48">
-      <c r="A22" s="82" t="inlineStr">
+    <row r="23" ht="15" customHeight="1" s="48">
+      <c r="A23" s="82" t="inlineStr">
         <is>
           <t>SCARA</t>
         </is>
       </c>
-      <c r="B22" s="83" t="n"/>
-      <c r="C22" s="83" t="n"/>
-      <c r="D22" s="83" t="n"/>
-      <c r="E22" s="83" t="n"/>
-      <c r="F22" s="83" t="n"/>
-      <c r="G22" s="83" t="n"/>
-      <c r="H22" s="83" t="n"/>
-      <c r="I22" s="84" t="n"/>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="48">
-      <c r="A23" s="94" t="inlineStr">
-        <is>
-          <t>Scara</t>
-        </is>
-      </c>
-      <c r="B23" s="95" t="inlineStr">
-        <is>
-          <t>Coarde scara KVH 60×140×3000</t>
-        </is>
-      </c>
-      <c r="C23" s="94" t="inlineStr">
-        <is>
-          <t>Hornbach</t>
-        </is>
-      </c>
-      <c r="D23" s="88" t="n">
-        <v>130</v>
-      </c>
-      <c r="E23" s="60" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" s="94" t="inlineStr">
-        <is>
-          <t>buc</t>
-        </is>
-      </c>
-      <c r="G23" s="62">
-        <f>IF(AND(D23&lt;&gt;"",E23&lt;&gt;""),D23*E23,"")</f>
-        <v/>
-      </c>
-      <c r="H23" s="95" t="inlineStr">
-        <is>
-          <t>Cele 2 grinzi inclinate (~2,9 m)</t>
-        </is>
-      </c>
-      <c r="I23" s="72" t="inlineStr">
-        <is>
-          <t>De cumparat (est.)</t>
-        </is>
-      </c>
+      <c r="B23" s="83" t="n"/>
+      <c r="C23" s="83" t="n"/>
+      <c r="D23" s="83" t="n"/>
+      <c r="E23" s="83" t="n"/>
+      <c r="F23" s="83" t="n"/>
+      <c r="G23" s="83" t="n"/>
+      <c r="H23" s="83" t="n"/>
+      <c r="I23" s="84" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="48">
       <c r="A24" s="94" t="inlineStr">
@@ -4279,7 +4321,7 @@
       </c>
       <c r="B24" s="95" t="inlineStr">
         <is>
-          <t>Trepte larice/dulap 45×190 ~600 mm</t>
+          <t>Coarde scara KVH 60×140×3000</t>
         </is>
       </c>
       <c r="C24" s="94" t="inlineStr">
@@ -4288,10 +4330,10 @@
         </is>
       </c>
       <c r="D24" s="88" t="n">
-        <v>25</v>
+        <v>130</v>
       </c>
       <c r="E24" s="60" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F24" s="94" t="inlineStr">
         <is>
@@ -4304,7 +4346,7 @@
       </c>
       <c r="H24" s="95" t="inlineStr">
         <is>
-          <t>10 trepte (11 niveluri) (riser 200, calcai 190)</t>
+          <t>Cele 2 grinzi inclinate (~2,9 m)</t>
         </is>
       </c>
       <c r="I24" s="72" t="inlineStr">
@@ -4321,7 +4363,7 @@
       </c>
       <c r="B25" s="95" t="inlineStr">
         <is>
-          <t>Mana curenta + stalpisori (lemn)</t>
+          <t>Trepte larice/dulap 45×190 ~600 mm</t>
         </is>
       </c>
       <c r="C25" s="94" t="inlineStr">
@@ -4330,14 +4372,14 @@
         </is>
       </c>
       <c r="D25" s="88" t="n">
-        <v>120</v>
+        <v>25</v>
       </c>
       <c r="E25" s="60" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F25" s="94" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>buc</t>
         </is>
       </c>
       <c r="G25" s="62">
@@ -4346,7 +4388,7 @@
       </c>
       <c r="H25" s="95" t="inlineStr">
         <is>
-          <t>Pe ambele parti</t>
+          <t>10 trepte (11 niveluri) (riser 200, calcai 190)</t>
         </is>
       </c>
       <c r="I25" s="72" t="inlineStr">
@@ -4363,7 +4405,7 @@
       </c>
       <c r="B26" s="95" t="inlineStr">
         <is>
-          <t>Feronerie scara (coltare + Heco + 2× M10)</t>
+          <t>Mana curenta + stalpisori (lemn)</t>
         </is>
       </c>
       <c r="C26" s="94" t="inlineStr">
@@ -4372,7 +4414,7 @@
         </is>
       </c>
       <c r="D26" s="88" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="E26" s="60" t="n">
         <v>1</v>
@@ -4388,7 +4430,7 @@
       </c>
       <c r="H26" s="95" t="inlineStr">
         <is>
-          <t>Prindere de platforma + trepte</t>
+          <t>Pe ambele parti</t>
         </is>
       </c>
       <c r="I26" s="72" t="inlineStr">
@@ -4405,7 +4447,7 @@
       </c>
       <c r="B27" s="95" t="inlineStr">
         <is>
-          <t>Dala/paver baza scara</t>
+          <t>Feronerie scara (coltare + Heco + 2× M10)</t>
         </is>
       </c>
       <c r="C27" s="94" t="inlineStr">
@@ -4414,14 +4456,14 @@
         </is>
       </c>
       <c r="D27" s="88" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="E27" s="60" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="94" t="inlineStr">
         <is>
-          <t>buc</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G27" s="62">
@@ -4430,71 +4472,71 @@
       </c>
       <c r="H27" s="95" t="inlineStr">
         <is>
+          <t>Prindere de platforma + trepte</t>
+        </is>
+      </c>
+      <c r="I27" s="72" t="inlineStr">
+        <is>
+          <t>De cumparat (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16.5" customHeight="1" s="48">
+      <c r="A28" s="94" t="inlineStr">
+        <is>
+          <t>Scara</t>
+        </is>
+      </c>
+      <c r="B28" s="95" t="inlineStr">
+        <is>
+          <t>Dala/paver baza scara</t>
+        </is>
+      </c>
+      <c r="C28" s="94" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="D28" s="88" t="n">
+        <v>20</v>
+      </c>
+      <c r="E28" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="94" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="G28" s="62">
+        <f>IF(AND(D28&lt;&gt;"",E28&lt;&gt;""),D28*E28,"")</f>
+        <v/>
+      </c>
+      <c r="H28" s="95" t="inlineStr">
+        <is>
           <t>Sub coarde, sa nu stea in pamant</t>
         </is>
       </c>
-      <c r="I27" s="72" t="inlineStr">
+      <c r="I28" s="72" t="inlineStr">
         <is>
           <t>De cumparat (est.)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="48">
-      <c r="A28" s="82" t="inlineStr">
+    <row r="29" ht="15" customHeight="1" s="48">
+      <c r="A29" s="82" t="inlineStr">
         <is>
           <t>FINISAJ</t>
         </is>
       </c>
-      <c r="B28" s="83" t="n"/>
-      <c r="C28" s="83" t="n"/>
-      <c r="D28" s="83" t="n"/>
-      <c r="E28" s="83" t="n"/>
-      <c r="F28" s="83" t="n"/>
-      <c r="G28" s="83" t="n"/>
-      <c r="H28" s="83" t="n"/>
-      <c r="I28" s="84" t="n"/>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="48">
-      <c r="A29" s="94" t="inlineStr">
-        <is>
-          <t>Finisaj</t>
-        </is>
-      </c>
-      <c r="B29" s="95" t="inlineStr">
-        <is>
-          <t>Ulei lemn tec Hornbach Plus 2,5 l</t>
-        </is>
-      </c>
-      <c r="C29" s="94" t="inlineStr">
-        <is>
-          <t>Hornbach</t>
-        </is>
-      </c>
-      <c r="D29" s="88" t="n">
-        <v>144.39</v>
-      </c>
-      <c r="E29" s="60" t="n">
-        <v>2</v>
-      </c>
-      <c r="F29" s="94" t="inlineStr">
-        <is>
-          <t>buc</t>
-        </is>
-      </c>
-      <c r="G29" s="62">
-        <f>IF(AND(D29&lt;&gt;"",E29&lt;&gt;""),D29*E29,"")</f>
-        <v/>
-      </c>
-      <c r="H29" s="95" t="inlineStr">
-        <is>
-          <t>Dusumea larice + grinzi/scara expuse</t>
-        </is>
-      </c>
-      <c r="I29" s="74" t="inlineStr">
-        <is>
-          <t>De cumparat</t>
-        </is>
-      </c>
+      <c r="B29" s="83" t="n"/>
+      <c r="C29" s="83" t="n"/>
+      <c r="D29" s="83" t="n"/>
+      <c r="E29" s="83" t="n"/>
+      <c r="F29" s="83" t="n"/>
+      <c r="G29" s="83" t="n"/>
+      <c r="H29" s="83" t="n"/>
+      <c r="I29" s="84" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="48">
       <c r="A30" s="94" t="inlineStr">
@@ -4504,7 +4546,7 @@
       </c>
       <c r="B30" s="95" t="inlineStr">
         <is>
-          <t>Grund impregnare Köber 4 L (AVEM)</t>
+          <t>Ulei lemn tec Hornbach Plus 2,5 l</t>
         </is>
       </c>
       <c r="C30" s="94" t="inlineStr">
@@ -4513,10 +4555,10 @@
         </is>
       </c>
       <c r="D30" s="88" t="n">
-        <v>0</v>
+        <v>144.39</v>
       </c>
       <c r="E30" s="60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" s="94" t="inlineStr">
         <is>
@@ -4529,61 +4571,61 @@
       </c>
       <c r="H30" s="95" t="inlineStr">
         <is>
+          <t>Dusumea larice + grinzi/scara expuse</t>
+        </is>
+      </c>
+      <c r="I30" s="74" t="inlineStr">
+        <is>
+          <t>De cumparat</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="94" t="inlineStr">
+        <is>
+          <t>Finisaj</t>
+        </is>
+      </c>
+      <c r="B31" s="95" t="inlineStr">
+        <is>
+          <t>Grund impregnare Köber 4 L (AVEM)</t>
+        </is>
+      </c>
+      <c r="C31" s="94" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="D31" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="94" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="G31" s="62">
+        <f>IF(AND(D31&lt;&gt;"",E31&lt;&gt;""),D31*E31,"")</f>
+        <v/>
+      </c>
+      <c r="H31" s="95" t="inlineStr">
+        <is>
           <t>Stalpi + joiste + capete</t>
         </is>
       </c>
-      <c r="I30" s="72" t="inlineStr">
+      <c r="I31" s="72" t="inlineStr">
         <is>
           <t>AVEM</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="47" t="inlineStr">
-        <is>
-          <t>BALUSTRADA</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="48">
       <c r="A32" s="47" t="inlineStr">
         <is>
-          <t>Balustrada</t>
-        </is>
-      </c>
-      <c r="B32" s="47" t="inlineStr">
-        <is>
-          <t>Stalpisori 58x58, h=100 cm</t>
-        </is>
-      </c>
-      <c r="C32" s="47" t="inlineStr">
-        <is>
-          <t>Hornbach</t>
-        </is>
-      </c>
-      <c r="D32" s="47" t="n">
-        <v>60.91</v>
-      </c>
-      <c r="E32" s="47" t="n">
-        <v>7</v>
-      </c>
-      <c r="F32" s="47" t="inlineStr">
-        <is>
-          <t>buc</t>
-        </is>
-      </c>
-      <c r="G32" s="47">
-        <f>IF(AND(D32&lt;&gt;"",E32&lt;&gt;""),D32*E32,"")</f>
-        <v/>
-      </c>
-      <c r="H32" s="47" t="inlineStr">
-        <is>
-          <t>Stalpisori balustrada, jur-imprejur</t>
-        </is>
-      </c>
-      <c r="I32" s="47" t="inlineStr">
-        <is>
-          <t>De cumparat (est.)</t>
+          <t>BALUSTRADA</t>
         </is>
       </c>
     </row>
@@ -4595,7 +4637,7 @@
       </c>
       <c r="B33" s="47" t="inlineStr">
         <is>
-          <t>Sipci 18x18 umplutura goluri</t>
+          <t>Stalpisori 58x58, h=100 cm</t>
         </is>
       </c>
       <c r="C33" s="47" t="inlineStr">
@@ -4604,10 +4646,10 @@
         </is>
       </c>
       <c r="D33" s="47" t="n">
-        <v>3.3</v>
+        <v>60.91</v>
       </c>
       <c r="E33" s="47" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="F33" s="47" t="inlineStr">
         <is>
@@ -4620,7 +4662,7 @@
       </c>
       <c r="H33" s="47" t="inlineStr">
         <is>
-          <t>Goluri sub 9 cm</t>
+          <t>Stalpisori balustrada, jur-imprejur</t>
         </is>
       </c>
       <c r="I33" s="47" t="inlineStr">
@@ -4637,7 +4679,7 @@
       </c>
       <c r="B34" s="47" t="inlineStr">
         <is>
-          <t>Mana curenta + rigla jos 45x70</t>
+          <t>Sipci 18x18 umplutura goluri</t>
         </is>
       </c>
       <c r="C34" s="47" t="inlineStr">
@@ -4645,22 +4687,24 @@
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="D34" s="47" t="inlineStr">
-        <is>
-          <t>est.</t>
-        </is>
+      <c r="D34" s="47" t="n">
+        <v>3.3</v>
       </c>
       <c r="E34" s="47" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="F34" s="47" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
       </c>
+      <c r="G34" s="47">
+        <f>IF(AND(D34&lt;&gt;"",E34&lt;&gt;""),D34*E34,"")</f>
+        <v/>
+      </c>
       <c r="H34" s="47" t="inlineStr">
         <is>
-          <t>Sus+jos, ~9 m total (3 laturi)</t>
+          <t>Goluri sub 9 cm</t>
         </is>
       </c>
       <c r="I34" s="47" t="inlineStr">
@@ -4677,7 +4721,7 @@
       </c>
       <c r="B35" s="47" t="inlineStr">
         <is>
-          <t>Buloane M10x120 + piulita + saiba</t>
+          <t>Mana curenta + rigla jos 45x70</t>
         </is>
       </c>
       <c r="C35" s="47" t="inlineStr">
@@ -4685,24 +4729,22 @@
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="D35" s="47" t="n">
-        <v>3.5</v>
+      <c r="D35" s="47" t="inlineStr">
+        <is>
+          <t>est.</t>
+        </is>
       </c>
       <c r="E35" s="47" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="F35" s="47" t="inlineStr">
         <is>
           <t>buc</t>
         </is>
       </c>
-      <c r="G35" s="47">
-        <f>IF(AND(D35&lt;&gt;"",E35&lt;&gt;""),D35*E35,"")</f>
-        <v/>
-      </c>
       <c r="H35" s="47" t="inlineStr">
         <is>
-          <t>Prindere stalpisori de cadru</t>
+          <t>Sus+jos, ~9 m total (3 laturi)</t>
         </is>
       </c>
       <c r="I35" s="47" t="inlineStr">
@@ -4719,62 +4761,104 @@
       </c>
       <c r="B36" s="47" t="inlineStr">
         <is>
+          <t>Buloane M10x120 + piulita + saiba</t>
+        </is>
+      </c>
+      <c r="C36" s="47" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="D36" s="47" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E36" s="47" t="n">
+        <v>14</v>
+      </c>
+      <c r="F36" s="47" t="inlineStr">
+        <is>
+          <t>buc</t>
+        </is>
+      </c>
+      <c r="G36" s="47">
+        <f>IF(AND(D36&lt;&gt;"",E36&lt;&gt;""),D36*E36,"")</f>
+        <v/>
+      </c>
+      <c r="H36" s="47" t="inlineStr">
+        <is>
+          <t>Prindere stalpisori de cadru</t>
+        </is>
+      </c>
+      <c r="I36" s="47" t="inlineStr">
+        <is>
+          <t>De cumparat (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="47" t="inlineStr">
+        <is>
+          <t>Balustrada</t>
+        </is>
+      </c>
+      <c r="B37" s="47" t="inlineStr">
+        <is>
           <t>Feronerie poarta (self-close)</t>
         </is>
       </c>
-      <c r="C36" s="47" t="inlineStr">
+      <c r="C37" s="47" t="inlineStr">
         <is>
           <t>Hornbach</t>
         </is>
       </c>
-      <c r="D36" s="47" t="inlineStr">
+      <c r="D37" s="47" t="inlineStr">
         <is>
           <t>est.</t>
         </is>
       </c>
-      <c r="E36" s="47" t="n">
+      <c r="E37" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="F36" s="47" t="inlineStr">
+      <c r="F37" s="47" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="H36" s="47" t="inlineStr">
+      <c r="H37" s="47" t="inlineStr">
         <is>
           <t>2x balama arc + zavor copil sus; de confirmat</t>
         </is>
       </c>
-      <c r="I36" s="47" t="inlineStr">
+      <c r="I37" s="47" t="inlineStr">
         <is>
           <t>De cumparat (est.)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="F38" s="89" t="inlineStr">
+    <row r="39">
+      <c r="F39" s="89" t="inlineStr">
         <is>
           <t>TOTAL platforma:</t>
         </is>
       </c>
-      <c r="G38" s="90">
-        <f>SUM(G5:G36)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="F39" s="76" t="inlineStr">
+      <c r="G39" s="90">
+        <f>SUM(G5:G37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="F40" s="76" t="inlineStr">
         <is>
           <t>din care DE CUMPARAT:</t>
         </is>
       </c>
-      <c r="G39" s="91">
-        <f>SUMIF(I5:I36,"De cumparat*",G5:G36)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="80" t="inlineStr">
+      <c r="G40" s="91">
+        <f>SUMIF(I5:I37,"De cumparat*",G5:G37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="80" t="inlineStr">
         <is>
           <t>Scara: 10 trepte (11 niveluri), riser 200 / calcai 190, ~49°, latime 600, mana curenta pe ambele parti, poarta la S3 (opus mesei de pe S4). Preturi 'est.' = de confirmat la magazin.</t>
         </is>
@@ -4782,14 +4866,14 @@
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A29:I29"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A28:I28"/>
-    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A32:I32"/>
+    <mergeCell ref="A14:I14"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A31:I31"/>
-    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A16:I16"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
audit-fixes v2: cote as-built + talpic + bannere audituri + tracker (surse text)
</commit_message>
<xml_diff>
--- a/Tracker_materiale_casuta.xlsx
+++ b/Tracker_materiale_casuta.xlsx
@@ -1854,7 +1854,7 @@
       <c r="K27" s="66" t="n"/>
       <c r="L27" s="66" t="inlineStr">
         <is>
-          <t>C1 grinda fata-&gt;stalp (4); C2 anti-ridicare (12 joiste + 2 grinda spate = 14) · comanda 09.06.2026</t>
+          <t>C1 grinda fata-&gt;stalp (4); C2 anti-ridicare: necesar as-built 18 (16 reazeme joiste+surori + 2 grinda spate). Ai 14 -&gt; de cumparat 4 (sau 6 daca la numaratoare ies 12). · comanda 09.06.2026</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2460,7 @@
       </c>
       <c r="D7" s="97" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>~1900</t>
         </is>
       </c>
       <c r="E7" s="97" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="H7" s="95" t="inlineStr">
         <is>
-          <t>Taiati la +1872 (sub podea: grinda 200 + joista 100 + dusumea 28 = 2200). Offcut ~2128 pt polite, talpice, contrafise/blocuri.</t>
+          <t>Taiati la ~1900 as-built (plan initial 1872). Buildup podea: glulam 200 -&gt; 2100, joiste 100 -&gt; 2200, dusumea 28 -&gt; 2228. Offcut ~2100 pt polite, talpice, contrafise/blocuri.</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="D9" s="97" t="inlineStr">
         <is>
-          <t>~2550</t>
+          <t>dupa masuratoare as-built (~2430-2450)</t>
         </is>
       </c>
       <c r="E9" s="97" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="H9" s="95" t="inlineStr">
         <is>
-          <t>Fata-spate (consola 700), CONTINUE. Pozitii de la S4: 100/280/720/1120/1550/1980 — ocolesc trunchiul.</t>
+          <t>Fata-spate (consola 700), CONTINUE. Pozitii as-built: 0/280/720/1120/1550/2100 (capete dublate pe axa stalpilor spate). Taie DOAR dupa masuratoare as-built (tinta ~2430-2450, NU 2550).</t>
         </is>
       </c>
     </row>
@@ -2655,16 +2655,44 @@
     <row r="12" ht="21.75" customHeight="1" s="48">
       <c r="A12" s="72" t="inlineStr">
         <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="B12" s="83" t="n"/>
-      <c r="C12" s="83" t="n"/>
-      <c r="D12" s="83" t="n"/>
-      <c r="E12" s="83" t="n"/>
-      <c r="F12" s="83" t="n"/>
-      <c r="G12" s="83" t="n"/>
-      <c r="H12" s="84" t="n"/>
+          <t>P4d</t>
+        </is>
+      </c>
+      <c r="B12" s="95" t="inlineStr">
+        <is>
+          <t>Joiste-sora (dublare capete)</t>
+        </is>
+      </c>
+      <c r="C12" s="95" t="inlineStr">
+        <is>
+          <t>KVH 100×100</t>
+        </is>
+      </c>
+      <c r="D12" s="97" t="inlineStr">
+        <is>
+          <t>dupa masuratoare as-built</t>
+        </is>
+      </c>
+      <c r="E12" s="97" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F12" s="74" t="inlineStr">
+        <is>
+          <t>DE CUMPARAT</t>
+        </is>
+      </c>
+      <c r="G12" s="94" t="inlineStr">
+        <is>
+          <t>Hornbach</t>
+        </is>
+      </c>
+      <c r="H12" s="95" t="inlineStr">
+        <is>
+          <t>2× joista suplimentara pe axele stalpilor (0 si 2100), lipite de joistele de capat = capete dublate (sister). Cod Hornbach 7337253; lungime dupa masuratoare as-built.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1" s="48">
       <c r="A13" s="82" t="inlineStr">
@@ -3522,8 +3550,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A12:H12"/>
+  <mergeCells count="11">
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="A30:H30"/>
@@ -3760,7 +3787,7 @@
       </c>
       <c r="I8" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3871,7 @@
       </c>
       <c r="I10" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
     </row>
@@ -3886,7 +3913,7 @@
       </c>
       <c r="I11" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4054,7 @@
       </c>
       <c r="I15" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4111,7 @@
       </c>
       <c r="I17" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4153,7 @@
       </c>
       <c r="I18" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4195,7 @@
       </c>
       <c r="I19" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4237,7 @@
       </c>
       <c r="I20" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4279,7 @@
       </c>
       <c r="I21" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
     </row>
@@ -4294,7 +4321,7 @@
       </c>
       <c r="I22" s="72" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
     </row>
@@ -4576,7 +4603,7 @@
       </c>
       <c r="I30" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>SOSIT 18.06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
continut v3: streasina 100/caprior 1342/fara jgheab, pereti canonic=GHID, scara amanata, tracker 8/16+skip sisters, SoT lant intreg
</commit_message>
<xml_diff>
--- a/Tracker_materiale_casuta.xlsx
+++ b/Tracker_materiale_casuta.xlsx
@@ -1401,7 +1401,7 @@
       </c>
       <c r="E18" s="65" t="n"/>
       <c r="F18" s="67" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G18" s="65" t="inlineStr">
         <is>
@@ -1503,7 +1503,7 @@
         </is>
       </c>
       <c r="F20" s="47" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G20" s="47" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
       <c r="K21" s="66" t="n"/>
       <c r="L21" s="66" t="inlineStr">
         <is>
-          <t>Pereti pana la jumatate + ferestre</t>
+          <t>Pereti Faza 2: vezi GHID-SIMPLU-casa §7 (lambriu direct pe rama, fara OSB, contrafise in colturi)</t>
         </is>
       </c>
     </row>
@@ -1695,7 +1695,7 @@
       </c>
       <c r="J24" s="74" t="inlineStr">
         <is>
-          <t>De cumparat</t>
+          <t>AMANAT 11.08 — scara</t>
         </is>
       </c>
       <c r="K24" s="95" t="n"/>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="F12" s="74" t="inlineStr">
         <is>
-          <t>DE CUMPARAT</t>
+          <t>SKIP DEFINITIV 06.08 — NU se cumpara</t>
         </is>
       </c>
       <c r="G12" s="94" t="inlineStr">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="E24" s="97" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F24" s="74" t="inlineStr">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="F28" s="74" t="inlineStr">
         <is>
-          <t>NOU</t>
+          <t>AMANAT 11.08</t>
         </is>
       </c>
       <c r="G28" s="94" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="F29" s="74" t="inlineStr">
         <is>
-          <t>NOU</t>
+          <t>AMANAT 11.08</t>
         </is>
       </c>
       <c r="G29" s="94" t="inlineStr">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="I24" s="72" t="inlineStr">
         <is>
-          <t>De cumparat (est.)</t>
+          <t>AMANAT 11.08</t>
         </is>
       </c>
     </row>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="I25" s="72" t="inlineStr">
         <is>
-          <t>De cumparat (est.)</t>
+          <t>AMANAT 11.08</t>
         </is>
       </c>
     </row>
@@ -4462,7 +4462,7 @@
       </c>
       <c r="I26" s="72" t="inlineStr">
         <is>
-          <t>De cumparat (est.)</t>
+          <t>AMANAT 11.08</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="I27" s="72" t="inlineStr">
         <is>
-          <t>De cumparat (est.)</t>
+          <t>AMANAT 11.08</t>
         </is>
       </c>
     </row>
@@ -4546,7 +4546,7 @@
       </c>
       <c r="I28" s="72" t="inlineStr">
         <is>
-          <t>De cumparat (est.)</t>
+          <t>AMANAT 11.08</t>
         </is>
       </c>
     </row>
@@ -4676,7 +4676,7 @@
         <v>60.91</v>
       </c>
       <c r="E33" s="47" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F33" s="47" t="inlineStr">
         <is>
@@ -4800,7 +4800,7 @@
         <v>3.5</v>
       </c>
       <c r="E36" s="47" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F36" s="47" t="inlineStr">
         <is>
@@ -5537,7 +5537,7 @@
       </c>
       <c r="F23" s="96" t="inlineStr">
         <is>
-          <t>de confirmat</t>
+          <t>AMANAT 11.08</t>
         </is>
       </c>
       <c r="G23" s="94" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="F24" s="96" t="inlineStr">
         <is>
-          <t>de confirmat</t>
+          <t>AMANAT 11.08</t>
         </is>
       </c>
       <c r="G24" s="94" t="inlineStr">
@@ -5601,7 +5601,7 @@
       </c>
       <c r="F25" s="96" t="inlineStr">
         <is>
-          <t>de confirmat</t>
+          <t>AMANAT 11.08</t>
         </is>
       </c>
       <c r="G25" s="94" t="inlineStr">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="F26" s="96" t="inlineStr">
         <is>
-          <t>de confirmat</t>
+          <t>AMANAT 11.08</t>
         </is>
       </c>
       <c r="G26" s="94" t="inlineStr">
@@ -5657,7 +5657,7 @@
         <v>3.5</v>
       </c>
       <c r="D27" s="92" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E27" s="93">
         <f>C27*D27</f>

</xml_diff>